<commit_message>
+ Add map scene UI.
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="UI" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="835">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="897" uniqueCount="855">
   <si>
     <t>ID</t>
   </si>
@@ -3504,6 +3504,66 @@
   </si>
   <si>
     <t>Na Tra</t>
+  </si>
+  <si>
+    <t>UI_LOCATION</t>
+  </si>
+  <si>
+    <t>Nơi này là đâu?</t>
+  </si>
+  <si>
+    <t>Where am I?</t>
+  </si>
+  <si>
+    <t>UI_MAP</t>
+  </si>
+  <si>
+    <t>Map</t>
+  </si>
+  <si>
+    <t>Bản đồ</t>
+  </si>
+  <si>
+    <t>UI_WATER_CURTAIN_CAVE</t>
+  </si>
+  <si>
+    <t>Water Curtain Cave</t>
+  </si>
+  <si>
+    <t>Thủy Liêm Động</t>
+  </si>
+  <si>
+    <t>East Sea Dragon Palace</t>
+  </si>
+  <si>
+    <t>UI_EAST_SEA</t>
+  </si>
+  <si>
+    <t>Flaming Mountains</t>
+  </si>
+  <si>
+    <t>UI_FLAMING_MOUNTAINS</t>
+  </si>
+  <si>
+    <t>Hỏa Diệm Sơn</t>
+  </si>
+  <si>
+    <t>Thiên Cung</t>
+  </si>
+  <si>
+    <t>Heavenly Palace</t>
+  </si>
+  <si>
+    <t>UI_HEAVENLY_PLACE</t>
+  </si>
+  <si>
+    <t>UI_GO</t>
+  </si>
+  <si>
+    <t>Go</t>
+  </si>
+  <si>
+    <t>Đến</t>
   </si>
 </sst>
 </file>
@@ -3848,10 +3908,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C68"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.85546875" customWidth="1"/>
     <col min="2" max="2" width="25.5703125" customWidth="1"/>
     <col min="3" max="3" width="30.5703125" customWidth="1"/>
   </cols>
@@ -4590,6 +4650,83 @@
       </c>
       <c r="C68" t="s">
         <v>723</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>835</v>
+      </c>
+      <c r="B69" t="s">
+        <v>837</v>
+      </c>
+      <c r="C69" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>838</v>
+      </c>
+      <c r="B70" t="s">
+        <v>839</v>
+      </c>
+      <c r="C70" t="s">
+        <v>840</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>841</v>
+      </c>
+      <c r="B71" t="s">
+        <v>842</v>
+      </c>
+      <c r="C71" t="s">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>845</v>
+      </c>
+      <c r="B72" t="s">
+        <v>844</v>
+      </c>
+      <c r="C72" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>847</v>
+      </c>
+      <c r="B73" t="s">
+        <v>846</v>
+      </c>
+      <c r="C73" t="s">
+        <v>848</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>851</v>
+      </c>
+      <c r="B74" t="s">
+        <v>850</v>
+      </c>
+      <c r="C74" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>852</v>
+      </c>
+      <c r="B75" t="s">
+        <v>853</v>
+      </c>
+      <c r="C75" t="s">
+        <v>854</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Make UI Scene Map and fix build Android.
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="UI" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="897" uniqueCount="855">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="900" uniqueCount="858">
   <si>
     <t>ID</t>
   </si>
@@ -3564,6 +3564,15 @@
   </si>
   <si>
     <t>Đến</t>
+  </si>
+  <si>
+    <t>STR_LOADING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loading… </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đang tải.. </t>
   </si>
 </sst>
 </file>
@@ -5161,7 +5170,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C176"/>
+  <dimension ref="A1:C177"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.7109375" bestFit="1" customWidth="1"/>
@@ -7082,6 +7091,17 @@
       </c>
       <c r="C176" t="s">
         <v>834</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>855</v>
+      </c>
+      <c r="B177" t="s">
+        <v>856</v>
+      </c>
+      <c r="C177" t="s">
+        <v>857</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- Clean code architecture for building a data tool and add all functions in the armor card of the character.
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
     <sheet name="UI" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1105" uniqueCount="977">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1114" uniqueCount="986">
   <si>
     <t>ID</t>
   </si>
@@ -2774,21 +2774,12 @@
     <t>UI_UPGRADE_MAX_LEVEL</t>
   </si>
   <si>
-    <t>Upgrade to Lv.10</t>
-  </si>
-  <si>
-    <t>Tăng tới cấp 10</t>
-  </si>
-  <si>
     <t>UI_DEF_SHRED</t>
   </si>
   <si>
     <t>DEF Shred</t>
   </si>
   <si>
-    <t>Khả năng giảm giáp</t>
-  </si>
-  <si>
     <t>UI_SKILLS</t>
   </si>
   <si>
@@ -3930,6 +3921,42 @@
   </si>
   <si>
     <t>Trừ máu mỗi hiệu {0}%</t>
+  </si>
+  <si>
+    <t>Upgrade to</t>
+  </si>
+  <si>
+    <t>Tăng tới cấp</t>
+  </si>
+  <si>
+    <t>Giảm giáp</t>
+  </si>
+  <si>
+    <t>UI_SET_BONUS</t>
+  </si>
+  <si>
+    <t>Set bonus({0} Part)</t>
+  </si>
+  <si>
+    <t>Phần thưởng bộ ({0} Mảnh)</t>
+  </si>
+  <si>
+    <t>UI_SET_BONUS_CONTENT</t>
+  </si>
+  <si>
+    <t>Increasece {0} by {1}.</t>
+  </si>
+  <si>
+    <t>Tăng {0} lên {1}.</t>
+  </si>
+  <si>
+    <t>STR_SET_BONUS</t>
+  </si>
+  <si>
+    <t>Set Bonus</t>
+  </si>
+  <si>
+    <t>Thưởng Bộ</t>
   </si>
 </sst>
 </file>
@@ -4281,7 +4308,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.85546875" customWidth="1"/>
@@ -4500,13 +4527,13 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>862</v>
+        <v>859</v>
       </c>
       <c r="B20" t="s">
-        <v>863</v>
+        <v>860</v>
       </c>
       <c r="C20" t="s">
-        <v>864</v>
+        <v>861</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -4682,7 +4709,7 @@
         <v>516</v>
       </c>
       <c r="C36" t="s">
-        <v>604</v>
+        <v>601</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -4910,62 +4937,62 @@
         <v>590</v>
       </c>
       <c r="B57" t="s">
-        <v>591</v>
+        <v>974</v>
       </c>
       <c r="C57" t="s">
-        <v>592</v>
+        <v>975</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B58" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="C58" t="s">
-        <v>595</v>
+        <v>976</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
       <c r="B59" t="s">
         <v>196</v>
       </c>
       <c r="C59" t="s">
-        <v>597</v>
+        <v>594</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>598</v>
+        <v>595</v>
       </c>
       <c r="B60" t="s">
-        <v>599</v>
+        <v>596</v>
       </c>
       <c r="C60" t="s">
-        <v>600</v>
+        <v>597</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>603</v>
+        <v>600</v>
       </c>
       <c r="B61" t="s">
-        <v>602</v>
+        <v>599</v>
       </c>
       <c r="C61" t="s">
-        <v>601</v>
+        <v>598</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>605</v>
+        <v>602</v>
       </c>
       <c r="B62" t="s">
-        <v>606</v>
+        <v>603</v>
       </c>
       <c r="C62" t="s">
         <v>589</v>
@@ -4973,144 +5000,177 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>607</v>
+        <v>604</v>
       </c>
       <c r="B63" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="C63" t="s">
-        <v>609</v>
+        <v>606</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="B64" t="s">
-        <v>641</v>
+        <v>638</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>639</v>
+      </c>
+      <c r="B65" t="s">
         <v>642</v>
-      </c>
-      <c r="B65" t="s">
-        <v>645</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>643</v>
+        <v>640</v>
       </c>
       <c r="B66" t="s">
-        <v>644</v>
+        <v>641</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
       <c r="B67" t="s">
-        <v>647</v>
+        <v>644</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="B68" t="s">
-        <v>719</v>
+        <v>716</v>
       </c>
       <c r="C68" t="s">
-        <v>720</v>
+        <v>717</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>844</v>
+        <v>841</v>
       </c>
       <c r="B69" t="s">
-        <v>845</v>
+        <v>842</v>
       </c>
       <c r="C69" t="s">
-        <v>846</v>
+        <v>843</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>824</v>
+        <v>821</v>
       </c>
       <c r="B70" t="s">
-        <v>825</v>
+        <v>822</v>
       </c>
       <c r="C70" t="s">
-        <v>826</v>
+        <v>823</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="B71" t="s">
-        <v>828</v>
+        <v>825</v>
       </c>
       <c r="C71" t="s">
-        <v>829</v>
+        <v>826</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>831</v>
+        <v>828</v>
       </c>
       <c r="B72" t="s">
-        <v>830</v>
+        <v>827</v>
       </c>
       <c r="C72" t="s">
-        <v>760</v>
+        <v>757</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="B73" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
       <c r="C73" t="s">
-        <v>834</v>
+        <v>831</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>837</v>
+        <v>834</v>
       </c>
       <c r="B74" t="s">
-        <v>836</v>
+        <v>833</v>
       </c>
       <c r="C74" t="s">
-        <v>835</v>
+        <v>832</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
       <c r="B75" t="s">
-        <v>839</v>
+        <v>836</v>
       </c>
       <c r="C75" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>865</v>
+        <v>862</v>
       </c>
       <c r="B76" t="s">
-        <v>866</v>
+        <v>863</v>
       </c>
       <c r="C76" t="s">
-        <v>867</v>
+        <v>864</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>983</v>
+      </c>
+      <c r="B77" t="s">
+        <v>978</v>
+      </c>
+      <c r="C77" t="s">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>980</v>
+      </c>
+      <c r="B78" t="s">
+        <v>981</v>
+      </c>
+      <c r="C78" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>977</v>
+      </c>
+      <c r="B79" t="s">
+        <v>984</v>
+      </c>
+      <c r="C79" t="s">
+        <v>985</v>
       </c>
     </row>
   </sheetData>
@@ -5141,381 +5201,381 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
       <c r="B2" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
       <c r="C2" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>663</v>
+        <v>660</v>
       </c>
       <c r="B3" t="s">
+        <v>661</v>
+      </c>
+      <c r="C3" t="s">
         <v>664</v>
-      </c>
-      <c r="C3" t="s">
-        <v>667</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>662</v>
+      </c>
+      <c r="B4" t="s">
+        <v>663</v>
+      </c>
+      <c r="C4" t="s">
         <v>665</v>
-      </c>
-      <c r="B4" t="s">
-        <v>666</v>
-      </c>
-      <c r="C4" t="s">
-        <v>668</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>670</v>
+        <v>667</v>
       </c>
       <c r="B5" t="s">
-        <v>669</v>
+        <v>666</v>
       </c>
       <c r="C5" t="s">
-        <v>671</v>
+        <v>668</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>676</v>
+        <v>673</v>
       </c>
       <c r="B6" t="s">
-        <v>675</v>
+        <v>672</v>
       </c>
       <c r="C6" t="s">
-        <v>674</v>
+        <v>671</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>677</v>
+        <v>674</v>
       </c>
       <c r="B7" t="s">
-        <v>678</v>
+        <v>675</v>
       </c>
       <c r="C7" t="s">
-        <v>679</v>
+        <v>676</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>680</v>
+        <v>677</v>
       </c>
       <c r="B8" t="s">
-        <v>681</v>
+        <v>678</v>
       </c>
       <c r="C8" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="B9" t="s">
-        <v>684</v>
+        <v>681</v>
       </c>
       <c r="C9" t="s">
-        <v>688</v>
+        <v>685</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>685</v>
+        <v>682</v>
       </c>
       <c r="B10" t="s">
-        <v>686</v>
+        <v>683</v>
       </c>
       <c r="C10" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>689</v>
+        <v>686</v>
       </c>
       <c r="B11" t="s">
-        <v>690</v>
+        <v>687</v>
       </c>
       <c r="C11" t="s">
-        <v>691</v>
+        <v>688</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>692</v>
+        <v>689</v>
       </c>
       <c r="C12" t="s">
-        <v>693</v>
+        <v>690</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
       <c r="C13" t="s">
-        <v>695</v>
+        <v>692</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>696</v>
+        <v>693</v>
       </c>
       <c r="C14" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>698</v>
+        <v>695</v>
       </c>
       <c r="C15" t="s">
-        <v>699</v>
+        <v>696</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
       <c r="C16" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>702</v>
+        <v>699</v>
       </c>
       <c r="C17" t="s">
-        <v>703</v>
+        <v>700</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>704</v>
+        <v>701</v>
       </c>
       <c r="C18" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>705</v>
+        <v>702</v>
       </c>
       <c r="C19" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="C20" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
       <c r="C21" t="s">
-        <v>710</v>
+        <v>707</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="C22" t="s">
-        <v>712</v>
+        <v>709</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>713</v>
+        <v>710</v>
       </c>
       <c r="C23" t="s">
-        <v>721</v>
+        <v>718</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="C24" t="s">
-        <v>715</v>
+        <v>712</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="C25" t="s">
-        <v>717</v>
+        <v>714</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
       <c r="C26" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="C27" t="s">
-        <v>730</v>
+        <v>727</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="C28" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="C29" t="s">
-        <v>731</v>
+        <v>728</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>722</v>
+        <v>719</v>
       </c>
       <c r="C30" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
       <c r="C31" t="s">
-        <v>749</v>
+        <v>746</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>732</v>
+        <v>729</v>
       </c>
       <c r="C32" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="C33" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
       <c r="C34" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
       <c r="C35" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>738</v>
+        <v>735</v>
       </c>
       <c r="C36" t="s">
-        <v>739</v>
+        <v>736</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>740</v>
+        <v>737</v>
       </c>
       <c r="C37" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
       <c r="C38" t="s">
-        <v>750</v>
+        <v>747</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
       <c r="C39" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
       <c r="C40" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="C41" t="s">
-        <v>751</v>
+        <v>748</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
       <c r="C42" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="C43" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
       <c r="C44" t="s">
-        <v>760</v>
+        <v>757</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>761</v>
+        <v>758</v>
       </c>
       <c r="C45" t="s">
         <v>166</v>
@@ -5523,18 +5583,18 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>762</v>
+        <v>759</v>
       </c>
       <c r="C46" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>764</v>
+        <v>761</v>
       </c>
       <c r="C47" t="s">
-        <v>765</v>
+        <v>762</v>
       </c>
     </row>
   </sheetData>
@@ -6991,7 +7051,7 @@
         <v>472</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>673</v>
+        <v>670</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
@@ -7013,7 +7073,7 @@
         <v>473</v>
       </c>
       <c r="C133" t="s">
-        <v>672</v>
+        <v>669</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
@@ -7194,10 +7254,10 @@
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>610</v>
+        <v>607</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>611</v>
+        <v>608</v>
       </c>
       <c r="C150" s="3" t="s">
         <v>581</v>
@@ -7205,7 +7265,7 @@
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>612</v>
+        <v>609</v>
       </c>
       <c r="B151" s="3" t="s">
         <v>583</v>
@@ -7216,18 +7276,18 @@
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="B152" t="s">
         <v>1</v>
       </c>
       <c r="C152" s="3" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="B153" t="s">
         <v>2</v>
@@ -7238,136 +7298,136 @@
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
+        <v>613</v>
+      </c>
+      <c r="B154" t="s">
         <v>616</v>
       </c>
-      <c r="B154" t="s">
-        <v>619</v>
-      </c>
       <c r="C154" s="3" t="s">
-        <v>652</v>
+        <v>649</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>626</v>
+        <v>623</v>
       </c>
       <c r="B155" t="s">
-        <v>627</v>
+        <v>624</v>
       </c>
       <c r="C155" s="3" t="s">
-        <v>648</v>
+        <v>645</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
+        <v>614</v>
+      </c>
+      <c r="B156" t="s">
         <v>617</v>
       </c>
-      <c r="B156" t="s">
-        <v>620</v>
-      </c>
       <c r="C156" s="3" t="s">
-        <v>654</v>
+        <v>651</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
+        <v>615</v>
+      </c>
+      <c r="B157" t="s">
         <v>618</v>
       </c>
-      <c r="B157" t="s">
-        <v>621</v>
-      </c>
       <c r="C157" s="3" t="s">
-        <v>655</v>
+        <v>652</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>622</v>
+        <v>619</v>
       </c>
       <c r="B158" t="s">
-        <v>628</v>
+        <v>625</v>
       </c>
       <c r="C158" s="3" t="s">
-        <v>650</v>
+        <v>647</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>625</v>
+        <v>622</v>
       </c>
       <c r="B159" t="s">
-        <v>629</v>
+        <v>626</v>
       </c>
       <c r="C159" t="s">
-        <v>649</v>
+        <v>646</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>623</v>
+        <v>620</v>
       </c>
       <c r="B160" t="s">
-        <v>630</v>
+        <v>627</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="B161" t="s">
-        <v>631</v>
+        <v>628</v>
       </c>
       <c r="C161" s="3" t="s">
-        <v>656</v>
+        <v>653</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="B162" t="s">
-        <v>637</v>
+        <v>634</v>
       </c>
       <c r="C162" t="s">
-        <v>653</v>
+        <v>650</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="B163" t="s">
-        <v>639</v>
+        <v>636</v>
       </c>
       <c r="C163" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>634</v>
+        <v>631</v>
       </c>
       <c r="B164" t="s">
-        <v>638</v>
+        <v>635</v>
       </c>
       <c r="C164" t="s">
-        <v>658</v>
+        <v>655</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>635</v>
+        <v>632</v>
       </c>
       <c r="B165" t="s">
-        <v>636</v>
+        <v>633</v>
       </c>
       <c r="C165" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="B166" t="s">
         <v>22</v>
@@ -7378,77 +7438,77 @@
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="C167" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="C168" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>808</v>
+        <v>805</v>
       </c>
       <c r="C169" t="s">
-        <v>809</v>
+        <v>806</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>810</v>
+        <v>807</v>
       </c>
       <c r="C170" t="s">
-        <v>811</v>
+        <v>808</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>812</v>
+        <v>809</v>
       </c>
       <c r="C171" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>814</v>
+        <v>811</v>
       </c>
       <c r="C172" t="s">
-        <v>815</v>
+        <v>812</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>816</v>
+        <v>813</v>
       </c>
       <c r="B173" t="s">
-        <v>822</v>
+        <v>819</v>
       </c>
       <c r="C173" t="s">
-        <v>821</v>
+        <v>818</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
+        <v>814</v>
+      </c>
+      <c r="B174" t="s">
         <v>817</v>
       </c>
-      <c r="B174" t="s">
-        <v>820</v>
-      </c>
       <c r="C174" t="s">
-        <v>819</v>
+        <v>816</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>818</v>
+        <v>815</v>
       </c>
       <c r="B175" t="s">
         <v>80</v>
@@ -7459,90 +7519,90 @@
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>823</v>
+        <v>820</v>
       </c>
       <c r="B176" t="s">
-        <v>847</v>
+        <v>844</v>
       </c>
       <c r="C176" t="s">
-        <v>848</v>
+        <v>845</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>841</v>
+        <v>838</v>
       </c>
       <c r="B177" t="s">
-        <v>842</v>
+        <v>839</v>
       </c>
       <c r="C177" t="s">
-        <v>843</v>
+        <v>840</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>849</v>
+        <v>846</v>
       </c>
       <c r="B178" t="s">
-        <v>850</v>
+        <v>847</v>
       </c>
       <c r="C178" t="s">
-        <v>851</v>
+        <v>848</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>857</v>
+        <v>854</v>
       </c>
       <c r="B179" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="C179" t="s">
-        <v>852</v>
+        <v>849</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>858</v>
+        <v>855</v>
       </c>
       <c r="B180" t="s">
-        <v>855</v>
+        <v>852</v>
       </c>
       <c r="C180" t="s">
-        <v>964</v>
+        <v>961</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>859</v>
+        <v>856</v>
       </c>
       <c r="B181" t="s">
-        <v>856</v>
+        <v>853</v>
       </c>
       <c r="C181" t="s">
-        <v>853</v>
+        <v>850</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>860</v>
+        <v>857</v>
       </c>
       <c r="B182" t="s">
-        <v>861</v>
+        <v>858</v>
       </c>
       <c r="C182" t="s">
-        <v>868</v>
+        <v>865</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>869</v>
+        <v>866</v>
       </c>
       <c r="B183" t="s">
-        <v>871</v>
+        <v>868</v>
       </c>
       <c r="C183" t="s">
-        <v>870</v>
+        <v>867</v>
       </c>
     </row>
   </sheetData>
@@ -7574,738 +7634,738 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>872</v>
+        <v>869</v>
       </c>
       <c r="C2" t="s">
-        <v>768</v>
+        <v>765</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>875</v>
+        <v>872</v>
       </c>
       <c r="C3" t="s">
-        <v>771</v>
+        <v>768</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>873</v>
+        <v>870</v>
       </c>
       <c r="C4" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>876</v>
+        <v>873</v>
       </c>
       <c r="C5" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>874</v>
+        <v>871</v>
       </c>
       <c r="C6" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>877</v>
+        <v>874</v>
       </c>
       <c r="C7" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>879</v>
+        <v>876</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>880</v>
+        <v>877</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
+        <v>878</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>881</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>884</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>882</v>
+        <v>879</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>883</v>
+        <v>880</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>885</v>
+        <v>882</v>
       </c>
       <c r="C14" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>886</v>
+        <v>883</v>
       </c>
       <c r="C15" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>887</v>
+        <v>884</v>
       </c>
       <c r="C16" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>888</v>
+        <v>885</v>
       </c>
       <c r="C17" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>889</v>
+        <v>886</v>
       </c>
       <c r="C18" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>890</v>
+        <v>887</v>
       </c>
       <c r="C19" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>891</v>
+        <v>888</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>892</v>
+        <v>889</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>893</v>
+        <v>890</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>890</v>
+        <v>887</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>894</v>
+        <v>891</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>895</v>
+        <v>892</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>896</v>
+        <v>893</v>
       </c>
       <c r="C26" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>897</v>
+        <v>894</v>
       </c>
       <c r="C27" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>898</v>
+        <v>895</v>
       </c>
       <c r="C28" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>899</v>
+        <v>896</v>
       </c>
       <c r="C29" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>900</v>
+        <v>897</v>
       </c>
       <c r="C30" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>901</v>
+        <v>898</v>
       </c>
       <c r="C31" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>902</v>
+        <v>899</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>903</v>
+        <v>900</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>904</v>
+        <v>901</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>905</v>
+        <v>902</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>906</v>
+        <v>903</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>907</v>
+        <v>904</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>908</v>
+        <v>905</v>
       </c>
       <c r="C38" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>909</v>
+        <v>906</v>
       </c>
       <c r="C39" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>910</v>
+        <v>907</v>
       </c>
       <c r="C40" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>911</v>
+        <v>908</v>
       </c>
       <c r="C41" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>912</v>
+        <v>909</v>
       </c>
       <c r="C42" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>913</v>
+        <v>910</v>
       </c>
       <c r="C43" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>914</v>
+        <v>911</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>915</v>
+        <v>912</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>916</v>
+        <v>913</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>917</v>
+        <v>914</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>918</v>
+        <v>915</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>919</v>
+        <v>916</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>920</v>
+        <v>917</v>
       </c>
       <c r="C50" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>921</v>
+        <v>918</v>
       </c>
       <c r="C51" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>922</v>
+        <v>919</v>
       </c>
       <c r="C52" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>923</v>
+        <v>920</v>
       </c>
       <c r="C53" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>924</v>
+        <v>921</v>
       </c>
       <c r="C54" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>925</v>
+        <v>922</v>
       </c>
       <c r="C55" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>926</v>
+        <v>923</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>927</v>
+        <v>924</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>928</v>
+        <v>925</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>931</v>
+        <v>928</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>932</v>
+        <v>929</v>
       </c>
       <c r="C62" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>933</v>
+        <v>930</v>
       </c>
       <c r="C63" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>934</v>
+        <v>931</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>935</v>
+        <v>932</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>936</v>
+        <v>933</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>937</v>
+        <v>934</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>938</v>
+        <v>935</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>939</v>
+        <v>936</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>940</v>
+        <v>937</v>
       </c>
       <c r="C70" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>941</v>
+        <v>938</v>
       </c>
       <c r="C71" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>942</v>
+        <v>939</v>
       </c>
       <c r="C72" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>943</v>
+        <v>940</v>
       </c>
       <c r="C73" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>944</v>
+        <v>941</v>
       </c>
       <c r="C74" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>945</v>
+        <v>942</v>
       </c>
       <c r="C75" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
-        <v>946</v>
+        <v>943</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
-        <v>947</v>
+        <v>944</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
-        <v>948</v>
+        <v>945</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
-        <v>949</v>
+        <v>946</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
-        <v>950</v>
+        <v>947</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
-        <v>951</v>
+        <v>948</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>952</v>
+        <v>949</v>
       </c>
       <c r="C82" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>953</v>
+        <v>950</v>
       </c>
       <c r="C83" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>954</v>
+        <v>951</v>
       </c>
       <c r="C84" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>955</v>
+        <v>952</v>
       </c>
       <c r="C85" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>956</v>
+        <v>953</v>
       </c>
       <c r="C86" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>957</v>
+        <v>954</v>
       </c>
       <c r="C87" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
-        <v>958</v>
+        <v>955</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
-        <v>959</v>
+        <v>956</v>
       </c>
       <c r="C89" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="s">
-        <v>960</v>
+        <v>957</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
-        <v>961</v>
+        <v>958</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="5" t="s">
-        <v>962</v>
+        <v>959</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="5" t="s">
-        <v>963</v>
+        <v>960</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
     </row>
   </sheetData>
@@ -8335,178 +8395,178 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>772</v>
+        <v>769</v>
       </c>
       <c r="C2" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="C3" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>776</v>
+        <v>773</v>
       </c>
       <c r="C4" t="s">
-        <v>775</v>
+        <v>772</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>777</v>
+        <v>774</v>
       </c>
       <c r="C5" t="s">
-        <v>778</v>
+        <v>775</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
       <c r="C6" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="C7" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>966</v>
+        <v>963</v>
       </c>
       <c r="C8" t="s">
-        <v>968</v>
+        <v>965</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>965</v>
+        <v>962</v>
       </c>
       <c r="C9" t="s">
-        <v>969</v>
+        <v>966</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
       <c r="C10" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>784</v>
+        <v>781</v>
       </c>
       <c r="C11" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>787</v>
+        <v>784</v>
       </c>
       <c r="C12" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
       <c r="C13" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
       <c r="C14" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
       <c r="C15" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
       <c r="C16" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
       <c r="C17" t="s">
-        <v>803</v>
+        <v>800</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>799</v>
+        <v>796</v>
       </c>
       <c r="C18" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="C19" t="s">
-        <v>801</v>
+        <v>798</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>971</v>
+        <v>968</v>
       </c>
       <c r="C20" t="s">
-        <v>967</v>
+        <v>964</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>972</v>
+        <v>969</v>
       </c>
       <c r="C21" t="s">
-        <v>970</v>
+        <v>967</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>973</v>
+        <v>970</v>
       </c>
       <c r="C22" t="s">
-        <v>975</v>
+        <v>972</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>974</v>
+        <v>971</v>
       </c>
       <c r="C23" t="s">
-        <v>976</v>
+        <v>973</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Add the Upgrade Armor UI Scene.
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="992">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1132" uniqueCount="1003">
   <si>
     <t>ID</t>
   </si>
@@ -3978,6 +3978,39 @@
   </si>
   <si>
     <t>UI_MAX_ASCEND_LEVEL</t>
+  </si>
+  <si>
+    <t>Câp cường hóa</t>
+  </si>
+  <si>
+    <t>Attributes</t>
+  </si>
+  <si>
+    <t>UI_ENHANCENMENT_LEVEL</t>
+  </si>
+  <si>
+    <t>UI_ATTRIBUTES</t>
+  </si>
+  <si>
+    <t>Thuộc tính</t>
+  </si>
+  <si>
+    <t>Enhancement Level</t>
+  </si>
+  <si>
+    <t>UI_SELECT_ENHANCEMENT_MATERIALS</t>
+  </si>
+  <si>
+    <t>Chọn vật liệu cường hóa</t>
+  </si>
+  <si>
+    <t>UI_RECALL</t>
+  </si>
+  <si>
+    <t>Recall</t>
+  </si>
+  <si>
+    <t>Thu hồi</t>
   </si>
 </sst>
 </file>
@@ -4329,10 +4362,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C81"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.85546875" customWidth="1"/>
+    <col min="1" max="1" width="36.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.5703125" customWidth="1"/>
     <col min="3" max="3" width="30.5703125" customWidth="1"/>
   </cols>
@@ -5214,6 +5247,50 @@
       </c>
       <c r="C81" t="s">
         <v>989</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>994</v>
+      </c>
+      <c r="B82" t="s">
+        <v>997</v>
+      </c>
+      <c r="C82" t="s">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>995</v>
+      </c>
+      <c r="B83" t="s">
+        <v>993</v>
+      </c>
+      <c r="C83" t="s">
+        <v>996</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>998</v>
+      </c>
+      <c r="B84" t="s">
+        <v>636</v>
+      </c>
+      <c r="C84" t="s">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B85" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C85" t="s">
+        <v>1002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Make the system upgrade skill of character.
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="3" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UI" sheetId="1" r:id="rId1"/>
@@ -3293,15 +3293,6 @@
     <t>Đòn Tàn Khốc</t>
   </si>
   <si>
-    <t>Gây 60% ST Tấn Công cho toàn bộ kẻ định đồng thời hồi 30% ST gây ra.</t>
-  </si>
-  <si>
-    <t>Gây 180% ST Tấn Công cho kẻ định, kèm thêm Giảm Phòng Thù cho mục tiêu, duy trì 2 hiệp</t>
-  </si>
-  <si>
-    <t>Gây ST bằng 80% Tấn Công cho 1 kẻ địch</t>
-  </si>
-  <si>
     <t>DEBUFF_DEF_NAME</t>
   </si>
   <si>
@@ -4011,6 +4002,15 @@
   </si>
   <si>
     <t>UI_CRIT_DMG_RES</t>
+  </si>
+  <si>
+    <t>Gây ST bằng {0}% Tấn Công cho 1 kẻ địch.</t>
+  </si>
+  <si>
+    <t>Gây {0}% ST Tấn Công cho toàn bộ kẻ định đồng thời hồi {1}% ST gây ra.</t>
+  </si>
+  <si>
+    <t>Gây {0}% ST Tấn Công cho kẻ định, kèm thêm Giảm Phòng Thù cho mục tiêu, duy trì 2 hiệp.</t>
   </si>
 </sst>
 </file>
@@ -4581,13 +4581,13 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>856</v>
+        <v>853</v>
       </c>
       <c r="B20" t="s">
-        <v>857</v>
+        <v>854</v>
       </c>
       <c r="C20" t="s">
-        <v>858</v>
+        <v>855</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -4966,7 +4966,7 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>1002</v>
+        <v>999</v>
       </c>
       <c r="B55" t="s">
         <v>580</v>
@@ -4991,10 +4991,10 @@
         <v>587</v>
       </c>
       <c r="B57" t="s">
-        <v>971</v>
+        <v>968</v>
       </c>
       <c r="C57" t="s">
-        <v>972</v>
+        <v>969</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -5005,7 +5005,7 @@
         <v>589</v>
       </c>
       <c r="C58" t="s">
-        <v>973</v>
+        <v>970</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -5108,43 +5108,43 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>838</v>
+        <v>835</v>
       </c>
       <c r="B69" t="s">
-        <v>839</v>
+        <v>836</v>
       </c>
       <c r="C69" t="s">
-        <v>840</v>
+        <v>837</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>818</v>
+        <v>815</v>
       </c>
       <c r="B70" t="s">
-        <v>819</v>
+        <v>816</v>
       </c>
       <c r="C70" t="s">
-        <v>820</v>
+        <v>817</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>821</v>
+        <v>818</v>
       </c>
       <c r="B71" t="s">
-        <v>822</v>
+        <v>819</v>
       </c>
       <c r="C71" t="s">
-        <v>823</v>
+        <v>820</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>825</v>
+        <v>822</v>
       </c>
       <c r="B72" t="s">
-        <v>824</v>
+        <v>821</v>
       </c>
       <c r="C72" t="s">
         <v>754</v>
@@ -5152,145 +5152,145 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>827</v>
+        <v>824</v>
       </c>
       <c r="B73" t="s">
-        <v>826</v>
+        <v>823</v>
       </c>
       <c r="C73" t="s">
-        <v>828</v>
+        <v>825</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>831</v>
+        <v>828</v>
       </c>
       <c r="B74" t="s">
-        <v>830</v>
+        <v>827</v>
       </c>
       <c r="C74" t="s">
-        <v>829</v>
+        <v>826</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>832</v>
+        <v>829</v>
       </c>
       <c r="B75" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="C75" t="s">
-        <v>834</v>
+        <v>831</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>859</v>
+        <v>856</v>
       </c>
       <c r="B76" t="s">
-        <v>860</v>
+        <v>857</v>
       </c>
       <c r="C76" t="s">
-        <v>861</v>
+        <v>858</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>980</v>
+        <v>977</v>
       </c>
       <c r="B77" t="s">
-        <v>975</v>
+        <v>972</v>
       </c>
       <c r="C77" t="s">
-        <v>976</v>
+        <v>973</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>977</v>
+        <v>974</v>
       </c>
       <c r="B78" t="s">
-        <v>978</v>
+        <v>975</v>
       </c>
       <c r="C78" t="s">
-        <v>979</v>
+        <v>976</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>974</v>
+        <v>971</v>
       </c>
       <c r="B79" t="s">
-        <v>981</v>
+        <v>978</v>
       </c>
       <c r="C79" t="s">
-        <v>982</v>
+        <v>979</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>990</v>
+        <v>987</v>
       </c>
       <c r="B80" t="s">
-        <v>986</v>
+        <v>983</v>
       </c>
       <c r="C80" t="s">
-        <v>987</v>
+        <v>984</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
+        <v>982</v>
+      </c>
+      <c r="B81" t="s">
+        <v>986</v>
+      </c>
+      <c r="C81" t="s">
         <v>985</v>
-      </c>
-      <c r="B81" t="s">
-        <v>989</v>
-      </c>
-      <c r="C81" t="s">
-        <v>988</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>990</v>
+      </c>
+      <c r="B82" t="s">
         <v>993</v>
       </c>
-      <c r="B82" t="s">
-        <v>996</v>
-      </c>
       <c r="C82" t="s">
-        <v>991</v>
+        <v>988</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>994</v>
+        <v>991</v>
       </c>
       <c r="B83" t="s">
+        <v>989</v>
+      </c>
+      <c r="C83" t="s">
         <v>992</v>
-      </c>
-      <c r="C83" t="s">
-        <v>995</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>997</v>
+        <v>994</v>
       </c>
       <c r="B84" t="s">
         <v>635</v>
       </c>
       <c r="C84" t="s">
-        <v>998</v>
+        <v>995</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>999</v>
+        <v>996</v>
       </c>
       <c r="B85" t="s">
-        <v>1000</v>
+        <v>997</v>
       </c>
       <c r="C85" t="s">
-        <v>1001</v>
+        <v>998</v>
       </c>
     </row>
   </sheetData>
@@ -5962,7 +5962,7 @@
         <v>135</v>
       </c>
       <c r="C21" t="s">
-        <v>984</v>
+        <v>981</v>
       </c>
     </row>
     <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -6160,7 +6160,7 @@
         <v>178</v>
       </c>
       <c r="C39" t="s">
-        <v>983</v>
+        <v>980</v>
       </c>
     </row>
     <row r="40" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
@@ -7559,77 +7559,77 @@
     </row>
     <row r="167" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>798</v>
+        <v>795</v>
       </c>
       <c r="C167" t="s">
-        <v>799</v>
+        <v>796</v>
       </c>
     </row>
     <row r="168" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>800</v>
+        <v>797</v>
       </c>
       <c r="C168" t="s">
-        <v>801</v>
+        <v>798</v>
       </c>
     </row>
     <row r="169" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>802</v>
+        <v>799</v>
       </c>
       <c r="C169" t="s">
-        <v>803</v>
+        <v>800</v>
       </c>
     </row>
     <row r="170" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>804</v>
+        <v>801</v>
       </c>
       <c r="C170" t="s">
-        <v>805</v>
+        <v>802</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>806</v>
+        <v>803</v>
       </c>
       <c r="C171" t="s">
-        <v>807</v>
+        <v>804</v>
       </c>
     </row>
     <row r="172" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>808</v>
+        <v>805</v>
       </c>
       <c r="C172" t="s">
-        <v>809</v>
+        <v>806</v>
       </c>
     </row>
     <row r="173" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>810</v>
+        <v>807</v>
       </c>
       <c r="B173" t="s">
-        <v>816</v>
+        <v>813</v>
       </c>
       <c r="C173" t="s">
-        <v>815</v>
+        <v>812</v>
       </c>
     </row>
     <row r="174" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
+        <v>808</v>
+      </c>
+      <c r="B174" t="s">
         <v>811</v>
       </c>
-      <c r="B174" t="s">
-        <v>814</v>
-      </c>
       <c r="C174" t="s">
-        <v>813</v>
+        <v>810</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>812</v>
+        <v>809</v>
       </c>
       <c r="B175" t="s">
         <v>80</v>
@@ -7640,90 +7640,90 @@
     </row>
     <row r="176" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>817</v>
+        <v>814</v>
       </c>
       <c r="B176" t="s">
-        <v>841</v>
+        <v>838</v>
       </c>
       <c r="C176" t="s">
-        <v>842</v>
+        <v>839</v>
       </c>
     </row>
     <row r="177" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>835</v>
+        <v>832</v>
       </c>
       <c r="B177" t="s">
-        <v>836</v>
+        <v>833</v>
       </c>
       <c r="C177" t="s">
-        <v>837</v>
+        <v>834</v>
       </c>
     </row>
     <row r="178" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>843</v>
+        <v>840</v>
       </c>
       <c r="B178" t="s">
-        <v>844</v>
+        <v>841</v>
       </c>
       <c r="C178" t="s">
-        <v>845</v>
+        <v>842</v>
       </c>
     </row>
     <row r="179" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>851</v>
+        <v>848</v>
       </c>
       <c r="B179" t="s">
-        <v>848</v>
+        <v>845</v>
       </c>
       <c r="C179" t="s">
-        <v>846</v>
+        <v>843</v>
       </c>
     </row>
     <row r="180" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>852</v>
+        <v>849</v>
       </c>
       <c r="B180" t="s">
-        <v>849</v>
+        <v>846</v>
       </c>
       <c r="C180" t="s">
-        <v>958</v>
+        <v>955</v>
       </c>
     </row>
     <row r="181" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>853</v>
+        <v>850</v>
       </c>
       <c r="B181" t="s">
-        <v>850</v>
+        <v>847</v>
       </c>
       <c r="C181" t="s">
-        <v>847</v>
+        <v>844</v>
       </c>
     </row>
     <row r="182" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
-        <v>854</v>
+        <v>851</v>
       </c>
       <c r="B182" t="s">
-        <v>855</v>
+        <v>852</v>
       </c>
       <c r="C182" t="s">
-        <v>862</v>
+        <v>859</v>
       </c>
     </row>
     <row r="183" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>863</v>
+        <v>860</v>
       </c>
       <c r="B183" t="s">
-        <v>865</v>
+        <v>862</v>
       </c>
       <c r="C183" t="s">
-        <v>864</v>
+        <v>861</v>
       </c>
     </row>
   </sheetData>
@@ -7778,7 +7778,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>866</v>
+        <v>863</v>
       </c>
       <c r="C2" t="s">
         <v>762</v>
@@ -7786,15 +7786,15 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>869</v>
+        <v>866</v>
       </c>
       <c r="C3" t="s">
-        <v>765</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>867</v>
+        <v>864</v>
       </c>
       <c r="C4" t="s">
         <v>761</v>
@@ -7802,15 +7802,15 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>870</v>
+        <v>867</v>
       </c>
       <c r="C5" t="s">
-        <v>763</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>868</v>
+        <v>865</v>
       </c>
       <c r="C6" t="s">
         <v>760</v>
@@ -7818,698 +7818,698 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>871</v>
+        <v>868</v>
       </c>
       <c r="C7" t="s">
-        <v>764</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>872</v>
+        <v>869</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>873</v>
+        <v>870</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>874</v>
+        <v>871</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
+        <v>872</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>875</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>878</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>876</v>
+        <v>873</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>877</v>
+        <v>874</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>879</v>
+        <v>876</v>
       </c>
       <c r="C14" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>880</v>
+        <v>877</v>
       </c>
       <c r="C15" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>881</v>
+        <v>878</v>
       </c>
       <c r="C16" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>882</v>
+        <v>879</v>
       </c>
       <c r="C17" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>883</v>
+        <v>880</v>
       </c>
       <c r="C18" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
       <c r="C19" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>885</v>
+        <v>882</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>886</v>
+        <v>883</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>887</v>
+        <v>884</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>884</v>
+        <v>881</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>888</v>
+        <v>885</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>889</v>
+        <v>886</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>890</v>
+        <v>887</v>
       </c>
       <c r="C26" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>891</v>
+        <v>888</v>
       </c>
       <c r="C27" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>892</v>
+        <v>889</v>
       </c>
       <c r="C28" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>893</v>
+        <v>890</v>
       </c>
       <c r="C29" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>894</v>
+        <v>891</v>
       </c>
       <c r="C30" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>895</v>
+        <v>892</v>
       </c>
       <c r="C31" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>896</v>
+        <v>893</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>897</v>
+        <v>894</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>898</v>
+        <v>895</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>899</v>
+        <v>896</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>900</v>
+        <v>897</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>901</v>
+        <v>898</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>902</v>
+        <v>899</v>
       </c>
       <c r="C38" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>903</v>
+        <v>900</v>
       </c>
       <c r="C39" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>904</v>
+        <v>901</v>
       </c>
       <c r="C40" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>905</v>
+        <v>902</v>
       </c>
       <c r="C41" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>906</v>
+        <v>903</v>
       </c>
       <c r="C42" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>907</v>
+        <v>904</v>
       </c>
       <c r="C43" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>908</v>
+        <v>905</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>909</v>
+        <v>906</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>910</v>
+        <v>907</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>911</v>
+        <v>908</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>912</v>
+        <v>909</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>913</v>
+        <v>910</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>914</v>
+        <v>911</v>
       </c>
       <c r="C50" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>915</v>
+        <v>912</v>
       </c>
       <c r="C51" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>916</v>
+        <v>913</v>
       </c>
       <c r="C52" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>917</v>
+        <v>914</v>
       </c>
       <c r="C53" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>918</v>
+        <v>915</v>
       </c>
       <c r="C54" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>919</v>
+        <v>916</v>
       </c>
       <c r="C55" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>920</v>
+        <v>917</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>921</v>
+        <v>918</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>922</v>
+        <v>919</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>923</v>
+        <v>920</v>
       </c>
       <c r="C59" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
-        <v>924</v>
+        <v>921</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>925</v>
+        <v>922</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>926</v>
+        <v>923</v>
       </c>
       <c r="C62" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>927</v>
+        <v>924</v>
       </c>
       <c r="C63" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>928</v>
+        <v>925</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>930</v>
+        <v>927</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>931</v>
+        <v>928</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>932</v>
+        <v>929</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>933</v>
+        <v>930</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>934</v>
+        <v>931</v>
       </c>
       <c r="C70" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>935</v>
+        <v>932</v>
       </c>
       <c r="C71" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>936</v>
+        <v>933</v>
       </c>
       <c r="C72" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>937</v>
+        <v>934</v>
       </c>
       <c r="C73" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>938</v>
+        <v>935</v>
       </c>
       <c r="C74" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>939</v>
+        <v>936</v>
       </c>
       <c r="C75" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
-        <v>940</v>
+        <v>937</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
-        <v>941</v>
+        <v>938</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
-        <v>942</v>
+        <v>939</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
-        <v>943</v>
+        <v>940</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
-        <v>944</v>
+        <v>941</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
-        <v>945</v>
+        <v>942</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>946</v>
+        <v>943</v>
       </c>
       <c r="C82" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>947</v>
+        <v>944</v>
       </c>
       <c r="C83" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>948</v>
+        <v>945</v>
       </c>
       <c r="C84" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>949</v>
+        <v>946</v>
       </c>
       <c r="C85" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>950</v>
+        <v>947</v>
       </c>
       <c r="C86" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>951</v>
+        <v>948</v>
       </c>
       <c r="C87" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
-        <v>952</v>
+        <v>949</v>
       </c>
       <c r="C88" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
-        <v>953</v>
+        <v>950</v>
       </c>
       <c r="C89" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="s">
-        <v>954</v>
+        <v>951</v>
       </c>
       <c r="C90" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
-        <v>955</v>
+        <v>952</v>
       </c>
       <c r="C91" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="5" t="s">
-        <v>956</v>
+        <v>953</v>
       </c>
       <c r="C92" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="5" t="s">
-        <v>957</v>
+        <v>954</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>878</v>
+        <v>875</v>
       </c>
     </row>
   </sheetData>
@@ -8539,178 +8539,178 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>766</v>
+        <v>763</v>
       </c>
       <c r="C2" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>768</v>
+        <v>765</v>
       </c>
       <c r="C3" t="s">
-        <v>788</v>
+        <v>785</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
       <c r="C4" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>771</v>
+        <v>768</v>
       </c>
       <c r="C5" t="s">
-        <v>772</v>
+        <v>769</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="C6" t="s">
-        <v>775</v>
+        <v>772</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>774</v>
+        <v>771</v>
       </c>
       <c r="C7" t="s">
-        <v>789</v>
+        <v>786</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>960</v>
+        <v>957</v>
       </c>
       <c r="C8" t="s">
-        <v>962</v>
+        <v>959</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>959</v>
+        <v>956</v>
       </c>
       <c r="C9" t="s">
-        <v>963</v>
+        <v>960</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>777</v>
+        <v>774</v>
       </c>
       <c r="C10" t="s">
-        <v>776</v>
+        <v>773</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>778</v>
+        <v>775</v>
       </c>
       <c r="C11" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="C12" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="C13" t="s">
-        <v>790</v>
+        <v>787</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
       <c r="C14" t="s">
-        <v>785</v>
+        <v>782</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>784</v>
+        <v>781</v>
       </c>
       <c r="C15" t="s">
-        <v>791</v>
+        <v>788</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="C16" t="s">
-        <v>796</v>
+        <v>793</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>787</v>
+        <v>784</v>
       </c>
       <c r="C17" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>793</v>
+        <v>790</v>
       </c>
       <c r="C18" t="s">
-        <v>792</v>
+        <v>789</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>794</v>
+        <v>791</v>
       </c>
       <c r="C19" t="s">
-        <v>795</v>
+        <v>792</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>965</v>
+        <v>962</v>
       </c>
       <c r="C20" t="s">
-        <v>961</v>
+        <v>958</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>966</v>
+        <v>963</v>
       </c>
       <c r="C21" t="s">
-        <v>964</v>
+        <v>961</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>967</v>
+        <v>964</v>
       </c>
       <c r="C22" t="s">
-        <v>969</v>
+        <v>966</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>968</v>
+        <v>965</v>
       </c>
       <c r="C23" t="s">
-        <v>970</v>
+        <v>967</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Create a Shop in game
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1135" uniqueCount="1006">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1156" uniqueCount="1023">
   <si>
     <t>ID</t>
   </si>
@@ -4020,6 +4020,57 @@
   </si>
   <si>
     <t>Dùng trong hành lý để tăng cho toàn bộ đội {0}% ST Bạo Kích trong 10 phút.</t>
+  </si>
+  <si>
+    <t>UI_COIN</t>
+  </si>
+  <si>
+    <t>Xu</t>
+  </si>
+  <si>
+    <t>UI_JADE</t>
+  </si>
+  <si>
+    <t>UI_DAILY</t>
+  </si>
+  <si>
+    <t>Daily</t>
+  </si>
+  <si>
+    <t>Ngày Thường</t>
+  </si>
+  <si>
+    <t>UI_RARE</t>
+  </si>
+  <si>
+    <t>UI_PROMOTION</t>
+  </si>
+  <si>
+    <t>Promotion</t>
+  </si>
+  <si>
+    <t>Quý hiếm</t>
+  </si>
+  <si>
+    <t>Ưu đãi</t>
+  </si>
+  <si>
+    <t>UI_BUNDLE</t>
+  </si>
+  <si>
+    <t>Bundle</t>
+  </si>
+  <si>
+    <t>Gói</t>
+  </si>
+  <si>
+    <t>STR_NUMBER_OF_PURCHASE</t>
+  </si>
+  <si>
+    <t>Number of purchase ({0}/{1})</t>
+  </si>
+  <si>
+    <t>Số lần mua ({0}/{1})</t>
   </si>
 </sst>
 </file>
@@ -4371,7 +4422,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.28515625" bestFit="1" customWidth="1"/>
@@ -5311,6 +5362,72 @@
       </c>
       <c r="C86" t="s">
         <v>1003</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>1006</v>
+      </c>
+      <c r="B87" t="s">
+        <v>611</v>
+      </c>
+      <c r="C87" t="s">
+        <v>1007</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B88" t="s">
+        <v>619</v>
+      </c>
+      <c r="C88" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B89" t="s">
+        <v>1010</v>
+      </c>
+      <c r="C89" t="s">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B90" t="s">
+        <v>447</v>
+      </c>
+      <c r="C90" t="s">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B91" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C91" t="s">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>1017</v>
+      </c>
+      <c r="B92" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C92" t="s">
+        <v>1019</v>
       </c>
     </row>
   </sheetData>
@@ -5745,7 +5862,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C183"/>
+  <dimension ref="A1:C184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.7109375" bestFit="1" customWidth="1"/>
@@ -7743,6 +7860,17 @@
       </c>
       <c r="C183" t="s">
         <v>859</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>1020</v>
+      </c>
+      <c r="B184" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C184" t="s">
+        <v>1022</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Make popup received items
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1168" uniqueCount="1033">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1171" uniqueCount="1036">
   <si>
     <t>ID</t>
   </si>
@@ -4101,6 +4101,15 @@
   </si>
   <si>
     <t>UI_UNIT_PRICE</t>
+  </si>
+  <si>
+    <t>UI_YOU_RECEIVED</t>
+  </si>
+  <si>
+    <t>Claimed successfully!</t>
+  </si>
+  <si>
+    <t>Chúc mừng đã nhận được</t>
   </si>
 </sst>
 </file>
@@ -4452,7 +4461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C93"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.28515625" bestFit="1" customWidth="1"/>
@@ -5469,6 +5478,17 @@
       </c>
       <c r="C93" t="s">
         <v>1031</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B94" t="s">
+        <v>1034</v>
+      </c>
+      <c r="C94" t="s">
+        <v>1035</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Make gacha system.
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1171" uniqueCount="1036">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1201" uniqueCount="1066">
   <si>
     <t>ID</t>
   </si>
@@ -4110,6 +4110,96 @@
   </si>
   <si>
     <t>Chúc mừng đã nhận được</t>
+  </si>
+  <si>
+    <t>STR_WEAPON_BANNER_TITLE</t>
+  </si>
+  <si>
+    <t>STR_CHARACTER_BANNER_TITLE</t>
+  </si>
+  <si>
+    <t>Anh Hùng Giáng Thế</t>
+  </si>
+  <si>
+    <t>Vũ Khí Truyền Thuyết</t>
+  </si>
+  <si>
+    <t>The Advent of Heroes</t>
+  </si>
+  <si>
+    <t>Legendary Weapon</t>
+  </si>
+  <si>
+    <t>UI_WISH</t>
+  </si>
+  <si>
+    <t>Wish</t>
+  </si>
+  <si>
+    <t>Tâm Nguyện</t>
+  </si>
+  <si>
+    <t>UI_TREASURE_SEEK</t>
+  </si>
+  <si>
+    <t>Treasure Seek</t>
+  </si>
+  <si>
+    <t>Tìm Báu</t>
+  </si>
+  <si>
+    <t>UI_GOD_SUMMON</t>
+  </si>
+  <si>
+    <t>God Summon</t>
+  </si>
+  <si>
+    <t>Thỉnh Thần</t>
+  </si>
+  <si>
+    <t>UI_PITY_NOTE</t>
+  </si>
+  <si>
+    <t>[SSR] guaranteed within x{0} summons.</t>
+  </si>
+  <si>
+    <t>Trong vòng {0} lần chắc chắn nhận được [SSR]</t>
+  </si>
+  <si>
+    <t>UI_SUMMON_5</t>
+  </si>
+  <si>
+    <t>Summon x5</t>
+  </si>
+  <si>
+    <t>Chiêu mộ x5</t>
+  </si>
+  <si>
+    <t>UI_SINGLE_SUMMON</t>
+  </si>
+  <si>
+    <t>Single Summon</t>
+  </si>
+  <si>
+    <t>Chiêu mộ đơn</t>
+  </si>
+  <si>
+    <t>UI_SUMMON_10</t>
+  </si>
+  <si>
+    <t>Summon x10</t>
+  </si>
+  <si>
+    <t>Chiêu mộ x10</t>
+  </si>
+  <si>
+    <t>UI_SKIP</t>
+  </si>
+  <si>
+    <t>Skip</t>
+  </si>
+  <si>
+    <t>Bỏ qua</t>
   </si>
 </sst>
 </file>
@@ -4461,7 +4551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C102"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.28515625" bestFit="1" customWidth="1"/>
@@ -5491,8 +5581,97 @@
         <v>1035</v>
       </c>
     </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>1042</v>
+      </c>
+      <c r="B95" t="s">
+        <v>1043</v>
+      </c>
+      <c r="C95" t="s">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B96" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C96" t="s">
+        <v>1047</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>1048</v>
+      </c>
+      <c r="B97" t="s">
+        <v>1049</v>
+      </c>
+      <c r="C97" t="s">
+        <v>1050</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>1051</v>
+      </c>
+      <c r="B98" t="s">
+        <v>1052</v>
+      </c>
+      <c r="C98" t="s">
+        <v>1053</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>1054</v>
+      </c>
+      <c r="B99" t="s">
+        <v>1055</v>
+      </c>
+      <c r="C99" t="s">
+        <v>1056</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>1057</v>
+      </c>
+      <c r="B100" t="s">
+        <v>1058</v>
+      </c>
+      <c r="C100" t="s">
+        <v>1059</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B101" t="s">
+        <v>1061</v>
+      </c>
+      <c r="C101" t="s">
+        <v>1062</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>1063</v>
+      </c>
+      <c r="B102" t="s">
+        <v>1064</v>
+      </c>
+      <c r="C102" t="s">
+        <v>1065</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -5923,7 +6102,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C187"/>
+  <dimension ref="A1:C189"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.7109375" bestFit="1" customWidth="1"/>
@@ -7965,6 +8144,28 @@
       </c>
       <c r="C187" t="s">
         <v>1031</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>1036</v>
+      </c>
+      <c r="B188" t="s">
+        <v>1040</v>
+      </c>
+      <c r="C188" t="s">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>1037</v>
+      </c>
+      <c r="B189" t="s">
+        <v>1041</v>
+      </c>
+      <c r="C189" t="s">
+        <v>1039</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Add pause menu in battle scene and fast forward and auto button for battle combat.
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="UI" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1258" uniqueCount="1121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1270" uniqueCount="1133">
   <si>
     <t>ID</t>
   </si>
@@ -4451,6 +4451,42 @@
   </si>
   <si>
     <t>Gacha</t>
+  </si>
+  <si>
+    <t>UI_QUIT</t>
+  </si>
+  <si>
+    <t>Quit</t>
+  </si>
+  <si>
+    <t>Thoát</t>
+  </si>
+  <si>
+    <t>UI_RETURN</t>
+  </si>
+  <si>
+    <t>Return</t>
+  </si>
+  <si>
+    <t>Trở lại</t>
+  </si>
+  <si>
+    <t>UI_RESTART</t>
+  </si>
+  <si>
+    <t>Restart</t>
+  </si>
+  <si>
+    <t>Chơi lại</t>
+  </si>
+  <si>
+    <t>STR_ARE_YOU_QUIT_BATTLE</t>
+  </si>
+  <si>
+    <t>Bạn có muốn rời khỏi trận đấu này chứ?</t>
+  </si>
+  <si>
+    <t>Are you sure you want to leave the match?</t>
   </si>
 </sst>
 </file>
@@ -4810,7 +4846,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C112"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.28515625" bestFit="1" customWidth="1"/>
@@ -6003,6 +6039,39 @@
       </c>
       <c r="C109" t="s">
         <v>1120</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>1121</v>
+      </c>
+      <c r="B110" t="s">
+        <v>1122</v>
+      </c>
+      <c r="C110" t="s">
+        <v>1123</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>1124</v>
+      </c>
+      <c r="B111" t="s">
+        <v>1125</v>
+      </c>
+      <c r="C111" t="s">
+        <v>1126</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B112" t="s">
+        <v>1128</v>
+      </c>
+      <c r="C112" t="s">
+        <v>1129</v>
       </c>
     </row>
   </sheetData>
@@ -6438,7 +6507,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C201"/>
+  <dimension ref="A1:C202"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.7109375" bestFit="1" customWidth="1"/>
@@ -8634,6 +8703,17 @@
       </c>
       <c r="C201" t="s">
         <v>1115</v>
+      </c>
+    </row>
+    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B202" t="s">
+        <v>1132</v>
+      </c>
+      <c r="C202" t="s">
+        <v>1131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Fix audio background sound and add localization for skill character.
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UI" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1409" uniqueCount="1277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1409" uniqueCount="1325">
   <si>
     <t>ID</t>
   </si>
@@ -2993,9 +2993,6 @@
     <t>Sa Ngộ Tĩnh</t>
   </si>
   <si>
-    <t>Đường Tăng Tạ</t>
-  </si>
-  <si>
     <t>Phật Tổ Như Lai</t>
   </si>
   <si>
@@ -3933,15 +3930,6 @@
   </si>
   <si>
     <t>UI_CRIT_DMG_RES</t>
-  </si>
-  <si>
-    <t>Gây ST bằng {0}% Tấn Công cho 1 kẻ địch.</t>
-  </si>
-  <si>
-    <t>Gây {0}% ST Tấn Công cho toàn bộ kẻ định đồng thời hồi {1}% ST gây ra.</t>
-  </si>
-  <si>
-    <t>Gây {0}% ST Tấn Công cho kẻ định, kèm thêm Giảm Phòng Thù cho mục tiêu, duy trì 2 hiệp.</t>
   </si>
   <si>
     <t>UI_COOLDOWN</t>
@@ -4919,6 +4907,162 @@
   </si>
   <si>
     <t>Mất lượt</t>
+  </si>
+  <si>
+    <t>Tam Nhẫn Trảm Không</t>
+  </si>
+  <si>
+    <t>Thiên Nhãn Phá Thần</t>
+  </si>
+  <si>
+    <t>Tam Tiên Đao</t>
+  </si>
+  <si>
+    <t>Phóng ra một tia thần quang hướng về phía mục tiêu, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Tung ra 3 nhát chém liên tiếp lên một kẻ địch, mỗi nhát gây ST bằng {0}% Tấn Công. Nếu mục tiêu bị hạ gục, các nhát chém còn lại sẽ tự động chuyển sang kẻ địch kế bên</t>
+  </si>
+  <si>
+    <t>Bạt Phong Trảm</t>
+  </si>
+  <si>
+    <t>Bảo Tháp Hộ Thể</t>
+  </si>
+  <si>
+    <t>rấn Ma Bảo Tháp</t>
+  </si>
+  <si>
+    <t>Tuốt kiếm chém nhanh một đòn dứt khoát, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Tung Lung Linh Bảo Tháp lên không trung, hóa thành khổng lồ gieo xuống như thái sơn áp đỉnh, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Bình Thiên Trảm</t>
+  </si>
+  <si>
+    <t>Ma Vương Bạt Khí</t>
+  </si>
+  <si>
+    <t>Kĩ năng XBích Thủy Tinh Thú Kích</t>
+  </si>
+  <si>
+    <t>Vung đại đao vung một nhát chém tựa dời núi lấp biển, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Ngưu Ma Vương ngửa mặt gầm lên một tiếng làm chấn động càn khôn, bộc phát ma khí ngút trời giúp bản thân vào trạng thái [Bình Thiên], tăng {0}% Tấn Công</t>
+  </si>
+  <si>
+    <t>Triệu hồi Bích Thủy Kim Tinh Thú giáng lâm, phóng ra luồng sóng chấn động mang kịch độc oanh kích mục tiêu, gây ST bằng {0}% Tấn Công cho [một kẻ địch / toàn bộ kẻ địch], đồng thời khiến đối phương rơi vào trạng thái [Kịch Độc], mỗi hiệp chịu ST Độc bằng {1}% Tấn Công trong {2} hiệp.</t>
+  </si>
+  <si>
+    <t>Cửu Xỉ Thần Bát</t>
+  </si>
+  <si>
+    <t>Thiên Bồng Giáp Trận</t>
+  </si>
+  <si>
+    <t>Thần Thể Biến Hóa</t>
+  </si>
+  <si>
+    <t>Vung Cửu Xỉ Đinh Ba gõ mạnh một cú chấn thiên, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Vận linh lực ngưng tụ thành lớp bảo hộ kiên cố, tạo cho bản thân lá chắn hấp thụ ST bằng {0}%HP.</t>
+  </si>
+  <si>
+    <t>Triệu hồi sức mạnh từ Lung Linh Bảo Tháp, tạo cho bản thân một lớp lá chắn hấp thụ lượng sát thương tương đương {0}% HP.</t>
+  </si>
+  <si>
+    <t>Thúc động bộc phát linh lực hóa thành cự thần khổng lồ, dốc toàn lực giáng một đòn trời giệt đất nát xuống mục tiêu, gây ST bằng {0}% Tấn Công cho một kẻ đich.</t>
+  </si>
+  <si>
+    <t>Hỏa Tiêm Đột Tấn</t>
+  </si>
+  <si>
+    <t>Càn Khôn Phá Trận</t>
+  </si>
+  <si>
+    <t>Hỏa Tiêm Liệt Hỏa</t>
+  </si>
+  <si>
+    <t>Áp sát mục tiêu, thúc động Hỏa Tiêm Thương bộc phát phun ra luồng lửa bão táp thiêu rụi đối phương, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Phóng Vòng Càn Khôn xoay chuyển cực tốc lao về phía mục tiêu, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Đâm mạnh Hỏa Tiêm Thương thẳng về phía trước, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Bảo Trượng Trảm</t>
+  </si>
+  <si>
+    <t>Lưu Cát Linh Dược</t>
+  </si>
+  <si>
+    <t>Lưu Cát Trầm Luân</t>
+  </si>
+  <si>
+    <t>Vung Huyền Trượng nện dứt khoát về phía trước, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Xoay mạnh Huyền Trượng rồi giáng một đòn cực uy lực xuống, cuốn theo sóng biển dâng trào càn quét đối phương, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Đường Tam Tạng</t>
+  </si>
+  <si>
+    <t>Tích Trượng Kim Quang</t>
+  </si>
+  <si>
+    <t>Kinh Mạn Kim Thân</t>
+  </si>
+  <si>
+    <t>Kính Bát Trấn Ma</t>
+  </si>
+  <si>
+    <t>Vung Tích Trượng về phía trước bắn ra luồng Phật quang thanh tẩy, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Ngưng tụ một màn kinh thư vàng xoay quanh bản thân, tạo lá chắn hấp thụ lượng sát thương tương đương {0}% Tấn Công</t>
+  </si>
+  <si>
+    <t>Áp sát kẻ địch, đưa Bát Vàng ra phóng chiếu luồng hào quang Phật pháp chói lọi, gây ST bằng {0}% Tấn Công cho một kẻ địch, đồng thời khiến mục tiêu bị [Choáng] trong 1 hiệp.</t>
+  </si>
+  <si>
+    <t>Bạch Long Kiếm Trảm</t>
+  </si>
+  <si>
+    <t>Càn Lôi Long Cầu</t>
+  </si>
+  <si>
+    <t>Hải Sóng Nộ Trào</t>
+  </si>
+  <si>
+    <t>Vung bảo kiếm chém dứt khoát một nhát về phía trước, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Triệu hồi Lôi Long ngưng tụ và bắn quả cầu sét về phía mục tiêu, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Vung bảo kiếm triệu hồi sóng thần cuộn trào càn quét toàn bộ trận địa, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Vung Tam Tiêm Đao chém dứt khoát một đòn về phía trước, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Tu một ngụm linh dược từ hồ lô, lập tức hồi phục {0}% Máu tối đa cho bản thân và tăng {1}% Phòng Thủ trong {2} hiệp.</t>
+  </si>
+  <si>
+    <t>Vung Như Ý Kim Cô Bổng giáng một đòn tàn khốc vỡ mật tan gan, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Vung Kim Cô Bổng hóa to nặng hàng ngàn cân giáng mạnh từ trên không xuống, sức nặng dời núi lấp biển, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
+  </si>
+  <si>
+    <t>Bứt một nhúm lông thổi nhẹ triệu hồi phân thân tham chiến, tấn công gây {0}% Tấn Công cho toàn bộ kẻ địch đồng thời phục hồi {1} % sát thương gây ra.</t>
   </si>
 </sst>
 </file>
@@ -4955,7 +5099,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4974,6 +5118,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -4987,7 +5137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4998,6 +5148,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5412,10 +5564,10 @@
         <v>32</v>
       </c>
       <c r="B12" t="s">
-        <v>1043</v>
+        <v>1039</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1042</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -5497,13 +5649,13 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>841</v>
+      </c>
+      <c r="B20" t="s">
         <v>842</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>843</v>
-      </c>
-      <c r="C20" t="s">
-        <v>844</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -5882,7 +6034,7 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="B55" t="s">
         <v>576</v>
@@ -5907,10 +6059,10 @@
         <v>583</v>
       </c>
       <c r="B57" t="s">
+        <v>944</v>
+      </c>
+      <c r="C57" t="s">
         <v>945</v>
-      </c>
-      <c r="C57" t="s">
-        <v>946</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -5921,7 +6073,7 @@
         <v>585</v>
       </c>
       <c r="C58" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -6013,227 +6165,227 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>707</v>
+      </c>
+      <c r="B68" t="s">
         <v>708</v>
       </c>
-      <c r="B68" t="s">
+      <c r="C68" t="s">
         <v>709</v>
-      </c>
-      <c r="C68" t="s">
-        <v>710</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>823</v>
+      </c>
+      <c r="B69" t="s">
         <v>824</v>
       </c>
-      <c r="B69" t="s">
+      <c r="C69" t="s">
         <v>825</v>
-      </c>
-      <c r="C69" t="s">
-        <v>826</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>803</v>
+      </c>
+      <c r="B70" t="s">
         <v>804</v>
       </c>
-      <c r="B70" t="s">
+      <c r="C70" t="s">
         <v>805</v>
-      </c>
-      <c r="C70" t="s">
-        <v>806</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>806</v>
+      </c>
+      <c r="B71" t="s">
         <v>807</v>
       </c>
-      <c r="B71" t="s">
+      <c r="C71" t="s">
         <v>808</v>
-      </c>
-      <c r="C71" t="s">
-        <v>809</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="B72" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="C72" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>812</v>
+      </c>
+      <c r="B73" t="s">
+        <v>811</v>
+      </c>
+      <c r="C73" t="s">
         <v>813</v>
-      </c>
-      <c r="B73" t="s">
-        <v>812</v>
-      </c>
-      <c r="C73" t="s">
-        <v>814</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>817</v>
+        <v>816</v>
       </c>
       <c r="B74" t="s">
-        <v>816</v>
+        <v>815</v>
       </c>
       <c r="C74" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>817</v>
+      </c>
+      <c r="B75" t="s">
         <v>818</v>
       </c>
-      <c r="B75" t="s">
+      <c r="C75" t="s">
         <v>819</v>
-      </c>
-      <c r="C75" t="s">
-        <v>820</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>844</v>
+      </c>
+      <c r="B76" t="s">
         <v>845</v>
       </c>
-      <c r="B76" t="s">
+      <c r="C76" t="s">
         <v>846</v>
-      </c>
-      <c r="C76" t="s">
-        <v>847</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="B77" t="s">
+        <v>948</v>
+      </c>
+      <c r="C77" t="s">
         <v>949</v>
-      </c>
-      <c r="C77" t="s">
-        <v>950</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>950</v>
+      </c>
+      <c r="B78" t="s">
         <v>951</v>
       </c>
-      <c r="B78" t="s">
+      <c r="C78" t="s">
         <v>952</v>
-      </c>
-      <c r="C78" t="s">
-        <v>953</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="B79" t="s">
+        <v>954</v>
+      </c>
+      <c r="C79" t="s">
         <v>955</v>
-      </c>
-      <c r="C79" t="s">
-        <v>956</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="B80" t="s">
+        <v>959</v>
+      </c>
+      <c r="C80" t="s">
         <v>960</v>
-      </c>
-      <c r="C80" t="s">
-        <v>961</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>959</v>
+        <v>958</v>
       </c>
       <c r="B81" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="C81" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>967</v>
+        <v>966</v>
       </c>
       <c r="B82" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="C82" t="s">
-        <v>965</v>
+        <v>964</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>967</v>
+      </c>
+      <c r="B83" t="s">
+        <v>965</v>
+      </c>
+      <c r="C83" t="s">
         <v>968</v>
-      </c>
-      <c r="B83" t="s">
-        <v>966</v>
-      </c>
-      <c r="C83" t="s">
-        <v>969</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="B84" t="s">
         <v>631</v>
       </c>
       <c r="C84" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>972</v>
+      </c>
+      <c r="B85" t="s">
         <v>973</v>
       </c>
-      <c r="B85" t="s">
+      <c r="C85" t="s">
         <v>974</v>
-      </c>
-      <c r="C85" t="s">
-        <v>975</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>980</v>
+        <v>976</v>
       </c>
       <c r="B86" t="s">
-        <v>981</v>
+        <v>977</v>
       </c>
       <c r="C86" t="s">
-        <v>982</v>
+        <v>978</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>985</v>
+        <v>981</v>
       </c>
       <c r="B87" t="s">
         <v>609</v>
       </c>
       <c r="C87" t="s">
-        <v>986</v>
+        <v>982</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>987</v>
+        <v>983</v>
       </c>
       <c r="B88" t="s">
         <v>617</v>
@@ -6244,219 +6396,219 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>988</v>
+        <v>984</v>
       </c>
       <c r="B89" t="s">
-        <v>989</v>
+        <v>985</v>
       </c>
       <c r="C89" t="s">
-        <v>990</v>
+        <v>986</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>991</v>
+        <v>987</v>
       </c>
       <c r="B90" t="s">
         <v>445</v>
       </c>
       <c r="C90" t="s">
-        <v>994</v>
+        <v>990</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>992</v>
+        <v>988</v>
       </c>
       <c r="B91" t="s">
-        <v>993</v>
+        <v>989</v>
       </c>
       <c r="C91" t="s">
-        <v>995</v>
+        <v>991</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>996</v>
+        <v>992</v>
       </c>
       <c r="B92" t="s">
-        <v>997</v>
+        <v>993</v>
       </c>
       <c r="C92" t="s">
-        <v>998</v>
+        <v>994</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>1011</v>
+        <v>1007</v>
       </c>
       <c r="B93" t="s">
-        <v>1009</v>
+        <v>1005</v>
       </c>
       <c r="C93" t="s">
-        <v>1010</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>1012</v>
+        <v>1008</v>
       </c>
       <c r="B94" t="s">
-        <v>1013</v>
+        <v>1009</v>
       </c>
       <c r="C94" t="s">
-        <v>1014</v>
+        <v>1010</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>1021</v>
+        <v>1017</v>
       </c>
       <c r="B95" t="s">
-        <v>1022</v>
+        <v>1018</v>
       </c>
       <c r="C95" t="s">
-        <v>1023</v>
+        <v>1019</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="B96" t="s">
-        <v>1025</v>
+        <v>1021</v>
       </c>
       <c r="C96" t="s">
-        <v>1026</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>1027</v>
+        <v>1023</v>
       </c>
       <c r="B97" t="s">
-        <v>1028</v>
+        <v>1024</v>
       </c>
       <c r="C97" t="s">
-        <v>1029</v>
+        <v>1025</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>1030</v>
+        <v>1026</v>
       </c>
       <c r="B98" t="s">
-        <v>1031</v>
+        <v>1027</v>
       </c>
       <c r="C98" t="s">
-        <v>1032</v>
+        <v>1028</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>1033</v>
+        <v>1029</v>
       </c>
       <c r="B99" t="s">
-        <v>1034</v>
+        <v>1030</v>
       </c>
       <c r="C99" t="s">
-        <v>1195</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>1035</v>
+        <v>1031</v>
       </c>
       <c r="B100" t="s">
-        <v>1036</v>
+        <v>1032</v>
       </c>
       <c r="C100" t="s">
-        <v>1196</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>1037</v>
+        <v>1033</v>
       </c>
       <c r="B101" t="s">
-        <v>1038</v>
+        <v>1034</v>
       </c>
       <c r="C101" t="s">
-        <v>1197</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>1039</v>
+        <v>1035</v>
       </c>
       <c r="B102" t="s">
-        <v>1040</v>
+        <v>1036</v>
       </c>
       <c r="C102" t="s">
-        <v>1041</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>1044</v>
+        <v>1040</v>
       </c>
       <c r="B103" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="C103" t="s">
-        <v>1046</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>1047</v>
+        <v>1043</v>
       </c>
       <c r="B104" t="s">
-        <v>1048</v>
+        <v>1044</v>
       </c>
       <c r="C104" t="s">
-        <v>1049</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>1050</v>
+        <v>1046</v>
       </c>
       <c r="B105" t="s">
-        <v>1051</v>
+        <v>1047</v>
       </c>
       <c r="C105" t="s">
-        <v>1052</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>1053</v>
+        <v>1049</v>
       </c>
       <c r="B106" t="s">
-        <v>1054</v>
+        <v>1050</v>
       </c>
       <c r="C106" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>1056</v>
+        <v>1052</v>
       </c>
       <c r="B107" t="s">
-        <v>1057</v>
+        <v>1053</v>
       </c>
       <c r="C107" t="s">
-        <v>1058</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>1059</v>
+        <v>1055</v>
       </c>
       <c r="B108" t="s">
-        <v>1060</v>
+        <v>1056</v>
       </c>
       <c r="C108" t="s">
         <v>43</v>
@@ -6464,123 +6616,123 @@
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>1097</v>
+        <v>1093</v>
       </c>
       <c r="B109" t="s">
-        <v>1098</v>
+        <v>1094</v>
       </c>
       <c r="C109" t="s">
-        <v>1098</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>1099</v>
+        <v>1095</v>
       </c>
       <c r="B110" t="s">
-        <v>1100</v>
+        <v>1096</v>
       </c>
       <c r="C110" t="s">
-        <v>1101</v>
+        <v>1097</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>1102</v>
+        <v>1098</v>
       </c>
       <c r="B111" t="s">
-        <v>1103</v>
+        <v>1099</v>
       </c>
       <c r="C111" t="s">
-        <v>1104</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>1105</v>
+        <v>1101</v>
       </c>
       <c r="B112" t="s">
-        <v>1106</v>
+        <v>1102</v>
       </c>
       <c r="C112" t="s">
-        <v>1107</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>1128</v>
+        <v>1124</v>
       </c>
       <c r="B113" t="s">
-        <v>1127</v>
+        <v>1123</v>
       </c>
       <c r="C113" t="s">
-        <v>1126</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>1202</v>
+        <v>1198</v>
       </c>
       <c r="B114" t="s">
-        <v>1203</v>
+        <v>1199</v>
       </c>
       <c r="C114" t="s">
-        <v>1204</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>1205</v>
+        <v>1201</v>
       </c>
       <c r="B115" t="s">
-        <v>1207</v>
+        <v>1203</v>
       </c>
       <c r="C115" t="s">
-        <v>1206</v>
+        <v>1202</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>1208</v>
+        <v>1204</v>
       </c>
       <c r="B116" t="s">
-        <v>1209</v>
+        <v>1205</v>
       </c>
       <c r="C116" t="s">
-        <v>1210</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>1211</v>
+        <v>1207</v>
       </c>
       <c r="B117" t="s">
-        <v>1212</v>
+        <v>1208</v>
       </c>
       <c r="C117" t="s">
-        <v>1213</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>1214</v>
+        <v>1210</v>
       </c>
       <c r="B118" t="s">
-        <v>1215</v>
+        <v>1211</v>
       </c>
       <c r="C118" t="s">
-        <v>1216</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>1258</v>
+        <v>1254</v>
       </c>
       <c r="B119" t="s">
-        <v>1259</v>
+        <v>1255</v>
       </c>
       <c r="C119" t="s">
-        <v>1260</v>
+        <v>1256</v>
       </c>
     </row>
   </sheetData>
@@ -6656,337 +6808,337 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
       <c r="B6" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="C6" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>666</v>
+      </c>
+      <c r="B7" t="s">
         <v>667</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>668</v>
-      </c>
-      <c r="C7" t="s">
-        <v>669</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>669</v>
+      </c>
+      <c r="B8" t="s">
         <v>670</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>671</v>
-      </c>
-      <c r="C8" t="s">
-        <v>672</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>672</v>
+      </c>
+      <c r="B9" t="s">
         <v>673</v>
       </c>
-      <c r="B9" t="s">
-        <v>674</v>
-      </c>
       <c r="C9" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>674</v>
+      </c>
+      <c r="B10" t="s">
         <v>675</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>676</v>
-      </c>
-      <c r="C10" t="s">
-        <v>677</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>678</v>
+      </c>
+      <c r="B11" t="s">
         <v>679</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>680</v>
-      </c>
-      <c r="C11" t="s">
-        <v>681</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>681</v>
+      </c>
+      <c r="C12" t="s">
         <v>682</v>
-      </c>
-      <c r="C12" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>683</v>
+      </c>
+      <c r="C13" t="s">
         <v>684</v>
-      </c>
-      <c r="C13" t="s">
-        <v>685</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>685</v>
+      </c>
+      <c r="C14" t="s">
         <v>686</v>
-      </c>
-      <c r="C14" t="s">
-        <v>687</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>687</v>
+      </c>
+      <c r="C15" t="s">
         <v>688</v>
-      </c>
-      <c r="C15" t="s">
-        <v>689</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>689</v>
+      </c>
+      <c r="C16" t="s">
         <v>690</v>
-      </c>
-      <c r="C16" t="s">
-        <v>691</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>691</v>
+      </c>
+      <c r="C17" t="s">
         <v>692</v>
-      </c>
-      <c r="C17" t="s">
-        <v>693</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
       <c r="C18" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>694</v>
+      </c>
+      <c r="C19" t="s">
         <v>695</v>
-      </c>
-      <c r="C19" t="s">
-        <v>696</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>696</v>
+      </c>
+      <c r="C20" t="s">
         <v>697</v>
-      </c>
-      <c r="C20" t="s">
-        <v>698</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>698</v>
+      </c>
+      <c r="C21" t="s">
         <v>699</v>
-      </c>
-      <c r="C21" t="s">
-        <v>700</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>700</v>
+      </c>
+      <c r="C22" t="s">
         <v>701</v>
-      </c>
-      <c r="C22" t="s">
-        <v>702</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
       <c r="C23" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>703</v>
+      </c>
+      <c r="C24" t="s">
         <v>704</v>
-      </c>
-      <c r="C24" t="s">
-        <v>705</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>705</v>
+      </c>
+      <c r="C25" t="s">
         <v>706</v>
-      </c>
-      <c r="C25" t="s">
-        <v>707</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>713</v>
+      </c>
+      <c r="C26" t="s">
         <v>714</v>
-      </c>
-      <c r="C26" t="s">
-        <v>715</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="C27" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>716</v>
+      </c>
+      <c r="C28" t="s">
         <v>717</v>
-      </c>
-      <c r="C28" t="s">
-        <v>718</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="C29" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="C30" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="C31" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="C32" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>722</v>
+      </c>
+      <c r="C33" t="s">
         <v>723</v>
-      </c>
-      <c r="C33" t="s">
-        <v>724</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="C34" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>725</v>
+      </c>
+      <c r="C35" t="s">
         <v>726</v>
-      </c>
-      <c r="C35" t="s">
-        <v>727</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>727</v>
+      </c>
+      <c r="C36" t="s">
         <v>728</v>
-      </c>
-      <c r="C36" t="s">
-        <v>729</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>729</v>
+      </c>
+      <c r="C37" t="s">
         <v>730</v>
-      </c>
-      <c r="C37" t="s">
-        <v>731</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="C38" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="C39" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="C40" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="C41" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="C42" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="C43" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="C44" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="C45" t="s">
         <v>163</v>
@@ -6994,18 +7146,18 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>751</v>
+      </c>
+      <c r="C46" t="s">
         <v>752</v>
-      </c>
-      <c r="C46" t="s">
-        <v>753</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>753</v>
+      </c>
+      <c r="C47" t="s">
         <v>754</v>
-      </c>
-      <c r="C47" t="s">
-        <v>755</v>
       </c>
     </row>
   </sheetData>
@@ -7252,7 +7404,7 @@
         <v>133</v>
       </c>
       <c r="C21" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -7450,7 +7602,7 @@
         <v>176</v>
       </c>
       <c r="C39" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -7681,7 +7833,7 @@
         <v>262</v>
       </c>
       <c r="C60" t="s">
-        <v>983</v>
+        <v>979</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -7747,7 +7899,7 @@
         <v>260</v>
       </c>
       <c r="C66" t="s">
-        <v>984</v>
+        <v>980</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
@@ -8462,7 +8614,7 @@
         <v>466</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>663</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
@@ -8849,77 +9001,77 @@
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
+        <v>790</v>
+      </c>
+      <c r="C167" t="s">
         <v>791</v>
-      </c>
-      <c r="C167" t="s">
-        <v>792</v>
       </c>
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
+        <v>792</v>
+      </c>
+      <c r="C168" t="s">
         <v>793</v>
-      </c>
-      <c r="C168" t="s">
-        <v>794</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
+        <v>794</v>
+      </c>
+      <c r="C169" t="s">
         <v>795</v>
-      </c>
-      <c r="C169" t="s">
-        <v>796</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
+        <v>796</v>
+      </c>
+      <c r="C170" t="s">
         <v>797</v>
-      </c>
-      <c r="C170" t="s">
-        <v>798</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
+        <v>798</v>
+      </c>
+      <c r="C171" t="s">
         <v>799</v>
-      </c>
-      <c r="C171" t="s">
-        <v>800</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
+        <v>800</v>
+      </c>
+      <c r="C172" t="s">
         <v>801</v>
-      </c>
-      <c r="C172" t="s">
-        <v>802</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>1261</v>
+        <v>1257</v>
       </c>
       <c r="B173" t="s">
-        <v>1262</v>
+        <v>1258</v>
       </c>
       <c r="C173" t="s">
-        <v>1263</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>1265</v>
+        <v>1261</v>
       </c>
       <c r="B174" t="s">
-        <v>1267</v>
+        <v>1263</v>
       </c>
       <c r="C174" t="s">
-        <v>1264</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>1266</v>
+        <v>1262</v>
       </c>
       <c r="B175" t="s">
         <v>78</v>
@@ -8930,761 +9082,761 @@
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="B176" t="s">
+        <v>826</v>
+      </c>
+      <c r="C176" t="s">
         <v>827</v>
-      </c>
-      <c r="C176" t="s">
-        <v>828</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
+        <v>820</v>
+      </c>
+      <c r="B177" t="s">
         <v>821</v>
       </c>
-      <c r="B177" t="s">
+      <c r="C177" t="s">
         <v>822</v>
-      </c>
-      <c r="C177" t="s">
-        <v>823</v>
       </c>
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
+        <v>828</v>
+      </c>
+      <c r="B178" t="s">
         <v>829</v>
       </c>
-      <c r="B178" t="s">
+      <c r="C178" t="s">
         <v>830</v>
-      </c>
-      <c r="C178" t="s">
-        <v>831</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="B179" t="s">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="C179" t="s">
-        <v>832</v>
+        <v>831</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="B180" t="s">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="C180" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="B181" t="s">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="C181" t="s">
-        <v>833</v>
+        <v>832</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
+        <v>839</v>
+      </c>
+      <c r="B182" t="s">
         <v>840</v>
       </c>
-      <c r="B182" t="s">
-        <v>841</v>
-      </c>
       <c r="C182" t="s">
-        <v>848</v>
+        <v>847</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
+        <v>848</v>
+      </c>
+      <c r="B183" t="s">
+        <v>850</v>
+      </c>
+      <c r="C183" t="s">
         <v>849</v>
-      </c>
-      <c r="B183" t="s">
-        <v>851</v>
-      </c>
-      <c r="C183" t="s">
-        <v>850</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
-        <v>999</v>
+        <v>995</v>
       </c>
       <c r="B184" t="s">
-        <v>1000</v>
+        <v>996</v>
       </c>
       <c r="C184" t="s">
-        <v>1001</v>
+        <v>997</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>1002</v>
+        <v>998</v>
       </c>
       <c r="B185" t="s">
-        <v>1004</v>
+        <v>1000</v>
       </c>
       <c r="C185" t="s">
-        <v>1005</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
+        <v>999</v>
+      </c>
+      <c r="B186" t="s">
         <v>1003</v>
       </c>
-      <c r="B186" t="s">
-        <v>1007</v>
-      </c>
       <c r="C186" t="s">
-        <v>1006</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>1008</v>
+        <v>1004</v>
       </c>
       <c r="B187" t="s">
-        <v>1009</v>
+        <v>1005</v>
       </c>
       <c r="C187" t="s">
-        <v>1010</v>
+        <v>1006</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
+        <v>1011</v>
+      </c>
+      <c r="B188" t="s">
         <v>1015</v>
       </c>
-      <c r="B188" t="s">
-        <v>1019</v>
-      </c>
       <c r="C188" t="s">
-        <v>1017</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B189" t="s">
         <v>1016</v>
       </c>
-      <c r="B189" t="s">
-        <v>1020</v>
-      </c>
       <c r="C189" t="s">
-        <v>1018</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>1061</v>
+        <v>1057</v>
       </c>
       <c r="B190" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="C190" t="s">
-        <v>1070</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>1062</v>
+        <v>1058</v>
       </c>
       <c r="B191" t="s">
-        <v>1079</v>
+        <v>1075</v>
       </c>
       <c r="C191" t="s">
-        <v>1072</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>1063</v>
+        <v>1059</v>
       </c>
       <c r="B192" t="s">
-        <v>1080</v>
+        <v>1076</v>
       </c>
       <c r="C192" t="s">
-        <v>1071</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>1064</v>
+        <v>1060</v>
       </c>
       <c r="B193" t="s">
-        <v>1081</v>
+        <v>1077</v>
       </c>
       <c r="C193" t="s">
-        <v>1076</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>1065</v>
+        <v>1061</v>
       </c>
       <c r="B194" t="s">
-        <v>1082</v>
+        <v>1078</v>
       </c>
       <c r="C194" t="s">
-        <v>1087</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>1066</v>
+        <v>1062</v>
       </c>
       <c r="B195" t="s">
-        <v>1085</v>
+        <v>1081</v>
       </c>
       <c r="C195" t="s">
-        <v>1077</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>1067</v>
+        <v>1063</v>
       </c>
       <c r="B196" t="s">
-        <v>1083</v>
+        <v>1079</v>
       </c>
       <c r="C196" t="s">
-        <v>1073</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>1068</v>
+        <v>1064</v>
       </c>
       <c r="B197" t="s">
-        <v>1084</v>
+        <v>1080</v>
       </c>
       <c r="C197" t="s">
-        <v>1074</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>1069</v>
+        <v>1065</v>
       </c>
       <c r="B198" t="s">
-        <v>1086</v>
+        <v>1082</v>
       </c>
       <c r="C198" t="s">
-        <v>1075</v>
+        <v>1071</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>1088</v>
+        <v>1084</v>
       </c>
       <c r="B199" t="s">
-        <v>1094</v>
+        <v>1090</v>
       </c>
       <c r="C199" t="s">
-        <v>1091</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>1089</v>
+        <v>1085</v>
       </c>
       <c r="B200" t="s">
-        <v>1095</v>
+        <v>1091</v>
       </c>
       <c r="C200" t="s">
-        <v>1092</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>1090</v>
+        <v>1086</v>
       </c>
       <c r="B201" t="s">
-        <v>1096</v>
+        <v>1092</v>
       </c>
       <c r="C201" t="s">
-        <v>1093</v>
+        <v>1089</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
-        <v>1108</v>
+        <v>1104</v>
       </c>
       <c r="B202" t="s">
-        <v>1110</v>
+        <v>1106</v>
       </c>
       <c r="C202" t="s">
-        <v>1109</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
+        <v>1107</v>
+      </c>
+      <c r="B203" t="s">
         <v>1111</v>
       </c>
-      <c r="B203" t="s">
-        <v>1115</v>
-      </c>
       <c r="C203" t="s">
-        <v>1112</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>1114</v>
+        <v>1110</v>
       </c>
       <c r="B204" t="s">
-        <v>1116</v>
+        <v>1112</v>
       </c>
       <c r="C204" t="s">
-        <v>1113</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
-        <v>1117</v>
+        <v>1113</v>
       </c>
       <c r="B205" t="s">
-        <v>1119</v>
+        <v>1115</v>
       </c>
       <c r="C205" t="s">
-        <v>1118</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>1120</v>
+        <v>1116</v>
       </c>
       <c r="B206" t="s">
-        <v>1121</v>
+        <v>1117</v>
       </c>
       <c r="C206" t="s">
-        <v>1122</v>
+        <v>1118</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>1123</v>
+        <v>1119</v>
       </c>
       <c r="B207" t="s">
-        <v>1124</v>
+        <v>1120</v>
       </c>
       <c r="C207" t="s">
-        <v>1125</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>1129</v>
+        <v>1125</v>
       </c>
       <c r="B208" t="s">
-        <v>1130</v>
+        <v>1126</v>
       </c>
       <c r="C208" t="s">
-        <v>1131</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>1132</v>
+        <v>1128</v>
       </c>
       <c r="B209" t="s">
-        <v>1134</v>
+        <v>1130</v>
       </c>
       <c r="C209" t="s">
-        <v>1133</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>1135</v>
+        <v>1131</v>
       </c>
       <c r="B210" t="s">
-        <v>1137</v>
+        <v>1133</v>
       </c>
       <c r="C210" t="s">
-        <v>1136</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>1138</v>
+        <v>1134</v>
       </c>
       <c r="B211" t="s">
-        <v>1147</v>
+        <v>1143</v>
       </c>
       <c r="C211" t="s">
-        <v>1146</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>1140</v>
+        <v>1136</v>
       </c>
       <c r="B212" t="s">
-        <v>1141</v>
+        <v>1137</v>
       </c>
       <c r="C212" t="s">
-        <v>1217</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>1142</v>
+        <v>1138</v>
       </c>
       <c r="B213" t="s">
-        <v>1144</v>
+        <v>1140</v>
       </c>
       <c r="C213" t="s">
-        <v>1143</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>1145</v>
+        <v>1141</v>
       </c>
       <c r="B214" t="s">
-        <v>1139</v>
+        <v>1135</v>
       </c>
       <c r="C214" t="s">
-        <v>1218</v>
+        <v>1214</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>1148</v>
+        <v>1144</v>
       </c>
       <c r="B215" t="s">
+        <v>1145</v>
+      </c>
+      <c r="C215" t="s">
         <v>1149</v>
-      </c>
-      <c r="C215" t="s">
-        <v>1153</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>1150</v>
+        <v>1146</v>
       </c>
       <c r="B216" t="s">
-        <v>1152</v>
+        <v>1148</v>
       </c>
       <c r="C216" t="s">
-        <v>1151</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>1154</v>
+        <v>1150</v>
       </c>
       <c r="B217" t="s">
-        <v>1156</v>
+        <v>1152</v>
       </c>
       <c r="C217" t="s">
-        <v>1155</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>1157</v>
+        <v>1153</v>
       </c>
       <c r="B218" t="s">
-        <v>1159</v>
+        <v>1155</v>
       </c>
       <c r="C218" t="s">
-        <v>1158</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>1160</v>
+        <v>1156</v>
       </c>
       <c r="B219" t="s">
-        <v>1162</v>
+        <v>1158</v>
       </c>
       <c r="C219" t="s">
-        <v>1161</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
+        <v>1159</v>
+      </c>
+      <c r="B220" t="s">
         <v>1163</v>
       </c>
-      <c r="B220" t="s">
-        <v>1167</v>
-      </c>
       <c r="C220" t="s">
-        <v>1166</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
+        <v>1160</v>
+      </c>
+      <c r="B221" t="s">
+        <v>1165</v>
+      </c>
+      <c r="C221" t="s">
         <v>1164</v>
-      </c>
-      <c r="B221" t="s">
-        <v>1169</v>
-      </c>
-      <c r="C221" t="s">
-        <v>1168</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>1165</v>
+        <v>1161</v>
       </c>
       <c r="B222" t="s">
-        <v>1170</v>
+        <v>1166</v>
       </c>
       <c r="C222" t="s">
-        <v>1171</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
+        <v>1168</v>
+      </c>
+      <c r="B223" t="s">
         <v>1172</v>
       </c>
-      <c r="B223" t="s">
-        <v>1176</v>
-      </c>
       <c r="C223" t="s">
-        <v>1175</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
+        <v>1169</v>
+      </c>
+      <c r="B224" t="s">
+        <v>1174</v>
+      </c>
+      <c r="C224" t="s">
         <v>1173</v>
-      </c>
-      <c r="B224" t="s">
-        <v>1178</v>
-      </c>
-      <c r="C224" t="s">
-        <v>1177</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>1174</v>
+        <v>1170</v>
       </c>
       <c r="B225" t="s">
-        <v>1180</v>
+        <v>1176</v>
       </c>
       <c r="C225" t="s">
-        <v>1179</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>1181</v>
+        <v>1177</v>
       </c>
       <c r="B226" t="s">
-        <v>1186</v>
+        <v>1182</v>
       </c>
       <c r="C226" t="s">
-        <v>1184</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>1182</v>
+        <v>1178</v>
       </c>
       <c r="B227" t="s">
-        <v>1187</v>
+        <v>1183</v>
       </c>
       <c r="C227" t="s">
-        <v>1194</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>1183</v>
+        <v>1179</v>
       </c>
       <c r="B228" t="s">
-        <v>1188</v>
+        <v>1184</v>
       </c>
       <c r="C228" t="s">
-        <v>1185</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>1189</v>
+        <v>1185</v>
       </c>
       <c r="B229" t="s">
-        <v>1199</v>
+        <v>1195</v>
       </c>
       <c r="C229" t="s">
-        <v>1192</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>1191</v>
+        <v>1187</v>
       </c>
       <c r="B230" t="s">
-        <v>1200</v>
+        <v>1196</v>
       </c>
       <c r="C230" t="s">
-        <v>1193</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>1190</v>
+        <v>1186</v>
       </c>
       <c r="B231" t="s">
-        <v>1201</v>
+        <v>1197</v>
       </c>
       <c r="C231" t="s">
-        <v>1198</v>
+        <v>1194</v>
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>1219</v>
+        <v>1215</v>
       </c>
       <c r="B232" t="s">
-        <v>1221</v>
+        <v>1217</v>
       </c>
       <c r="C232" t="s">
-        <v>1220</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>1222</v>
+        <v>1218</v>
       </c>
       <c r="B233" t="s">
-        <v>1223</v>
+        <v>1219</v>
       </c>
       <c r="C233" t="s">
-        <v>1224</v>
+        <v>1220</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>1225</v>
+        <v>1221</v>
       </c>
       <c r="B234" t="s">
-        <v>1226</v>
+        <v>1222</v>
       </c>
       <c r="C234" t="s">
-        <v>1227</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>1228</v>
+        <v>1224</v>
       </c>
       <c r="B235" t="s">
-        <v>1229</v>
+        <v>1225</v>
       </c>
       <c r="C235" t="s">
-        <v>1230</v>
+        <v>1226</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>1231</v>
+        <v>1227</v>
       </c>
       <c r="B236" t="s">
-        <v>1232</v>
+        <v>1228</v>
       </c>
       <c r="C236" t="s">
-        <v>1233</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>1237</v>
+        <v>1233</v>
       </c>
       <c r="B237" t="s">
-        <v>1238</v>
+        <v>1234</v>
       </c>
       <c r="C237" t="s">
-        <v>1239</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>1234</v>
+        <v>1230</v>
       </c>
       <c r="B238" t="s">
-        <v>1235</v>
+        <v>1231</v>
       </c>
       <c r="C238" t="s">
-        <v>1236</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>1240</v>
+        <v>1236</v>
       </c>
       <c r="B239" t="s">
-        <v>1241</v>
+        <v>1237</v>
       </c>
       <c r="C239" t="s">
-        <v>1242</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>1245</v>
+        <v>1241</v>
       </c>
       <c r="B240" t="s">
-        <v>1243</v>
+        <v>1239</v>
       </c>
       <c r="C240" t="s">
-        <v>1244</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>1246</v>
+        <v>1242</v>
       </c>
       <c r="B241" t="s">
-        <v>1247</v>
+        <v>1243</v>
       </c>
       <c r="C241" t="s">
-        <v>1248</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>1255</v>
+        <v>1251</v>
       </c>
       <c r="B242" t="s">
-        <v>1256</v>
+        <v>1252</v>
       </c>
       <c r="C242" t="s">
-        <v>1257</v>
+        <v>1253</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>1268</v>
+        <v>1264</v>
       </c>
       <c r="B243" t="s">
-        <v>1270</v>
+        <v>1266</v>
       </c>
       <c r="C243" t="s">
-        <v>1269</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>1274</v>
+        <v>1270</v>
       </c>
       <c r="B244" t="s">
-        <v>1275</v>
+        <v>1271</v>
       </c>
       <c r="C244" t="s">
-        <v>1276</v>
+        <v>1272</v>
       </c>
     </row>
   </sheetData>
@@ -9701,7 +9853,7 @@
   <cols>
     <col min="1" max="1" width="34.28515625" customWidth="1"/>
     <col min="2" max="2" width="31.7109375" customWidth="1"/>
-    <col min="3" max="3" width="36.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="82" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -9717,690 +9869,690 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="C2" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="C3" t="s">
-        <v>977</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="C4" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="C5" t="s">
-        <v>978</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="C6" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="C7" t="s">
-        <v>979</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>864</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>864</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>860</v>
+        <v>859</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>864</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>861</v>
+        <v>860</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>864</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>862</v>
+        <v>861</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>864</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>863</v>
+        <v>862</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>864</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>865</v>
+        <v>864</v>
       </c>
       <c r="C14" t="s">
-        <v>864</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>866</v>
+        <v>865</v>
       </c>
       <c r="C15" t="s">
-        <v>864</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="C16" t="s">
-        <v>864</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>868</v>
+        <v>867</v>
       </c>
       <c r="C17" t="s">
-        <v>864</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>869</v>
+        <v>868</v>
       </c>
       <c r="C18" t="s">
-        <v>864</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="C19" t="s">
-        <v>864</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>871</v>
+        <v>870</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>864</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>872</v>
+        <v>871</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>864</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>873</v>
+        <v>872</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>864</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>870</v>
+        <v>869</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>864</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>874</v>
+        <v>873</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>864</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
+        <v>874</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>1306</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
         <v>875</v>
       </c>
-      <c r="C25" s="5" t="s">
-        <v>864</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="5" t="s">
+      <c r="C26" s="7" t="s">
+        <v>1296</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="7" t="s">
         <v>876</v>
       </c>
-      <c r="C26" s="5" t="s">
-        <v>864</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="5" t="s">
+      <c r="C27" s="7" t="s">
+        <v>1297</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="7" t="s">
         <v>877</v>
       </c>
-      <c r="C27" s="5" t="s">
-        <v>864</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="5" t="s">
+      <c r="C28" s="7" t="s">
+        <v>1298</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="7" t="s">
         <v>878</v>
       </c>
-      <c r="C28" s="5" t="s">
-        <v>864</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
+      <c r="C29" s="7" t="s">
+        <v>1301</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
         <v>879</v>
       </c>
-      <c r="C29" s="5" t="s">
-        <v>864</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="5" t="s">
+      <c r="C30" s="7" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="7" t="s">
         <v>880</v>
       </c>
-      <c r="C30" s="5" t="s">
-        <v>864</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="5" t="s">
-        <v>881</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>864</v>
+      <c r="C31" s="7" t="s">
+        <v>1299</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="C32" t="s">
-        <v>864</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="C33" t="s">
-        <v>864</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="C34" t="s">
-        <v>864</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="C35" t="s">
-        <v>864</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="C36" t="s">
-        <v>864</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="C37" t="s">
-        <v>864</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>864</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>864</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>864</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>864</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>864</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>864</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="C44" t="s">
-        <v>864</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="C45" t="s">
-        <v>864</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="C46" t="s">
-        <v>864</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="C47" t="s">
-        <v>864</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="C48" t="s">
-        <v>864</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="C49" t="s">
-        <v>864</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="C50" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="C51" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="C58" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C59" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="C60" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="C61" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="C62" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="C63" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="C64" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="C65" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="C66" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="C67" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="C70" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="C71" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="C72" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="C73" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="C74" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="C75" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="C77" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>864</v>
+        <v>863</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>1249</v>
+        <v>1245</v>
       </c>
       <c r="C82" t="s">
-        <v>864</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>1250</v>
-      </c>
-      <c r="C83" t="s">
-        <v>864</v>
+        <v>1246</v>
+      </c>
+      <c r="C83" s="6" t="s">
+        <v>1279</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>1251</v>
-      </c>
-      <c r="C84" t="s">
-        <v>864</v>
+        <v>1247</v>
+      </c>
+      <c r="C84" s="6" t="s">
+        <v>1280</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>1252</v>
-      </c>
-      <c r="C85" t="s">
-        <v>864</v>
+        <v>1248</v>
+      </c>
+      <c r="C85" s="6" t="s">
+        <v>1281</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>1253</v>
-      </c>
-      <c r="C86" t="s">
-        <v>864</v>
+        <v>1249</v>
+      </c>
+      <c r="C86" s="6" t="s">
+        <v>1294</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>1254</v>
-      </c>
-      <c r="C87" t="s">
-        <v>864</v>
+        <v>1250</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>1282</v>
       </c>
     </row>
   </sheetData>
@@ -10430,194 +10582,194 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>758</v>
+      </c>
+      <c r="C2" t="s">
         <v>759</v>
-      </c>
-      <c r="C2" t="s">
-        <v>760</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="C3" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="C4" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>763</v>
+      </c>
+      <c r="C5" t="s">
         <v>764</v>
-      </c>
-      <c r="C5" t="s">
-        <v>765</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="C6" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="C7" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="C8" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="C9" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="C10" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>770</v>
+      </c>
+      <c r="C11" t="s">
         <v>771</v>
-      </c>
-      <c r="C11" t="s">
-        <v>772</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="C12" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="C13" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="C14" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="C15" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C16" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="C17" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="C18" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>786</v>
+      </c>
+      <c r="C19" t="s">
         <v>787</v>
-      </c>
-      <c r="C19" t="s">
-        <v>788</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="C20" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="C21" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C22" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="C23" t="s">
-        <v>944</v>
+        <v>943</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>1271</v>
+        <v>1267</v>
       </c>
       <c r="C24" t="s">
-        <v>1272</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>1273</v>
+        <v>1269</v>
       </c>
       <c r="C25" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
! Fix bug in battle scene and some bugs of localization.
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -3623,9 +3623,6 @@
     <t>ShaWujing_U_Name</t>
   </si>
   <si>
-    <t>ShaWujing_B_Des</t>
-  </si>
-  <si>
     <t>ShaWujing_M_Des</t>
   </si>
   <si>
@@ -4945,18 +4942,12 @@
     <t>Ma Vương Bạt Khí</t>
   </si>
   <si>
-    <t>Kĩ năng XBích Thủy Tinh Thú Kích</t>
-  </si>
-  <si>
     <t>Vung đại đao vung một nhát chém tựa dời núi lấp biển, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
   </si>
   <si>
     <t>Ngưu Ma Vương ngửa mặt gầm lên một tiếng làm chấn động càn khôn, bộc phát ma khí ngút trời giúp bản thân vào trạng thái [Bình Thiên], tăng {0}% Tấn Công</t>
   </si>
   <si>
-    <t>Triệu hồi Bích Thủy Kim Tinh Thú giáng lâm, phóng ra luồng sóng chấn động mang kịch độc oanh kích mục tiêu, gây ST bằng {0}% Tấn Công cho [một kẻ địch / toàn bộ kẻ địch], đồng thời khiến đối phương rơi vào trạng thái [Kịch Độc], mỗi hiệp chịu ST Độc bằng {1}% Tấn Công trong {2} hiệp.</t>
-  </si>
-  <si>
     <t>Cửu Xỉ Thần Bát</t>
   </si>
   <si>
@@ -5063,6 +5054,15 @@
   </si>
   <si>
     <t>Bứt một nhúm lông thổi nhẹ triệu hồi phân thân tham chiến, tấn công gây {0}% Tấn Công cho toàn bộ kẻ địch đồng thời phục hồi {1} % sát thương gây ra.</t>
+  </si>
+  <si>
+    <t>Bích Thủy Tinh Thú Kích</t>
+  </si>
+  <si>
+    <t>Triệu hồi Bích Thủy Kim Tinh Thú giáng lâm, phóng ra luồng sóng chấn động mang kịch độc oanh kích mục tiêu, gây ST bằng {0}% Tấn Công cho một kẻ địch, đồng thời khiến đối phương rơi vào trạng thái [Kịch Độc], mỗi hiệp chịu ST Độc bằng {1}% Tấn Công trong {2} hiệp.</t>
+  </si>
+  <si>
+    <t>ShaWujing_U_Des</t>
   </si>
 </sst>
 </file>
@@ -5564,10 +5564,10 @@
         <v>32</v>
       </c>
       <c r="B12" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -6034,7 +6034,7 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="B55" t="s">
         <v>576</v>
@@ -6059,10 +6059,10 @@
         <v>583</v>
       </c>
       <c r="B57" t="s">
+        <v>943</v>
+      </c>
+      <c r="C57" t="s">
         <v>944</v>
-      </c>
-      <c r="C57" t="s">
-        <v>945</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -6073,7 +6073,7 @@
         <v>585</v>
       </c>
       <c r="C58" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -6264,128 +6264,128 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="B77" t="s">
+        <v>947</v>
+      </c>
+      <c r="C77" t="s">
         <v>948</v>
-      </c>
-      <c r="C77" t="s">
-        <v>949</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>949</v>
+      </c>
+      <c r="B78" t="s">
         <v>950</v>
       </c>
-      <c r="B78" t="s">
+      <c r="C78" t="s">
         <v>951</v>
-      </c>
-      <c r="C78" t="s">
-        <v>952</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="B79" t="s">
+        <v>953</v>
+      </c>
+      <c r="C79" t="s">
         <v>954</v>
-      </c>
-      <c r="C79" t="s">
-        <v>955</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="B80" t="s">
+        <v>958</v>
+      </c>
+      <c r="C80" t="s">
         <v>959</v>
-      </c>
-      <c r="C80" t="s">
-        <v>960</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>958</v>
+        <v>957</v>
       </c>
       <c r="B81" t="s">
-        <v>962</v>
+        <v>961</v>
       </c>
       <c r="C81" t="s">
-        <v>961</v>
+        <v>960</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>966</v>
+        <v>965</v>
       </c>
       <c r="B82" t="s">
-        <v>969</v>
+        <v>968</v>
       </c>
       <c r="C82" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>966</v>
+      </c>
+      <c r="B83" t="s">
+        <v>964</v>
+      </c>
+      <c r="C83" t="s">
         <v>967</v>
-      </c>
-      <c r="B83" t="s">
-        <v>965</v>
-      </c>
-      <c r="C83" t="s">
-        <v>968</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="B84" t="s">
         <v>631</v>
       </c>
       <c r="C84" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>971</v>
+      </c>
+      <c r="B85" t="s">
         <v>972</v>
       </c>
-      <c r="B85" t="s">
+      <c r="C85" t="s">
         <v>973</v>
-      </c>
-      <c r="C85" t="s">
-        <v>974</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>975</v>
+      </c>
+      <c r="B86" t="s">
         <v>976</v>
       </c>
-      <c r="B86" t="s">
+      <c r="C86" t="s">
         <v>977</v>
-      </c>
-      <c r="C86" t="s">
-        <v>978</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="B87" t="s">
         <v>609</v>
       </c>
       <c r="C87" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="B88" t="s">
         <v>617</v>
@@ -6396,219 +6396,219 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>983</v>
+      </c>
+      <c r="B89" t="s">
         <v>984</v>
       </c>
-      <c r="B89" t="s">
+      <c r="C89" t="s">
         <v>985</v>
-      </c>
-      <c r="C89" t="s">
-        <v>986</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="B90" t="s">
         <v>445</v>
       </c>
       <c r="C90" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
+        <v>987</v>
+      </c>
+      <c r="B91" t="s">
         <v>988</v>
       </c>
-      <c r="B91" t="s">
-        <v>989</v>
-      </c>
       <c r="C91" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
+        <v>991</v>
+      </c>
+      <c r="B92" t="s">
         <v>992</v>
       </c>
-      <c r="B92" t="s">
+      <c r="C92" t="s">
         <v>993</v>
-      </c>
-      <c r="C92" t="s">
-        <v>994</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="B93" t="s">
+        <v>1004</v>
+      </c>
+      <c r="C93" t="s">
         <v>1005</v>
-      </c>
-      <c r="C93" t="s">
-        <v>1006</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
+        <v>1007</v>
+      </c>
+      <c r="B94" t="s">
         <v>1008</v>
       </c>
-      <c r="B94" t="s">
+      <c r="C94" t="s">
         <v>1009</v>
-      </c>
-      <c r="C94" t="s">
-        <v>1010</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B95" t="s">
         <v>1017</v>
       </c>
-      <c r="B95" t="s">
+      <c r="C95" t="s">
         <v>1018</v>
-      </c>
-      <c r="C95" t="s">
-        <v>1019</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
+        <v>1019</v>
+      </c>
+      <c r="B96" t="s">
         <v>1020</v>
       </c>
-      <c r="B96" t="s">
+      <c r="C96" t="s">
         <v>1021</v>
-      </c>
-      <c r="C96" t="s">
-        <v>1022</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
+        <v>1022</v>
+      </c>
+      <c r="B97" t="s">
         <v>1023</v>
       </c>
-      <c r="B97" t="s">
+      <c r="C97" t="s">
         <v>1024</v>
-      </c>
-      <c r="C97" t="s">
-        <v>1025</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B98" t="s">
         <v>1026</v>
       </c>
-      <c r="B98" t="s">
+      <c r="C98" t="s">
         <v>1027</v>
-      </c>
-      <c r="C98" t="s">
-        <v>1028</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B99" t="s">
         <v>1029</v>
       </c>
-      <c r="B99" t="s">
-        <v>1030</v>
-      </c>
       <c r="C99" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B100" t="s">
         <v>1031</v>
       </c>
-      <c r="B100" t="s">
-        <v>1032</v>
-      </c>
       <c r="C100" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B101" t="s">
         <v>1033</v>
       </c>
-      <c r="B101" t="s">
-        <v>1034</v>
-      </c>
       <c r="C101" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
+        <v>1034</v>
+      </c>
+      <c r="B102" t="s">
         <v>1035</v>
       </c>
-      <c r="B102" t="s">
+      <c r="C102" t="s">
         <v>1036</v>
-      </c>
-      <c r="C102" t="s">
-        <v>1037</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
+        <v>1039</v>
+      </c>
+      <c r="B103" t="s">
         <v>1040</v>
       </c>
-      <c r="B103" t="s">
+      <c r="C103" t="s">
         <v>1041</v>
-      </c>
-      <c r="C103" t="s">
-        <v>1042</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
+        <v>1042</v>
+      </c>
+      <c r="B104" t="s">
         <v>1043</v>
       </c>
-      <c r="B104" t="s">
+      <c r="C104" t="s">
         <v>1044</v>
-      </c>
-      <c r="C104" t="s">
-        <v>1045</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
+        <v>1045</v>
+      </c>
+      <c r="B105" t="s">
         <v>1046</v>
       </c>
-      <c r="B105" t="s">
+      <c r="C105" t="s">
         <v>1047</v>
-      </c>
-      <c r="C105" t="s">
-        <v>1048</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
+        <v>1048</v>
+      </c>
+      <c r="B106" t="s">
         <v>1049</v>
       </c>
-      <c r="B106" t="s">
+      <c r="C106" t="s">
         <v>1050</v>
-      </c>
-      <c r="C106" t="s">
-        <v>1051</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
+        <v>1051</v>
+      </c>
+      <c r="B107" t="s">
         <v>1052</v>
       </c>
-      <c r="B107" t="s">
+      <c r="C107" t="s">
         <v>1053</v>
-      </c>
-      <c r="C107" t="s">
-        <v>1054</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
+        <v>1054</v>
+      </c>
+      <c r="B108" t="s">
         <v>1055</v>
-      </c>
-      <c r="B108" t="s">
-        <v>1056</v>
       </c>
       <c r="C108" t="s">
         <v>43</v>
@@ -6616,123 +6616,123 @@
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
+        <v>1092</v>
+      </c>
+      <c r="B109" t="s">
         <v>1093</v>
       </c>
-      <c r="B109" t="s">
-        <v>1094</v>
-      </c>
       <c r="C109" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
+        <v>1094</v>
+      </c>
+      <c r="B110" t="s">
         <v>1095</v>
       </c>
-      <c r="B110" t="s">
+      <c r="C110" t="s">
         <v>1096</v>
-      </c>
-      <c r="C110" t="s">
-        <v>1097</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
+        <v>1097</v>
+      </c>
+      <c r="B111" t="s">
         <v>1098</v>
       </c>
-      <c r="B111" t="s">
+      <c r="C111" t="s">
         <v>1099</v>
-      </c>
-      <c r="C111" t="s">
-        <v>1100</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
+        <v>1100</v>
+      </c>
+      <c r="B112" t="s">
         <v>1101</v>
       </c>
-      <c r="B112" t="s">
+      <c r="C112" t="s">
         <v>1102</v>
-      </c>
-      <c r="C112" t="s">
-        <v>1103</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="B113" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="C113" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
+        <v>1197</v>
+      </c>
+      <c r="B114" t="s">
         <v>1198</v>
       </c>
-      <c r="B114" t="s">
+      <c r="C114" t="s">
         <v>1199</v>
-      </c>
-      <c r="C114" t="s">
-        <v>1200</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
+        <v>1200</v>
+      </c>
+      <c r="B115" t="s">
+        <v>1202</v>
+      </c>
+      <c r="C115" t="s">
         <v>1201</v>
-      </c>
-      <c r="B115" t="s">
-        <v>1203</v>
-      </c>
-      <c r="C115" t="s">
-        <v>1202</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
+        <v>1203</v>
+      </c>
+      <c r="B116" t="s">
         <v>1204</v>
       </c>
-      <c r="B116" t="s">
+      <c r="C116" t="s">
         <v>1205</v>
-      </c>
-      <c r="C116" t="s">
-        <v>1206</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
+        <v>1206</v>
+      </c>
+      <c r="B117" t="s">
         <v>1207</v>
       </c>
-      <c r="B117" t="s">
+      <c r="C117" t="s">
         <v>1208</v>
-      </c>
-      <c r="C117" t="s">
-        <v>1209</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
+        <v>1209</v>
+      </c>
+      <c r="B118" t="s">
         <v>1210</v>
       </c>
-      <c r="B118" t="s">
+      <c r="C118" t="s">
         <v>1211</v>
-      </c>
-      <c r="C118" t="s">
-        <v>1212</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
+        <v>1253</v>
+      </c>
+      <c r="B119" t="s">
         <v>1254</v>
       </c>
-      <c r="B119" t="s">
+      <c r="C119" t="s">
         <v>1255</v>
-      </c>
-      <c r="C119" t="s">
-        <v>1256</v>
       </c>
     </row>
   </sheetData>
@@ -7404,7 +7404,7 @@
         <v>133</v>
       </c>
       <c r="C21" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -7602,7 +7602,7 @@
         <v>176</v>
       </c>
       <c r="C39" t="s">
-        <v>956</v>
+        <v>955</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -7833,7 +7833,7 @@
         <v>262</v>
       </c>
       <c r="C60" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -7899,7 +7899,7 @@
         <v>260</v>
       </c>
       <c r="C66" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
@@ -8614,7 +8614,7 @@
         <v>466</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>1307</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
@@ -9049,29 +9049,29 @@
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
+        <v>1256</v>
+      </c>
+      <c r="B173" t="s">
         <v>1257</v>
       </c>
-      <c r="B173" t="s">
+      <c r="C173" t="s">
         <v>1258</v>
-      </c>
-      <c r="C173" t="s">
-        <v>1259</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>1261</v>
+        <v>1260</v>
       </c>
       <c r="B174" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
       <c r="C174" t="s">
-        <v>1260</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="B175" t="s">
         <v>78</v>
@@ -9132,7 +9132,7 @@
         <v>834</v>
       </c>
       <c r="C180" t="s">
-        <v>931</v>
+        <v>930</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
@@ -9170,673 +9170,673 @@
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
+        <v>994</v>
+      </c>
+      <c r="B184" t="s">
         <v>995</v>
       </c>
-      <c r="B184" t="s">
+      <c r="C184" t="s">
         <v>996</v>
-      </c>
-      <c r="C184" t="s">
-        <v>997</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="B185" t="s">
+        <v>999</v>
+      </c>
+      <c r="C185" t="s">
         <v>1000</v>
-      </c>
-      <c r="C185" t="s">
-        <v>1001</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="B186" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="C186" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B187" t="s">
         <v>1004</v>
       </c>
-      <c r="B187" t="s">
+      <c r="C187" t="s">
         <v>1005</v>
-      </c>
-      <c r="C187" t="s">
-        <v>1006</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="B188" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="C188" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="B189" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="C189" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="B190" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="C190" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="B191" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="C191" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="B192" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="C192" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="B193" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="C193" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="B194" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="C194" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="B195" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="C195" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="B196" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="C196" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="B197" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="C197" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="B198" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="C198" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="B199" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="C199" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="B200" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="C200" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="B201" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="C201" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B202" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C202" t="s">
         <v>1104</v>
-      </c>
-      <c r="B202" t="s">
-        <v>1106</v>
-      </c>
-      <c r="C202" t="s">
-        <v>1105</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
+        <v>1106</v>
+      </c>
+      <c r="B203" t="s">
+        <v>1110</v>
+      </c>
+      <c r="C203" t="s">
         <v>1107</v>
-      </c>
-      <c r="B203" t="s">
-        <v>1111</v>
-      </c>
-      <c r="C203" t="s">
-        <v>1108</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="B204" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="C204" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
+        <v>1112</v>
+      </c>
+      <c r="B205" t="s">
+        <v>1114</v>
+      </c>
+      <c r="C205" t="s">
         <v>1113</v>
-      </c>
-      <c r="B205" t="s">
-        <v>1115</v>
-      </c>
-      <c r="C205" t="s">
-        <v>1114</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B206" t="s">
         <v>1116</v>
       </c>
-      <c r="B206" t="s">
+      <c r="C206" t="s">
         <v>1117</v>
-      </c>
-      <c r="C206" t="s">
-        <v>1118</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
+        <v>1118</v>
+      </c>
+      <c r="B207" t="s">
         <v>1119</v>
       </c>
-      <c r="B207" t="s">
+      <c r="C207" t="s">
         <v>1120</v>
-      </c>
-      <c r="C207" t="s">
-        <v>1121</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
+        <v>1124</v>
+      </c>
+      <c r="B208" t="s">
         <v>1125</v>
       </c>
-      <c r="B208" t="s">
+      <c r="C208" t="s">
         <v>1126</v>
-      </c>
-      <c r="C208" t="s">
-        <v>1127</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B209" t="s">
+        <v>1129</v>
+      </c>
+      <c r="C209" t="s">
         <v>1128</v>
-      </c>
-      <c r="B209" t="s">
-        <v>1130</v>
-      </c>
-      <c r="C209" t="s">
-        <v>1129</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B210" t="s">
+        <v>1132</v>
+      </c>
+      <c r="C210" t="s">
         <v>1131</v>
-      </c>
-      <c r="B210" t="s">
-        <v>1133</v>
-      </c>
-      <c r="C210" t="s">
-        <v>1132</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="B211" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="C211" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
+        <v>1135</v>
+      </c>
+      <c r="B212" t="s">
         <v>1136</v>
       </c>
-      <c r="B212" t="s">
-        <v>1137</v>
-      </c>
       <c r="C212" t="s">
-        <v>1213</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
+        <v>1137</v>
+      </c>
+      <c r="B213" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C213" t="s">
         <v>1138</v>
-      </c>
-      <c r="B213" t="s">
-        <v>1140</v>
-      </c>
-      <c r="C213" t="s">
-        <v>1139</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="B214" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="C214" t="s">
-        <v>1214</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
+        <v>1143</v>
+      </c>
+      <c r="B215" t="s">
         <v>1144</v>
       </c>
-      <c r="B215" t="s">
-        <v>1145</v>
-      </c>
       <c r="C215" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
+        <v>1145</v>
+      </c>
+      <c r="B216" t="s">
+        <v>1147</v>
+      </c>
+      <c r="C216" t="s">
         <v>1146</v>
-      </c>
-      <c r="B216" t="s">
-        <v>1148</v>
-      </c>
-      <c r="C216" t="s">
-        <v>1147</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
+        <v>1149</v>
+      </c>
+      <c r="B217" t="s">
+        <v>1151</v>
+      </c>
+      <c r="C217" t="s">
         <v>1150</v>
-      </c>
-      <c r="B217" t="s">
-        <v>1152</v>
-      </c>
-      <c r="C217" t="s">
-        <v>1151</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
+        <v>1152</v>
+      </c>
+      <c r="B218" t="s">
+        <v>1154</v>
+      </c>
+      <c r="C218" t="s">
         <v>1153</v>
-      </c>
-      <c r="B218" t="s">
-        <v>1155</v>
-      </c>
-      <c r="C218" t="s">
-        <v>1154</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
+        <v>1155</v>
+      </c>
+      <c r="B219" t="s">
+        <v>1157</v>
+      </c>
+      <c r="C219" t="s">
         <v>1156</v>
-      </c>
-      <c r="B219" t="s">
-        <v>1158</v>
-      </c>
-      <c r="C219" t="s">
-        <v>1157</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="B220" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
       <c r="C220" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="B221" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="C221" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
       <c r="B222" t="s">
+        <v>1165</v>
+      </c>
+      <c r="C222" t="s">
         <v>1166</v>
-      </c>
-      <c r="C222" t="s">
-        <v>1167</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="B223" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="C223" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="B224" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="C224" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="B225" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="C225" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="B226" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="C226" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="B227" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="C227" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="B228" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="C228" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="B229" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C229" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="B230" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="C230" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="B231" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="C231" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
+        <v>1214</v>
+      </c>
+      <c r="B232" t="s">
+        <v>1216</v>
+      </c>
+      <c r="C232" t="s">
         <v>1215</v>
-      </c>
-      <c r="B232" t="s">
-        <v>1217</v>
-      </c>
-      <c r="C232" t="s">
-        <v>1216</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
+        <v>1217</v>
+      </c>
+      <c r="B233" t="s">
         <v>1218</v>
       </c>
-      <c r="B233" t="s">
+      <c r="C233" t="s">
         <v>1219</v>
-      </c>
-      <c r="C233" t="s">
-        <v>1220</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
+        <v>1220</v>
+      </c>
+      <c r="B234" t="s">
         <v>1221</v>
       </c>
-      <c r="B234" t="s">
+      <c r="C234" t="s">
         <v>1222</v>
-      </c>
-      <c r="C234" t="s">
-        <v>1223</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
+        <v>1223</v>
+      </c>
+      <c r="B235" t="s">
         <v>1224</v>
       </c>
-      <c r="B235" t="s">
+      <c r="C235" t="s">
         <v>1225</v>
-      </c>
-      <c r="C235" t="s">
-        <v>1226</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
+        <v>1226</v>
+      </c>
+      <c r="B236" t="s">
         <v>1227</v>
       </c>
-      <c r="B236" t="s">
+      <c r="C236" t="s">
         <v>1228</v>
-      </c>
-      <c r="C236" t="s">
-        <v>1229</v>
       </c>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
+        <v>1232</v>
+      </c>
+      <c r="B237" t="s">
         <v>1233</v>
       </c>
-      <c r="B237" t="s">
+      <c r="C237" t="s">
         <v>1234</v>
-      </c>
-      <c r="C237" t="s">
-        <v>1235</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
+        <v>1229</v>
+      </c>
+      <c r="B238" t="s">
         <v>1230</v>
       </c>
-      <c r="B238" t="s">
+      <c r="C238" t="s">
         <v>1231</v>
-      </c>
-      <c r="C238" t="s">
-        <v>1232</v>
       </c>
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
+        <v>1235</v>
+      </c>
+      <c r="B239" t="s">
         <v>1236</v>
       </c>
-      <c r="B239" t="s">
+      <c r="C239" t="s">
         <v>1237</v>
-      </c>
-      <c r="C239" t="s">
-        <v>1238</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="B240" t="s">
+        <v>1238</v>
+      </c>
+      <c r="C240" t="s">
         <v>1239</v>
-      </c>
-      <c r="C240" t="s">
-        <v>1240</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
+        <v>1241</v>
+      </c>
+      <c r="B241" t="s">
         <v>1242</v>
       </c>
-      <c r="B241" t="s">
+      <c r="C241" t="s">
         <v>1243</v>
-      </c>
-      <c r="C241" t="s">
-        <v>1244</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
+        <v>1250</v>
+      </c>
+      <c r="B242" t="s">
         <v>1251</v>
       </c>
-      <c r="B242" t="s">
+      <c r="C242" t="s">
         <v>1252</v>
-      </c>
-      <c r="C242" t="s">
-        <v>1253</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
+        <v>1263</v>
+      </c>
+      <c r="B243" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C243" t="s">
         <v>1264</v>
-      </c>
-      <c r="B243" t="s">
-        <v>1266</v>
-      </c>
-      <c r="C243" t="s">
-        <v>1265</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
+        <v>1269</v>
+      </c>
+      <c r="B244" t="s">
         <v>1270</v>
       </c>
-      <c r="B244" t="s">
+      <c r="C244" t="s">
         <v>1271</v>
-      </c>
-      <c r="C244" t="s">
-        <v>1272</v>
       </c>
     </row>
   </sheetData>
@@ -9880,7 +9880,7 @@
         <v>854</v>
       </c>
       <c r="C3" t="s">
-        <v>1322</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -9896,7 +9896,7 @@
         <v>855</v>
       </c>
       <c r="C5" t="s">
-        <v>1324</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -9912,7 +9912,7 @@
         <v>856</v>
       </c>
       <c r="C7" t="s">
-        <v>1323</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -9920,7 +9920,7 @@
         <v>857</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>1308</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -9928,7 +9928,7 @@
         <v>858</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>1309</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -9936,7 +9936,7 @@
         <v>859</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>1310</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -9944,7 +9944,7 @@
         <v>860</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>1311</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -9952,7 +9952,7 @@
         <v>861</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>1312</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -9960,7 +9960,7 @@
         <v>862</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>1313</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -9968,7 +9968,7 @@
         <v>864</v>
       </c>
       <c r="C14" t="s">
-        <v>1289</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -9976,7 +9976,7 @@
         <v>865</v>
       </c>
       <c r="C15" t="s">
-        <v>1290</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -9984,7 +9984,7 @@
         <v>866</v>
       </c>
       <c r="C16" t="s">
-        <v>1291</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -9992,7 +9992,7 @@
         <v>867</v>
       </c>
       <c r="C17" t="s">
-        <v>1292</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -10000,7 +10000,7 @@
         <v>868</v>
       </c>
       <c r="C18" t="s">
-        <v>1293</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -10008,7 +10008,7 @@
         <v>869</v>
       </c>
       <c r="C19" t="s">
-        <v>1295</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -10016,7 +10016,7 @@
         <v>870</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>1302</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -10024,7 +10024,7 @@
         <v>871</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>1303</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -10032,15 +10032,15 @@
         <v>872</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>1304</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>1305</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -10048,212 +10048,212 @@
         <v>873</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>1321</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>874</v>
+        <v>1324</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>1306</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
-        <v>875</v>
+        <v>874</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>1296</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>876</v>
+        <v>875</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>1297</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>1298</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>878</v>
+        <v>877</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>1301</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
-        <v>879</v>
+        <v>878</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>1300</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>880</v>
+        <v>879</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>1299</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>881</v>
+        <v>880</v>
       </c>
       <c r="C32" t="s">
-        <v>1314</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="C33" t="s">
-        <v>1315</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>883</v>
+        <v>882</v>
       </c>
       <c r="C34" t="s">
-        <v>1316</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>884</v>
+        <v>883</v>
       </c>
       <c r="C35" t="s">
-        <v>1317</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>885</v>
+        <v>884</v>
       </c>
       <c r="C36" t="s">
-        <v>1318</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="C37" t="s">
-        <v>1319</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>1285</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>1286</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>891</v>
+        <v>890</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>1288</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="C44" t="s">
-        <v>1275</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="C45" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>895</v>
+        <v>894</v>
       </c>
       <c r="C46" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>896</v>
+        <v>895</v>
       </c>
       <c r="C47" t="s">
-        <v>1320</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>897</v>
+        <v>896</v>
       </c>
       <c r="C48" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>898</v>
+        <v>897</v>
       </c>
       <c r="C49" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="C50" t="s">
         <v>863</v>
@@ -10261,7 +10261,7 @@
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>900</v>
+        <v>899</v>
       </c>
       <c r="C51" t="s">
         <v>863</v>
@@ -10269,7 +10269,7 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>901</v>
+        <v>900</v>
       </c>
       <c r="C52" s="5" t="s">
         <v>863</v>
@@ -10277,7 +10277,7 @@
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>902</v>
+        <v>901</v>
       </c>
       <c r="C53" s="5" t="s">
         <v>863</v>
@@ -10285,7 +10285,7 @@
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="C54" s="5" t="s">
         <v>863</v>
@@ -10293,7 +10293,7 @@
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="C55" s="5" t="s">
         <v>863</v>
@@ -10301,7 +10301,7 @@
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="C56" s="5" t="s">
         <v>863</v>
@@ -10309,7 +10309,7 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="C57" s="5" t="s">
         <v>863</v>
@@ -10317,7 +10317,7 @@
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>907</v>
+        <v>906</v>
       </c>
       <c r="C58" t="s">
         <v>863</v>
@@ -10325,7 +10325,7 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>908</v>
+        <v>907</v>
       </c>
       <c r="C59" t="s">
         <v>863</v>
@@ -10333,7 +10333,7 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="C60" t="s">
         <v>863</v>
@@ -10341,7 +10341,7 @@
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="C61" t="s">
         <v>863</v>
@@ -10349,7 +10349,7 @@
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="C62" t="s">
         <v>863</v>
@@ -10357,7 +10357,7 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="C63" t="s">
         <v>863</v>
@@ -10365,7 +10365,7 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="C64" s="5" t="s">
         <v>863</v>
@@ -10373,7 +10373,7 @@
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="C65" s="5" t="s">
         <v>863</v>
@@ -10381,7 +10381,7 @@
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="C66" s="5" t="s">
         <v>863</v>
@@ -10389,7 +10389,7 @@
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>916</v>
+        <v>915</v>
       </c>
       <c r="C67" s="5" t="s">
         <v>863</v>
@@ -10397,7 +10397,7 @@
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>917</v>
+        <v>916</v>
       </c>
       <c r="C68" s="5" t="s">
         <v>863</v>
@@ -10405,7 +10405,7 @@
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="C69" s="5" t="s">
         <v>863</v>
@@ -10413,7 +10413,7 @@
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="C70" t="s">
         <v>863</v>
@@ -10421,7 +10421,7 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="C71" t="s">
         <v>863</v>
@@ -10429,7 +10429,7 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>921</v>
+        <v>920</v>
       </c>
       <c r="C72" t="s">
         <v>863</v>
@@ -10437,7 +10437,7 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="C73" t="s">
         <v>863</v>
@@ -10445,7 +10445,7 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="C74" t="s">
         <v>863</v>
@@ -10453,7 +10453,7 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>924</v>
+        <v>923</v>
       </c>
       <c r="C75" t="s">
         <v>863</v>
@@ -10461,7 +10461,7 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="C76" s="5" t="s">
         <v>863</v>
@@ -10469,7 +10469,7 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="C77" s="5" t="s">
         <v>863</v>
@@ -10477,7 +10477,7 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
-        <v>927</v>
+        <v>926</v>
       </c>
       <c r="C78" s="5" t="s">
         <v>863</v>
@@ -10485,7 +10485,7 @@
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
-        <v>928</v>
+        <v>927</v>
       </c>
       <c r="C79" s="5" t="s">
         <v>863</v>
@@ -10493,7 +10493,7 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="C80" s="5" t="s">
         <v>863</v>
@@ -10501,7 +10501,7 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
-        <v>930</v>
+        <v>929</v>
       </c>
       <c r="C81" s="5" t="s">
         <v>863</v>
@@ -10509,50 +10509,50 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
       <c r="C82" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>1294</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>1250</v>
+        <v>1249</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
     </row>
   </sheetData>
@@ -10630,18 +10630,18 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>933</v>
+        <v>932</v>
       </c>
       <c r="C8" t="s">
-        <v>935</v>
+        <v>934</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="C9" t="s">
-        <v>936</v>
+        <v>935</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -10726,47 +10726,47 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>938</v>
+        <v>937</v>
       </c>
       <c r="C20" t="s">
-        <v>934</v>
+        <v>933</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>939</v>
+        <v>938</v>
       </c>
       <c r="C21" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>940</v>
+        <v>939</v>
       </c>
       <c r="C22" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>941</v>
+        <v>940</v>
       </c>
       <c r="C23" t="s">
-        <v>943</v>
+        <v>942</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>1266</v>
+      </c>
+      <c r="C24" t="s">
         <v>1267</v>
-      </c>
-      <c r="C24" t="s">
-        <v>1268</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>1269</v>
+        <v>1268</v>
       </c>
       <c r="C25" t="s">
         <v>787</v>

</xml_diff>

<commit_message>
+ Clean code and add a new loading screen background.
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="UI" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1475" uniqueCount="1391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1475" uniqueCount="1392">
   <si>
     <t>ID</t>
   </si>
@@ -4921,9 +4921,6 @@
     <t>Bảo Tháp Hộ Thể</t>
   </si>
   <si>
-    <t>rấn Ma Bảo Tháp</t>
-  </si>
-  <si>
     <t>Tuốt kiếm chém nhanh một đòn dứt khoát, gây ST bằng {0}% Tấn Công cho một kẻ địch.</t>
   </si>
   <si>
@@ -5357,6 +5354,12 @@
   </si>
   <si>
     <t>Động Liên Hoa - Thu Phục Ngân Giác, Kim Giác</t>
+  </si>
+  <si>
+    <t>Trấn Ma Bảo Tháp</t>
+  </si>
+  <si>
+    <t>ShaWujing_B_Des</t>
   </si>
 </sst>
 </file>
@@ -7040,57 +7043,57 @@
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
+        <v>1322</v>
+      </c>
+      <c r="B120" t="s">
         <v>1323</v>
       </c>
-      <c r="B120" t="s">
+      <c r="C120" t="s">
         <v>1324</v>
-      </c>
-      <c r="C120" t="s">
-        <v>1325</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B121" t="s">
         <v>1326</v>
       </c>
-      <c r="B121" t="s">
+      <c r="C121" t="s">
         <v>1327</v>
-      </c>
-      <c r="C121" t="s">
-        <v>1328</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
+        <v>1328</v>
+      </c>
+      <c r="B122" t="s">
         <v>1329</v>
       </c>
-      <c r="B122" t="s">
+      <c r="C122" t="s">
         <v>1330</v>
-      </c>
-      <c r="C122" t="s">
-        <v>1331</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B123" t="s">
+        <v>1331</v>
+      </c>
+      <c r="C123" t="s">
         <v>1332</v>
-      </c>
-      <c r="C123" t="s">
-        <v>1333</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
+        <v>1334</v>
+      </c>
+      <c r="B124" t="s">
         <v>1335</v>
       </c>
-      <c r="B124" t="s">
+      <c r="C124" t="s">
         <v>1336</v>
-      </c>
-      <c r="C124" t="s">
-        <v>1337</v>
       </c>
     </row>
   </sheetData>
@@ -8972,7 +8975,7 @@
         <v>466</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
@@ -9509,10 +9512,10 @@
         <v>839</v>
       </c>
       <c r="B182" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="C182" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
@@ -10199,189 +10202,189 @@
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
+        <v>1339</v>
+      </c>
+      <c r="B245" t="s">
+        <v>1341</v>
+      </c>
+      <c r="C245" t="s">
         <v>1340</v>
-      </c>
-      <c r="B245" t="s">
-        <v>1342</v>
-      </c>
-      <c r="C245" t="s">
-        <v>1341</v>
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>1343</v>
+        <v>1342</v>
       </c>
       <c r="B246" t="s">
-        <v>1346</v>
+        <v>1345</v>
       </c>
       <c r="C246" t="s">
-        <v>1349</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
+        <v>1343</v>
+      </c>
+      <c r="B247" t="s">
+        <v>1346</v>
+      </c>
+      <c r="C247" t="s">
         <v>1344</v>
-      </c>
-      <c r="B247" t="s">
-        <v>1347</v>
-      </c>
-      <c r="C247" t="s">
-        <v>1345</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>1348</v>
+        <v>1347</v>
       </c>
       <c r="B248" t="s">
-        <v>1353</v>
+        <v>1352</v>
       </c>
       <c r="C248" t="s">
-        <v>1350</v>
+        <v>1349</v>
       </c>
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
+        <v>1350</v>
+      </c>
+      <c r="B249" t="s">
+        <v>1353</v>
+      </c>
+      <c r="C249" t="s">
         <v>1351</v>
-      </c>
-      <c r="B249" t="s">
-        <v>1354</v>
-      </c>
-      <c r="C249" t="s">
-        <v>1352</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
+        <v>1354</v>
+      </c>
+      <c r="B250" t="s">
+        <v>1357</v>
+      </c>
+      <c r="C250" t="s">
         <v>1355</v>
-      </c>
-      <c r="B250" t="s">
-        <v>1358</v>
-      </c>
-      <c r="C250" t="s">
-        <v>1356</v>
       </c>
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>1360</v>
+        <v>1359</v>
       </c>
       <c r="B251" t="s">
-        <v>1359</v>
+        <v>1358</v>
       </c>
       <c r="C251" t="s">
-        <v>1357</v>
+        <v>1356</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>1361</v>
+        <v>1360</v>
       </c>
       <c r="B252" t="s">
-        <v>1365</v>
+        <v>1364</v>
       </c>
       <c r="C252" t="s">
-        <v>1363</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>1362</v>
+        <v>1361</v>
       </c>
       <c r="B253" t="s">
-        <v>1366</v>
+        <v>1365</v>
       </c>
       <c r="C253" t="s">
-        <v>1364</v>
+        <v>1363</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>1367</v>
+        <v>1366</v>
       </c>
       <c r="B254" t="s">
-        <v>1371</v>
+        <v>1370</v>
       </c>
       <c r="C254" t="s">
-        <v>1369</v>
+        <v>1368</v>
       </c>
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>1368</v>
+        <v>1367</v>
       </c>
       <c r="B255" t="s">
-        <v>1372</v>
+        <v>1371</v>
       </c>
       <c r="C255" t="s">
-        <v>1370</v>
+        <v>1369</v>
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>1373</v>
+        <v>1372</v>
       </c>
       <c r="B256" t="s">
-        <v>1375</v>
+        <v>1374</v>
       </c>
       <c r="C256" t="s">
-        <v>1390</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
+        <v>1375</v>
+      </c>
+      <c r="B257" t="s">
         <v>1376</v>
       </c>
-      <c r="B257" t="s">
-        <v>1377</v>
-      </c>
       <c r="C257" t="s">
-        <v>1374</v>
+        <v>1373</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>1378</v>
+        <v>1377</v>
       </c>
       <c r="B258" t="s">
-        <v>1382</v>
+        <v>1381</v>
       </c>
       <c r="C258" t="s">
-        <v>1380</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>1379</v>
+        <v>1378</v>
       </c>
       <c r="B259" t="s">
-        <v>1383</v>
+        <v>1382</v>
       </c>
       <c r="C259" t="s">
-        <v>1381</v>
+        <v>1380</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>1384</v>
+        <v>1383</v>
       </c>
       <c r="B260" t="s">
-        <v>1388</v>
+        <v>1387</v>
       </c>
       <c r="C260" t="s">
-        <v>1387</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
+        <v>1384</v>
+      </c>
+      <c r="B261" t="s">
+        <v>1388</v>
+      </c>
+      <c r="C261" s="8" t="s">
         <v>1385</v>
-      </c>
-      <c r="B261" t="s">
-        <v>1389</v>
-      </c>
-      <c r="C261" s="8" t="s">
-        <v>1386</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.25">
@@ -10428,7 +10431,7 @@
         <v>852</v>
       </c>
       <c r="C3" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -10444,7 +10447,7 @@
         <v>853</v>
       </c>
       <c r="C5" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -10460,7 +10463,7 @@
         <v>854</v>
       </c>
       <c r="C7" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -10468,7 +10471,7 @@
         <v>855</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -10476,7 +10479,7 @@
         <v>856</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -10484,7 +10487,7 @@
         <v>857</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -10492,7 +10495,7 @@
         <v>858</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -10500,7 +10503,7 @@
         <v>859</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -10508,7 +10511,7 @@
         <v>860</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -10516,7 +10519,7 @@
         <v>862</v>
       </c>
       <c r="C14" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -10524,7 +10527,7 @@
         <v>863</v>
       </c>
       <c r="C15" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -10532,7 +10535,7 @@
         <v>864</v>
       </c>
       <c r="C16" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -10540,7 +10543,7 @@
         <v>865</v>
       </c>
       <c r="C17" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -10548,7 +10551,7 @@
         <v>866</v>
       </c>
       <c r="C18" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -10556,7 +10559,7 @@
         <v>867</v>
       </c>
       <c r="C19" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -10564,7 +10567,7 @@
         <v>868</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -10572,7 +10575,7 @@
         <v>869</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -10580,15 +10583,15 @@
         <v>870</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>865</v>
+        <v>1391</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -10596,15 +10599,15 @@
         <v>871</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -10612,7 +10615,7 @@
         <v>872</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -10620,7 +10623,7 @@
         <v>873</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -10628,7 +10631,7 @@
         <v>874</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -10636,7 +10639,7 @@
         <v>875</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -10644,7 +10647,7 @@
         <v>876</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -10652,7 +10655,7 @@
         <v>877</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -10660,7 +10663,7 @@
         <v>878</v>
       </c>
       <c r="C32" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -10668,7 +10671,7 @@
         <v>879</v>
       </c>
       <c r="C33" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -10676,7 +10679,7 @@
         <v>880</v>
       </c>
       <c r="C34" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -10684,7 +10687,7 @@
         <v>881</v>
       </c>
       <c r="C35" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -10692,7 +10695,7 @@
         <v>882</v>
       </c>
       <c r="C36" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -10700,7 +10703,7 @@
         <v>883</v>
       </c>
       <c r="C37" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -10708,7 +10711,7 @@
         <v>884</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -10716,7 +10719,7 @@
         <v>885</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -10724,7 +10727,7 @@
         <v>886</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -10732,7 +10735,7 @@
         <v>887</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -10740,7 +10743,7 @@
         <v>888</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -10748,7 +10751,7 @@
         <v>889</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -10780,7 +10783,7 @@
         <v>893</v>
       </c>
       <c r="C47" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -11076,7 +11079,7 @@
         <v>1244</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>1277</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
@@ -11084,7 +11087,7 @@
         <v>1245</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
@@ -11092,7 +11095,7 @@
         <v>1246</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
@@ -11100,7 +11103,7 @@
         <v>1247</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Add Default Dialogue for all NPC in the map.
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1497" uniqueCount="1413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1908" uniqueCount="1821">
   <si>
     <t>ID</t>
   </si>
@@ -4819,9 +4819,6 @@
     <t>Marshal Tianpeng</t>
   </si>
   <si>
-    <t>Thiên Bồng Nguyên Soái</t>
-  </si>
-  <si>
     <t>UI_GAO_FAMILY_VILLAGE</t>
   </si>
   <si>
@@ -5419,10 +5416,1260 @@
     <t>STR_DLG_Dragon_king_Eatern_Sea_Default_Choice_Ask</t>
   </si>
   <si>
-    <t>Ta chỉ tiền đường qua đây thôi.</t>
-  </si>
-  <si>
-    <t>Việc của nhà lão tao không muốn can dự.</t>
+    <t>STR_DLG_Dragon_king_Eatern_Sea_Default_Choice_Ask_Weathrer</t>
+  </si>
+  <si>
+    <t>Hỏi về thời tiết ở Hoa Quả Sơn</t>
+  </si>
+  <si>
+    <t>STR_DLG_Dragon_king_Eatern_Sea_Default_Node_Ask_Weather</t>
+  </si>
+  <si>
+    <t>Này lão Long Vương! Dạo này Hoa Quả Sơn của ta nắng mưa thất thường, ngài cai quản thời tiết kiểu gì thế?</t>
+  </si>
+  <si>
+    <t>STR_DLG_Dragon_king_Eatern_Sea_Default_Node_Answer_Weather</t>
+  </si>
+  <si>
+    <t>STR_DLG_Dragon_king_Eatern_Sea_Default_Node_Ask_Weather_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Dragon_king_Eatern_Sea_Default_Node_Answer_Weather_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Dragon_king_Eatern_Sea_Default_Node_Ask_Weather_02</t>
+  </si>
+  <si>
+    <t>Đại Thánh bớt giận, thời tiết Hoa Quả Sơn ngày mai  Sáng sớm có sương mù nhẹ vài nơi, trưa chiều giảm mây trời nắng. | Thời tiết mát mẻ, tạnh ráo, rất thuật lợi cho các hoạt động ngoài trời.</t>
+  </si>
+  <si>
+    <t>Tạ có chút việc hẹn Ngài khi khác nói chuyện.</t>
+  </si>
+  <si>
+    <t>Thiên Bồng Đại Nguyên Soái</t>
+  </si>
+  <si>
+    <t>STR_DLG_Marshal_Tianpeng_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>Người là ai mà dám tới đây làm loạn?</t>
+  </si>
+  <si>
+    <t>STR_DLG_Marshal_Tianpeng_Default_Choice_Ask</t>
+  </si>
+  <si>
+    <t>STR_DLG_Marshal_Tianpeng_Default_Choice_End</t>
+  </si>
+  <si>
+    <t>Ngươi là ai mà dám ngăn cản ta?</t>
+  </si>
+  <si>
+    <t>Từ chối xưng tên</t>
+  </si>
+  <si>
+    <t>STR_DLG_Marshal_Tianpeng_Default_Node_End</t>
+  </si>
+  <si>
+    <t>STR_DLG_Marshal_Tianpeng_Default_Node_Ask</t>
+  </si>
+  <si>
+    <t>Ta không có ý định gây rối chỉ là hiểu nhầm thôi.</t>
+  </si>
+  <si>
+    <t>Ngươi là ai?</t>
+  </si>
+  <si>
+    <t>STR_DLG_Marshal_Tianpeng_Default_Node_Answer</t>
+  </si>
+  <si>
+    <t>Ta là Thiên Bồng Đại Nguyên Soái chỉ huy tám vạn thủy Quân Thiên Hà. Ta đang nhận lệnh canh giữ nơi này.</t>
+  </si>
+  <si>
+    <t>STR_DLG_Marshal_Tianpeng_Default_Node_Ask_01</t>
+  </si>
+  <si>
+    <t>Thì ra Đại Nguyên Soái, xin lỗi nhé! Còn ta là Tôn Ngộ Không đại danh Bật Mã Ôn mới nhận chức.</t>
+  </si>
+  <si>
+    <t>STR_DLG_Marshal_Tianpeng_Default_Node_Answer_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Marshal_Tianpeng_Default_Node_Ask_02</t>
+  </si>
+  <si>
+    <t>Ta cũng đang muốn lĩnh giáo đây.</t>
+  </si>
+  <si>
+    <t>Thì ra là tên chăn ngựa chả biết phép tắc gì cả, ngươi hãy cẩn thận với chiếc Cào Cửu Xỉ Đinh Ba trong tay ta.</t>
+  </si>
+  <si>
+    <t>Ta không cần biết! Ngài là Thủy Thần cai quản vùng này. Giờ ta hỏi ngắn gọn: Ngày mai thời tiết Hoa Quả Sơn thế nào? | Có đẹp trời để khỉ con nhà ta đi hái đào không?</t>
+  </si>
+  <si>
+    <t>Thế thì ta đa tạ Ngài. Khi khác ta lại ghé thăm, ta đi đây.</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_Marshal_Tianpeng_Default_Choice_Request_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Marshal_Tianpeng_Default_Choice_Request_02</t>
+  </si>
+  <si>
+    <t>Nhắc nhờ bảo vệ Sư Phụ</t>
+  </si>
+  <si>
+    <t>Bảo Bát Giới đi hỏi đường</t>
+  </si>
+  <si>
+    <t>Trêu chọc</t>
+  </si>
+  <si>
+    <t>Lão Trư sắp chết đói rồi! Ta không đi nữa đâu!</t>
+  </si>
+  <si>
+    <t>Tên heo mập ngốc nghếch kia! Mới đi được vài bước đã thở hồng hộc.| Hay là ta chia hành lý cho người về Cao Gia Trang làm rể ở đó.</t>
+  </si>
+  <si>
+    <t>Lại bắt đệ dắt ngựa.</t>
+  </si>
+  <si>
+    <t>Đệ không thể sánh được với người ăn gió uống sương như sư huynh đâu. | Hầu ca không biết từ ngày theo sư phụ đệ chưa được bữa ăn no nào cả.</t>
+  </si>
+  <si>
+    <t>Sư phụ con chỉ nói là đói bụng thế mà đại sư huynh bảo con là nhớ nhà. | Con đã hứa bảo vệ sư phụ đi lấy kinh thì sẽ không bao giờ hối hận đâu thế sao lại đuổi con về.</t>
+  </si>
+  <si>
+    <t>Sư phụ à lão Chư đói chóng cả mặt.</t>
+  </si>
+  <si>
+    <t>Ngộ Không con đi tìm ít thức ăn về đây nhé!</t>
+  </si>
+  <si>
+    <t>Sư phụ nơi này hoang vu không một bóng người con biết đi đâu mà tìm.</t>
+  </si>
+  <si>
+    <t>Sư huynh nhún một cái là bay đi một vạn tám ngàn dặm cơ mà, kiếm bữa cơm chay thì có gì khó khăn đâu.</t>
+  </si>
+  <si>
+    <t>Nơi đây vùng núi hoang vu có nhiều yêu quái, nếu ta đi yêu quái đến hại sư phụ thì ngươi tính làm sao đây.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ban ngày ban mặt lấy đâu ra yêu quái chứ. </t>
+  </si>
+  <si>
+    <t>Phía bên kia có một cánh rừng để ta qua đó kiếm chút hoa quả, đệ bảo vệ sư phụ cẩn thận.| Nếu để xẩy ra chuyện gì với sư phụ thì biết tay ta.</t>
+  </si>
+  <si>
+    <t>Bát Giới ta bảo người đi hỏi đường thì người hỏi như nào rồi?</t>
+  </si>
+  <si>
+    <t>Hang này là hang gì?</t>
+  </si>
+  <si>
+    <t>Núi này là núi gì?</t>
+  </si>
+  <si>
+    <t>Hang đá.</t>
+  </si>
+  <si>
+    <t>Núi đá.</t>
+  </si>
+  <si>
+    <t>Ngoài hang có cửa gì?</t>
+  </si>
+  <si>
+    <t>Cửa sắt đầy đinh.</t>
+  </si>
+  <si>
+    <t>Trong hang dài bao nhiêu? Trong hang có ba cánh cửa trên cánh cửa có nhiều đinh, bao nhiêu thì lão Chư nhớ không rõ đúng không?</t>
+  </si>
+  <si>
+    <t>Sư huynh chưa lên núi làm sao mà biết được?</t>
+  </si>
+  <si>
+    <t>Ngộ Không bảo con nói dối ta không tin, nào ngờ đúng là như vậy con đáng bị ăn đòn lắm.</t>
+  </si>
+  <si>
+    <t>Ấy Sư phụ</t>
+  </si>
+  <si>
+    <t>Ngộ không thôi đừng đánh nó hãy để xem nó sau này như nào rồi hãng ra đòn.</t>
+  </si>
+  <si>
+    <t>Đệ không dám nữa. Sư phụ con đi ngay đây.</t>
+  </si>
+  <si>
+    <t>STR_DLG_Marshal_Tianpeng_Default_Choice_Request_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_03_00</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_03_01</t>
+  </si>
+  <si>
+    <t>Bát Giới nếu nhớ nhà thì con hãy về đi.</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_03_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_03_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_03_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_03_05</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_03_06</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_01_00</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_01_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_01_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_01_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_01_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_01_05</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_01_06</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_02_00</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_02_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_02_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_02_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_02_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_02_05</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_02_06</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_02_07</t>
+  </si>
+  <si>
+    <t>Cái con chim đó là do huynh biến hóa đó à. | Sư phụ, Sư phụ cứu con với ạ.</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_02_09</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_02_10</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_02_11</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_02_12</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_02_13</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_02_14</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_02_15</t>
+  </si>
+  <si>
+    <t>STR_DLG_Zhu_Baije_Default_Node_Request_02_08</t>
+  </si>
+  <si>
+    <t>Ta phải cho người biết tay. Ngươi đâu lên núi ngươi trốn đi ngủ. | Nếu con chim gõ kiến không gõ vào mũi của người thì người còn gáy khò khò.</t>
+  </si>
+  <si>
+    <t>Vậy thì con hãy mau đi nhanh đi.</t>
+  </si>
+  <si>
+    <t>Bát Giới , mau đi dắt ngựa đi.</t>
+  </si>
+  <si>
+    <t>Tôn Hầu Tử!</t>
+  </si>
+  <si>
+    <t>Ngươi là con cái nhà ai mà dám ra đây cản ta.</t>
+  </si>
+  <si>
+    <t>Ha ha, khá lắm nhà ngươi vắt mũi còn chưa sạch mà nói lời to tác vậy. Thôi nhanh về nhà với cha mẹ ngươi đi.</t>
+  </si>
+  <si>
+    <t>Ta là Tam Thái Tử Na Tra, nay vâng thánh chỉ đến bắt nhà ngươi đây.</t>
+  </si>
+  <si>
+    <t>Yêu hầu chớ vô lễ, hãy xem thương của ta đây.</t>
+  </si>
+  <si>
+    <t>Bất mãn</t>
+  </si>
+  <si>
+    <t>Ta hiểu nỗi uất hận của ngươi... Nhưng lấy bạo lực đối đầu với Thiên Quy chỉ đem lại tai họa cho Hoa Quả Sơn thôi!</t>
+  </si>
+  <si>
+    <t>So tài</t>
+  </si>
+  <si>
+    <t>Này Na Tra có dám đua với ta một chuyến tới Nam Thiên Môn không?</t>
+  </si>
+  <si>
+    <t>Được! Nếu ta thắng ngươi phải bao ta một chầu rượu ngon ở Thiên Đình! Xuất Phát!</t>
+  </si>
+  <si>
+    <t>STR_DLG_Third_Prince_Nezha_Default_Choice_Request_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Third_Prince_Nezha_Default_Choice_Request_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Third_Prince_Nezha_Default_Choice_Request_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Third_Prince_Nezha_Default_Node_Request_01_00</t>
+  </si>
+  <si>
+    <t>STR_DLG_Third_Prince_Nezha_Default_Node_Request_01_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Third_Prince_Nezha_Default_Node_Request_01_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Third_Prince_Nezha_Default_Node_Request_01_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Third_Prince_Nezha_Default_Node_Request_01_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_Third_Prince_Nezha_Default_Node_Request_02_00</t>
+  </si>
+  <si>
+    <t>STR_DLG_Third_Prince_Nezha_Default_Node_Request_02_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Third_Prince_Nezha_Default_Node_Request_02_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Third_Prince_Nezha_Default_Node_Request_02_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Third_Prince_Nezha_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>Chà chà, ta lại được một trận đùa với trẻ con đây rồi.</t>
+  </si>
+  <si>
+    <t>Na Tra ngươi là Tam Thái Tử còn ta chỉ là một Hầu Vương từ trong đá mà chui ra.| Ngươi là cây cầu trên trời còn ta bùn đất ở dưới trần thì sao ngươi hiểu được chứ. | Trời đất này do thực lực nói chuyện! Thiên Đình ép ta, ta đập tan Thiên Đình. Để xem ai làm gì nổi Tề Thiên Đại Thánh!</t>
+  </si>
+  <si>
+    <t>STR_DLG_Third_Prince_Nezha_Default_Node_Request_03_00</t>
+  </si>
+  <si>
+    <t>STR_DLG_Third_Prince_Nezha_Default_Node_Request_03_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Third_Prince_Nezha_Default_Node_Request_03_02</t>
+  </si>
+  <si>
+    <t>Đại Thánh! Người đời cứ đồn Cân Đẩu Vân của người là đệ nhất thiên hạ. |Phong Hỏa Luân của ta lướt gió xe mây cũng đâu có kém! Đua thì được thui nhưng nếu thua Ngươi phải chỉ ta phép Phân Thân đấy.</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>Yêu hầu kia còn không mau tuông tay chiu trói.</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_01_00</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Choice_Request_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Choice_Request_02</t>
+  </si>
+  <si>
+    <t>Ta được phong là Chiêu Huệ Linh Hiển Vương, Nhị Lang Thần là ta. Nay phụng mệnh đến bắt Bạch Mã Ôn tạo phản Thiên Cung.</t>
+  </si>
+  <si>
+    <t>Ta nhớ Ngọc Đế có một muội muội vì tình hạ giới kết duyên cùng người phàm họ Dương. | Hạ sinh ra một đứa con trai vác búa lên núi để giải cứu mẫu thân. | Đó là ngươi sao.</t>
+  </si>
+  <si>
+    <t>Chính là Chân Quân ta.</t>
+  </si>
+  <si>
+    <t>Cái gì mà Chân Quân vs Giả Quân. Người còn có một cái tên gọi là Tiểu Thánh có đúng không?</t>
+  </si>
+  <si>
+    <t>Đúng vậy.</t>
+  </si>
+  <si>
+    <t>Vậy đúng rồi, ta đây là Đại Thánh còn ngươi là Tiểu Thánh. Nếu tính về cấp bậc ngươi còn kém ta xa đó.</t>
+  </si>
+  <si>
+    <t>Yêu hầu miệng lưỡi ngươi cũng lợi hại lắm. Hãy tiếp chiêu của ta đây.</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_01_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_01_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_01_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_01_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_01_05</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_01_06</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_01_07</t>
+  </si>
+  <si>
+    <t>Nghe danh Thiên Nhãn của ngươi đã lâu. Hôm nay xem nó có nhìn thấu 72 phép biến hóa của ta không!</t>
+  </si>
+  <si>
+    <t>Cứ thi triển đi. Chỉ cần còn một sơ hở, ngươi không thoát khỏi mắt ta.</t>
+  </si>
+  <si>
+    <t>Ta hóa thành chim sẻ, xem ngươi đuổi kịp không!</t>
+  </si>
+  <si>
+    <t>Muốn bay à? Vậy ta hóa chim ưng!</t>
+  </si>
+  <si>
+    <t>Hừ! Ta lao xuống nước, hóa thành cá nhỏ!</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Ta hóa </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>chim hạc</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, chuyên bắt cá!</t>
+    </r>
+  </si>
+  <si>
+    <t>Hay cho tên Dương Tiễn kia. | Thế thì ta biến cả thân mình thành ngôi miếu, xem ngươi nhận ra nổi không!</t>
+  </si>
+  <si>
+    <t>Miếu nào lại có cột cờ dựng sau điện? Cái đuôi khỉ của ngươi đã lộ rồi!</t>
+  </si>
+  <si>
+    <t>Ha ha! Quả nhiên Thiên Nhãn danh bất hư truyền. Hôm nay xem như gặp đúng đối thủ!</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_02_00</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_02_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_02_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_02_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_02_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_02_05</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_02_06</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_02_07</t>
+  </si>
+  <si>
+    <t>STR_DLG_ErlangShen_Default_Node_Request_02_08</t>
+  </si>
+  <si>
+    <t>STR_LOCAL_SPIRIT</t>
+  </si>
+  <si>
+    <t>Local Spirit of the Flat-Peach Garden</t>
+  </si>
+  <si>
+    <t>Thổ địa vừa đào tiên</t>
+  </si>
+  <si>
+    <t>Hỏi về vường đào tiên</t>
+  </si>
+  <si>
+    <t>Ngọc Hoàng sai ta cai quản vườn đào này nên ta đến xem thế nào. Mà người là ai vậy?</t>
+  </si>
+  <si>
+    <t>Thọ ngang trời đất cơ à. Để ta thử xem nào.</t>
+  </si>
+  <si>
+    <t>Ây không được phép đâu ngài</t>
+  </si>
+  <si>
+    <t>Vâng. Thần xin cáo lui.</t>
+  </si>
+  <si>
+    <t>STR_DLG_Local_Spirit_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_Local_Spirit_Default_Node_Ask</t>
+  </si>
+  <si>
+    <t>STR_DLG_Local_Spirit_Default_Choice_Ask</t>
+  </si>
+  <si>
+    <t>STR_DLG_Local_Spirit_Default_Node_Answer</t>
+  </si>
+  <si>
+    <t>STR_DLG_Local_Spirit_Default_Node_Answer_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Local_Spirit_Default_Node_Answer_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Local_Spirit_Default_Node_Answer_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Local_Spirit_Default_Node_Answer_04</t>
+  </si>
+  <si>
+    <t>Ta là quan thổ địa ở đây. Mời ngài đi kiểm tra. | Đại Thanh toàn bộ khu vườn này có 3600 gốc đào. | Phía trước có 1200 gốc, ba ngàn năm mới có quả chín. Ăn vào người mạnh khỏe nhẽ nhõm. | Đại Thánh, ở giữa cũng có 1200 gốc, sáu ngàn năm mới có quả chín. Ăn vào rồi thì trường sinh bất lão. | Phía sau cũng có 1200 gốc, chín ngàn năm mới có quả chín. Ăn vào rồi thì thọ ngang trời đất.</t>
+  </si>
+  <si>
+    <t>Ta mệt quá rồi cần nghỉ ngơi một nát, cho nhà người lui đó.</t>
+  </si>
+  <si>
+    <t>Đại Thánh, sao người rảnh rỗi tới chơi vườn đào thế này.</t>
+  </si>
+  <si>
+    <t>Ngươi là tiểu tướng phương nào mà dám tới đây khiêu chiến với ta chứ.</t>
+  </si>
+  <si>
+    <t>Đại Thánh! Bản lĩnh của người thần thông, Tam Đầu Lục Tí của ta cũng không áp chế được ngươi. | Nhưng ngươi quá kiêu ngạo rồi! Bản lĩnh ngươi cao thật, nhưng thiên ngoại hữu thiên.| Nếu ngươi cứ đại náo tiếp thì tự dồn vào chỗ chết thui.</t>
+  </si>
+  <si>
+    <t>Dừng lại sao? | Họ coi ta là con khỉ quê mùa, phong cái chức Bật Mã Ôn coi chuồng ngựa để nhạo báng ta! Bản lĩnh này của ta há để họ chà đạp?</t>
+  </si>
+  <si>
+    <t>Sư phụ bảo ta đừng đánh ta sẽ tha cho ngươi. Nhưng sẽ phạt ngươi đi tuần núi. Mau đi đi.</t>
+  </si>
+  <si>
+    <t>Đại Thánh oan cho thần quá! Thần quản sông quản biển chứ đâu có quản thời tiết của Hoa Quả Sơn. | Mưa gió là do Lôi Công, Điện Mẫu với Phong Bác tạo ra đấy chứ!</t>
+  </si>
+  <si>
+    <t>Này cháu của ta, còn không mau qua đây nhận thúc thúc của ngươi đi.</t>
+  </si>
+  <si>
+    <t>Nhảm nhí, ai họ hàng gì với ngươi, người là người ở đâu còn ta là người ở đâu sao có thể huynh đệ của phụ vương ta được.</t>
+  </si>
+  <si>
+    <t>STR_DLG_TheBoySage_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_TheBoySage_Default_Node_Start_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_TheBoySage_Default_Node_Start_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_TheBoySage_Default_Node_Start_03</t>
+  </si>
+  <si>
+    <t>Cháu không biết đó thôi. Ta là Tề Thiên Đại Thánh, 500 năm trước từng đại náo Thiên Cung. | Khi ta kết nghĩa phụ thân của ngươi, ngươi vẫn còn chưa ra đời đâu. | Ngươi nên gọi ta một tiếng thúc thúc phải không?</t>
+  </si>
+  <si>
+    <t>Con khỉ chết tiệt này, ngươi dám khinh ta là trẻ con ta quyết không tha cho ngươi. Hãy xem Tam Muội Chân Hỏa của ta đây.</t>
+  </si>
+  <si>
+    <t>Ngươi là Tôn Ngộ Không?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đúng rồi! Đã lâu không gặp, trông đại ca phong độ hơn xưa. </t>
+  </si>
+  <si>
+    <t>STR_DLG_Bull_Demon_ King_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bull_Demon_ King_Default_Node_Start_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bull_Demon_ King_Default_Node_Start_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bull_Demon_ King_Default_Node_Start_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bull_Demon_ King_Default_Node_Start_04</t>
+  </si>
+  <si>
+    <t>Ngưu đại ca, đại ca còn nhận ra tiểu đệ không?</t>
+  </si>
+  <si>
+    <t>Việc của nhà lão ta không muốn can dự.</t>
+  </si>
+  <si>
+    <t>Thế còn hồ lô của ngươi lấy từ đâu ra.</t>
+  </si>
+  <si>
+    <t>Thì hồ lô của ta cũng lấy từ cây thần đó.</t>
+  </si>
+  <si>
+    <t>Lúc đó trên cây tiên già có hai quả hồ lô. Của mi là hồ lô cái còn của ta là hồ lô đực.</t>
+  </si>
+  <si>
+    <t>Ta không cần biết là đực hay cái. Ta gọi tên ngươi, người có dám trả lời ta không?</t>
+  </si>
+  <si>
+    <t>Ông nội của ngươi đây.</t>
+  </si>
+  <si>
+    <t>Hả! Sao lại không được.</t>
+  </si>
+  <si>
+    <t>Đệ đệ ở đây ta có bức hình có vẽ lại 4 thầy trò đường tăng.</t>
+  </si>
+  <si>
+    <t>Cái miệng tên hòa thượng này rất là dài.</t>
+  </si>
+  <si>
+    <t>Hòa thượng mau đưa cái miệng ra.</t>
+  </si>
+  <si>
+    <t>Để đệ móc mõm của nó ra.</t>
+  </si>
+  <si>
+    <t>Ha ha ha. Bắt tên Trư Bát Giới lại.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đại sư huynh ơi mau tới cứu đệ. </t>
+  </si>
+  <si>
+    <t>Người phía trước là ai.</t>
+  </si>
+  <si>
+    <t>Ai nói dài đâu mà dài.</t>
+  </si>
+  <si>
+    <t>Đây đây các ngươi nhìn thỏa thích đi.</t>
+  </si>
+  <si>
+    <t>Yêu quái hãy xem một gậy của ta đây.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mi là ai mà dám tới đây la ó. </t>
+  </si>
+  <si>
+    <t>Ta là Hành Giả Tôn anh em của Tôn Hành Giả.</t>
+  </si>
+  <si>
+    <t>Hồ lô của ta do một ông tiên Thái Sơn hái từ một cây tiên già trên núi Côn Lôn từ thủa khai thiên lập địa mà có.</t>
+  </si>
+  <si>
+    <t>Được! Vậy thì ngươi cứ gọi đi.</t>
+  </si>
+  <si>
+    <t>Hành Giả Tôn.</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Choice_Request_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Choice_Request_02</t>
+  </si>
+  <si>
+    <t>Khiêu khích</t>
+  </si>
+  <si>
+    <t>Tuần núi</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_01_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_01_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_01_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_01_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_01_05</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_01_06</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_01_07</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_01_08</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_01_09</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_01_10</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_01_11</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_01_12</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_01_13</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_01_14</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_01_00</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_02_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_02_00</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_02_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_02_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_02_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_02_05</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_02_06</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_02_07</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_02_08</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_02_09</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_02_10</t>
+  </si>
+  <si>
+    <t>STR_DLG_SilverHornKing_Default_Node_Request_02_11</t>
+  </si>
+  <si>
+    <t>Bọn may đâu mau đi bắt Đường Tăng về đây.</t>
+  </si>
+  <si>
+    <t>Nếu ta nói là hòa thượng đi thỉnh kinh thì chắc chắn bị chúng bắt về. | Tôi chỉ là người đi đường thui.</t>
+  </si>
+  <si>
+    <t>Tên mặt đầy lông lá này chính là Tôn Ngộ Không còn tên tai to mõm dài này là Trư Bát Giới. | Ngươi chính là Trư Bát Giới có đúng không?</t>
+  </si>
+  <si>
+    <t>Hành Giả Tôn ngươi lấy đâu ra cái bình hồ lô đó.</t>
+  </si>
+  <si>
+    <t>Ngươi đừng có mà khoác loác.</t>
+  </si>
+  <si>
+    <t>Cái gì! Ah ah ah.</t>
+  </si>
+  <si>
+    <t>Ha Ha Ha! Bây giời thời thế khác rồi. Hồ lô của ngươi thấy con đực không dám ra oai nữa đấy. | Hãy xem hồ lô của ta đây. Ngân Giác Đại Vương!</t>
+  </si>
+  <si>
+    <t>Cái tên nửa sư nửa khỉ kia dám đến đây gây rối.</t>
+  </si>
+  <si>
+    <t>Người không biết tên ông ngoại của ngươi à. |  Nếu còn không mang giao trả sư phụ cho ta, ta sẽ san phẳng ngọn núi này cho các ngươi đoạn tử tuyệt tôn,</t>
+  </si>
+  <si>
+    <t>Hử! Con khỉ kia ngươi là cái thá gì mà dám khuênh khoang vậy chứ.</t>
+  </si>
+  <si>
+    <t>Ta chính là Tề Thiên Đại Thánh Tôn Ngộ Không đã từng đại náo Thiên Cung năm trăm năm trước đây.</t>
+  </si>
+  <si>
+    <t>Còn tưởng là ai, hóa ra là Bật Mã Ôn đây. Chỉ là tên chăn ngựa cho Ngọc Hoàng.</t>
+  </si>
+  <si>
+    <t>Ah ah ah, Yêu quái hãy đỡ một gậy của lão Tôn đây.</t>
+  </si>
+  <si>
+    <t>STR_DLG_YellowWindMonster_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_YellowWindMonster_Default_Node_Start_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_YellowWindMonster_Default_Node_Start_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_YellowWindMonster_Default_Node_Start_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_YellowWindMonster_Default_Node_Start_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_YellowWindMonster_Default_Node_Start_05</t>
+  </si>
+  <si>
+    <t>Hư liên quan gì tới ngươi.</t>
+  </si>
+  <si>
+    <t>Ngươi to gan thật đấy. Ngay đến cha ngươi cũng phải ngường nhịn ta. Ngươi dám dở trò ma quái bắt cóc sư phụ ta.</t>
+  </si>
+  <si>
+    <t>Tên nghiệt súc này ngươi còn dám ăn nói ngông cuồng nữa hả.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tên nghiệt súc này hóa ra ngươi ở đây tác quái. </t>
+  </si>
+  <si>
+    <t>Có gì mà ta không dám, bọn chúng sợ ngươi còn ta thì không. | Nếu không phải bọn hèn nhát đấy, thì ta đã ăn thịt của Đường Tăng rồi.</t>
+  </si>
+  <si>
+    <t>Tên ngông cuồng này hết thuốc chữa rồi. Lão Tôn này định cho ngươi một gậy. Nhưng sợ cây gậy này đánh quá sẽ đánh chết ngươi. | Nể mặt lão Long Vương ta sẽ tha chết cho ngươi. | Nói mau ngươi nhốt sư phụ của ta ở dâu.</t>
+  </si>
+  <si>
+    <t>STR_DLG_ThirdDragonPrince_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_ThirdDragonPrince_Default_Node_Start_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_ThirdDragonPrince_Default_Node_Start_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_ThirdDragonPrince_Default_Node_Start_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_ThirdDragonPrince_Default_Node_Start_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_ThirdDragonPrince_Default_Node_Start_05</t>
+  </si>
+  <si>
+    <t>Lại là con khỉ đột nhà ngươi.</t>
+  </si>
+  <si>
+    <t>Yêu quái mau mau giao sư phụ của ta ra đây ngay.</t>
+  </si>
+  <si>
+    <t>Muốn cứu được sư phụ ngươi thì hãy thắng được hai cây ngân trùy của ta rồi nói.</t>
+  </si>
+  <si>
+    <t>Ngân trùy cái gì, chỉ là thứ sắt vụn mà thôi.</t>
+  </si>
+  <si>
+    <t>Ta khinh, trước mặt Kim Cô Bổng của Tôn Ngộ Không ta thì thứ gì cũng chỉ là sắt vụn thôi. Hây, xem gậy của ta đây.</t>
+  </si>
+  <si>
+    <t>STR_DLG_GoldfishDemon_Default_Node_Start_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_GoldfishDemon_Default_Node_Start_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_GoldfishDemon_Default_Node_Start_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_GoldfishDemon_Default_Node_Start_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_GoldfishDemon_Default_Node_Start_05</t>
+  </si>
+  <si>
+    <t>STR_DLG_GoldfishDemon_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>Cửu Biện Xích Đồng Trùy của ta được tạo ra từ hồ sen trên trời, được ta dốc sức mà luyện thành. | Binh khí thần thánh lợi hại nào ở trước mặt ta đều không đỡ được một búa đâu.</t>
+  </si>
+  <si>
+    <t>Vì ngươi không thành tâm tu luyện phò tá Đường Tăng cho nên ta mới dùng vòng Kim Cô để quản thúc ngươi.</t>
+  </si>
+  <si>
+    <t>Xin Bồ Tác hãy tháo vòng Kim Cô cho con đi, con xin lậy Bồ Tác.</t>
+  </si>
+  <si>
+    <t>Ngộ Không, không được nói bậy. Bây giời ngươi đã được thoát nạn không được lười biếng. | Dốc lòng phò tá Đường Tăng đi lấy kinh xong việc ngươi sẽ thành Chính Quả. | Trên Đường đi nếu gặp nạn ta sẽ cứu giúp.</t>
+  </si>
+  <si>
+    <t>Phò tá Đường Tăng không thể cưỡi mây vượt gió được, biết bao giờ mới tới được Tây Trúc lấy kinh. | Con không đi nữa đâu.</t>
+  </si>
+  <si>
+    <t>Tạ ơn Bồ Tát.</t>
+  </si>
+  <si>
+    <t>STR_DLG_Guanyin_Bodhisattva_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_Guanyin_Bodhisattva_Default_Node_Start_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Guanyin_Bodhisattva_Default_Node_Start_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Guanyin_Bodhisattva_Default_Node_Start_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Guanyin_Bodhisattva_Default_Node_Start_04</t>
+  </si>
+  <si>
+    <t>Bái sư.</t>
+  </si>
+  <si>
+    <t>Nhà ngươi là ai? Đến đây làm gì?</t>
+  </si>
+  <si>
+    <t>Thế tên họ ngươi là gì?</t>
+  </si>
+  <si>
+    <t>Thưa sư tổ con xin đến đây học đạo. Xin sư tổ hãy nhận con đi.</t>
+  </si>
+  <si>
+    <t>Thưa Sư tổ con không họ cũng không tên chỉ biết con nứt ra từ một phiến đá ở Hoa Quả Sơn thui.</t>
+  </si>
+  <si>
+    <t>Sư phụ nhận con rồi ạ. | Ta đã có tên rồi. | Tên của ta là Tôn Ngộ Không. | Ha ha ha!</t>
+  </si>
+  <si>
+    <t>Học phép thuật</t>
+  </si>
+  <si>
+    <t>Được!</t>
+  </si>
+  <si>
+    <t>Ngươi cũng đến chỗ ta học đạo được 7 năm rồi. Vậy ngươi muốn được học pháp thuật gì?</t>
+  </si>
+  <si>
+    <t>Sư phụ dạy gì thì con học đấy, cốt là được trường sinh bất tử thui ạ.</t>
+  </si>
+  <si>
+    <t>Vậy có sống lâu được không?</t>
+  </si>
+  <si>
+    <t>Ta sẽ dậy ngươi Tục Kinh Niệm Phật</t>
+  </si>
+  <si>
+    <t>Không được, muốn sống lâu không khác gì mò trăng đáy nước.</t>
+  </si>
+  <si>
+    <t>Theo sư phụ nói thì cũng chẳng lâu bền. Không học. Không học.</t>
+  </si>
+  <si>
+    <t>Thế có trường sinh được không ạ?</t>
+  </si>
+  <si>
+    <t>Sư phụ dậy con cả 72 phép luôn ạ.</t>
+  </si>
+  <si>
+    <t>Cái con khỉ kia đạo này không học, đạo kia cũng không học.</t>
+  </si>
+  <si>
+    <t>Con đã luyện được đến đâu rồi.</t>
+  </si>
+  <si>
+    <t>Thưa sư phụ, con đã cưỡi mây vượt gió rồi ạ.</t>
+  </si>
+  <si>
+    <t>Con mới bay nhảy cách mặt đất bốn năm trượng thôi, chưa gọi là cưỡi mây mà gọi là bò ở trên mây. | Cưỡi mây là bay nhanh qua biển cả mênh mông ấy.</t>
+  </si>
+  <si>
+    <t>Khó lắm đấy phải khổ luyện thì mới được.</t>
+  </si>
+  <si>
+    <t>Khổ mấy con cũng xin học.</t>
+  </si>
+  <si>
+    <t>Được! Ta sẽ dạy con phép Cân Đẩu Vân. Chỉ cần nhúng người sẽ bay xa mười vạn tám ngàn dặm.</t>
+  </si>
+  <si>
+    <t>Tuyệt quá sư phụ.</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Choice_Request_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Choice_Request_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Choice_Request_03</t>
+  </si>
+  <si>
+    <t>Học Cân Đẩu Vân</t>
+  </si>
+  <si>
+    <t>Sư phụ! Đệ tử chí thành khấu đầu!</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_01_00</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_01_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_01_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_01_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_01_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_01_05</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_02_00</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_02_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_02_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_02_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_02_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_02_05</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_02_06</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_02_07</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_02_08</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_02_09</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_02_10</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_02_11</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_02_12</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_02_13</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_03_00</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_03_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_03_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_03_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_03_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_03_05</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_03_06</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_03_07</t>
+  </si>
+  <si>
+    <t>Thì ra thế. Nhà ngươi là con đất con trời. Tướng mạo giống trẻ con thì lấy họ là Tôn. | Ngươi lại muốn tu đạo hiền thì lấy tên Ngộ Không nhé.</t>
+  </si>
+  <si>
+    <t>Sư phụ dạy con có được không ạ?</t>
+  </si>
+  <si>
+    <t>Vật như hư, đệ tử theo học cũng hoài công vô ích!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Học môn này mà muốn trường sinh thì giống như hái hoa trong gương vậy. </t>
+  </si>
+  <si>
+    <t>Thế ta dạy ngươi môn Than Thiền Đả Toạn được không?</t>
+  </si>
+  <si>
+    <t>Lâu nay con chỉ mong ước luyện được phép trường sinh. Mong sư phụ dạy con đi ạ.</t>
+  </si>
+  <si>
+    <t>Ta có hai loại phép thuật tránh được tam tai, một loại có 36 phép một loại có 72 phép. | Vậy ngươi muốn học loại nào?</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bodhi_Patriarch_Default_Node_Request_02_14</t>
+  </si>
+  <si>
+    <t>Con khỉ này lần trước đã chén hết mấy hồ lô linh đan mà mấy ngày năm ta đã luyện được. | Hôm nay đến đây làm gì?</t>
+  </si>
+  <si>
+    <t>Chẳng qua đi ngang qua Nam Thiên Môn, nhớ mùi trà thơm của ngài nên ghé vào xin một chén, sẵn tiện nghỉ chân chút thôi.</t>
+  </si>
+  <si>
+    <t>Lão Quân, xin hãy dừng bước.</t>
+  </si>
+  <si>
+    <t>STR_DLG_Taishang_Laojun_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_Taishang_Laojun_Default_Node_Start_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Taishang_Laojun_Default_Node_Start_02</t>
+  </si>
+  <si>
+    <t>Ta lại e ngươi chê trà của ta không ngọt bằng đan dược ngày trước.</t>
+  </si>
+  <si>
+    <t>STR_DLG_Taishang_Laojun_Default_Node_Start_03</t>
+  </si>
+  <si>
+    <t>Đừng có có khua môi múa mép nữa, tại sao ngươi lại bắt nạt vợ ta chứ.</t>
+  </si>
+  <si>
+    <t>Con khỉ kia. Ngươi bắt nạt vợ ta, hại con ta, đánh thiếp của ta mà còn vác mặt tới đây nói chuyện tình nghĩ nữa hả. | Hãy xem một đao của ta đây.</t>
+  </si>
+  <si>
+    <t>Nếu ngươi đấu được với ta thì ta bảo vợ ta cho mượn quạt.</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bull_Demon_ King_Default_Node_Start_05</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bull_Demon_ King_Default_Node_Start_06</t>
+  </si>
+  <si>
+    <t>STR_DLG_Bull_Demon_ King_Default_Node_Start_07</t>
+  </si>
+  <si>
+    <t>Tôn Ngộ Không à, chắc con khỉ đấy lại gặp rắc rối rồi đây. | Cho nó vào đây.</t>
+  </si>
+  <si>
+    <t>Ngọc Hoàng, Lão Tôn đến làm phiền ngài đây.</t>
+  </si>
+  <si>
+    <t>Sao hôm nay con khỉ này lễ phép thế nhỉ?</t>
+  </si>
+  <si>
+    <t>Vâng ạ.</t>
+  </si>
+  <si>
+    <t>Ngài mau đi nhanh kẻo sư phụ của ta bị ăn thịt mất. | Xin đa tạ.</t>
+  </si>
+  <si>
+    <t>Khởi bẩng Ngọc Hoàng có Tôn Ngộ Không cầu kiến.</t>
+  </si>
+  <si>
+    <t>Lão Tôn lên trên này nhờ Ngọc Hoàng kiểm tra xem trên trời có hung tinh hạ phàm chặn đường đi của Lão Tôn hay không? | Xin Ngọc Hoàng hãy cho người đi thu phục tên yêu quái đó. | Lão Tôn xin biết ơn vô hạn.</t>
+  </si>
+  <si>
+    <t>Thái Bạch Kim Tinh, ngươi hãy đi hỏi Thiên Tinh Đẩu và các vị Thần Vương xem có tiên phàm hạ giới không?</t>
+  </si>
+  <si>
+    <t>STR_DLG_Jade_Emperor_Default_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_Jade_Emperor_Default_Node_Start_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Jade_Emperor_Default_Node_Start_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Jade_Emperor_Default_Node_Start_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Jade_Emperor_Default_Node_Start_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_Jade_Emperor_Default_Node_Start_05</t>
+  </si>
+  <si>
+    <t>STR_DLG_Jade_Emperor_Default_Node_Start_06</t>
+  </si>
+  <si>
+    <t>STR_DLG_Jade_Emperor_Default_Node_Start_07</t>
+  </si>
+  <si>
+    <t>STR_DLG_Jade_Emperor_Default_Node_Start_08</t>
+  </si>
+  <si>
+    <t>Tôn Ngộ Không chẳng phải ngươi đang bảo vệ Đường Tăng đi Tây Thiên lấy kinh hay sao?</t>
+  </si>
+  <si>
+    <t>Đại cơ bớt giận, tiểu đệ nhất thời lỗ mãn làm đại tẩu sợ hãi. Xin đại ca tha cho nhé. | Tiểu đệ đang phò tá Đường Tăng tớ Tây Trúc thỉnh kinh. Nhưng đi tới Hỏa Diệm Sơn thì không qua được.| Đệ đã tới mượn đại tẩu chiếc quạt quí, ai ngờ đại tẩu nhất quyết không cho mượn. | Cho nên nhờ đại ca mượn giúp.</t>
+  </si>
+  <si>
+    <t>Đại ca đấu thì đấu, hãy cho ta mượn quạt đi.</t>
   </si>
 </sst>
 </file>
@@ -5467,7 +6714,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -5492,6 +6739,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -5505,7 +6758,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5519,6 +6772,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7095,68 +8349,68 @@
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
+        <v>1243</v>
+      </c>
+      <c r="B119" t="s">
         <v>1244</v>
       </c>
-      <c r="B119" t="s">
+      <c r="C119" t="s">
         <v>1245</v>
-      </c>
-      <c r="C119" t="s">
-        <v>1246</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
+        <v>1314</v>
+      </c>
+      <c r="B120" t="s">
         <v>1315</v>
       </c>
-      <c r="B120" t="s">
+      <c r="C120" t="s">
         <v>1316</v>
-      </c>
-      <c r="C120" t="s">
-        <v>1317</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
+        <v>1317</v>
+      </c>
+      <c r="B121" t="s">
         <v>1318</v>
       </c>
-      <c r="B121" t="s">
+      <c r="C121" t="s">
         <v>1319</v>
-      </c>
-      <c r="C121" t="s">
-        <v>1320</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
+        <v>1320</v>
+      </c>
+      <c r="B122" t="s">
         <v>1321</v>
       </c>
-      <c r="B122" t="s">
+      <c r="C122" t="s">
         <v>1322</v>
-      </c>
-      <c r="C122" t="s">
-        <v>1323</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
       <c r="B123" t="s">
+        <v>1323</v>
+      </c>
+      <c r="C123" t="s">
         <v>1324</v>
-      </c>
-      <c r="C123" t="s">
-        <v>1325</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
+        <v>1326</v>
+      </c>
+      <c r="B124" t="s">
         <v>1327</v>
       </c>
-      <c r="B124" t="s">
+      <c r="C124" t="s">
         <v>1328</v>
-      </c>
-      <c r="C124" t="s">
-        <v>1329</v>
       </c>
     </row>
   </sheetData>
@@ -7167,12 +8421,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C262"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="51" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="36.7109375" customWidth="1"/>
-    <col min="3" max="3" width="47.140625" customWidth="1"/>
+    <col min="1" max="1" width="61.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.140625" customWidth="1"/>
+    <col min="3" max="3" width="255.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -7546,7 +8800,7 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>1386</v>
+        <v>1385</v>
       </c>
       <c r="C43" t="s">
         <v>746</v>
@@ -7554,15 +8808,15 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>1387</v>
+        <v>1386</v>
       </c>
       <c r="C44" t="s">
-        <v>1385</v>
+        <v>1384</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>1388</v>
+        <v>1387</v>
       </c>
       <c r="C45" t="s">
         <v>163</v>
@@ -7570,7 +8824,7 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>1389</v>
+        <v>1388</v>
       </c>
       <c r="C46" t="s">
         <v>747</v>
@@ -7578,39 +8832,39 @@
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>1397</v>
+        <v>1396</v>
       </c>
       <c r="C47" t="s">
-        <v>1390</v>
+        <v>1389</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>1398</v>
+        <v>1397</v>
       </c>
       <c r="C48" t="s">
-        <v>1392</v>
+        <v>1391</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>1399</v>
+        <v>1398</v>
       </c>
       <c r="C49" t="s">
-        <v>1411</v>
+        <v>1419</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>1410</v>
+        <v>1409</v>
       </c>
       <c r="C50" t="s">
-        <v>1391</v>
+        <v>1390</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>1400</v>
+        <v>1399</v>
       </c>
       <c r="C51" t="s">
         <v>717</v>
@@ -7618,58 +8872,1690 @@
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>1401</v>
+        <v>1400</v>
       </c>
       <c r="C52" t="s">
-        <v>1393</v>
+        <v>1392</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>1401</v>
+      </c>
+      <c r="C53" t="s">
+        <v>1393</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>1410</v>
+      </c>
+      <c r="C54" t="s">
+        <v>1411</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C55" t="s">
+        <v>1413</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>1414</v>
+      </c>
+      <c r="C56" t="s">
+        <v>1597</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>1415</v>
+      </c>
+      <c r="C57" t="s">
+        <v>1439</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>1416</v>
+      </c>
+      <c r="C58" t="s">
+        <v>1418</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>1417</v>
+      </c>
+      <c r="C59" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="7" t="s">
         <v>1402</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C60" t="s">
+        <v>1395</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="7" t="s">
+        <v>1403</v>
+      </c>
+      <c r="C61" t="s">
         <v>1394</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" s="7" t="s">
-        <v>1403</v>
-      </c>
-      <c r="C54" t="s">
-        <v>1396</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" s="7" t="s">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" s="7" t="s">
         <v>1404</v>
       </c>
-      <c r="C55" t="s">
-        <v>1395</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" s="7" t="s">
+      <c r="C62" t="s">
+        <v>1614</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" s="7" t="s">
         <v>1405</v>
       </c>
-      <c r="C56" t="s">
-        <v>1412</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" s="7" t="s">
+      <c r="C63" t="s">
+        <v>1407</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="7" t="s">
         <v>1406</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C64" t="s">
         <v>1408</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" s="7" t="s">
-        <v>1407</v>
-      </c>
-      <c r="C58" t="s">
-        <v>1409</v>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="9" t="s">
+        <v>1421</v>
+      </c>
+      <c r="C65" t="s">
+        <v>1422</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="9" t="s">
+        <v>1423</v>
+      </c>
+      <c r="C66" t="s">
+        <v>1430</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" s="9" t="s">
+        <v>1424</v>
+      </c>
+      <c r="C67" t="s">
+        <v>1426</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" s="9" t="s">
+        <v>1427</v>
+      </c>
+      <c r="C68" t="s">
+        <v>1429</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" s="9" t="s">
+        <v>1428</v>
+      </c>
+      <c r="C69" t="s">
+        <v>1425</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" s="9" t="s">
+        <v>1431</v>
+      </c>
+      <c r="C70" t="s">
+        <v>1432</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" s="9" t="s">
+        <v>1433</v>
+      </c>
+      <c r="C71" t="s">
+        <v>1434</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" s="9" t="s">
+        <v>1435</v>
+      </c>
+      <c r="C72" t="s">
+        <v>1438</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" s="9" t="s">
+        <v>1436</v>
+      </c>
+      <c r="C73" t="s">
+        <v>1437</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>1441</v>
+      </c>
+      <c r="C74" t="s">
+        <v>1447</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>1442</v>
+      </c>
+      <c r="C75" t="s">
+        <v>1444</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>1443</v>
+      </c>
+      <c r="C76" t="s">
+        <v>1445</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>1472</v>
+      </c>
+      <c r="C77" t="s">
+        <v>1446</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>1473</v>
+      </c>
+      <c r="C78" t="s">
+        <v>1448</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>1474</v>
+      </c>
+      <c r="C79" t="s">
+        <v>1450</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>1476</v>
+      </c>
+      <c r="C80" t="s">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>1477</v>
+      </c>
+      <c r="C81" t="s">
+        <v>1451</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>1478</v>
+      </c>
+      <c r="C82" t="s">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>1479</v>
+      </c>
+      <c r="C83" t="s">
+        <v>1507</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>1480</v>
+      </c>
+      <c r="C84" t="s">
+        <v>1449</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>1481</v>
+      </c>
+      <c r="C85" t="s">
+        <v>1452</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>1482</v>
+      </c>
+      <c r="C86" t="s">
+        <v>1453</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>1483</v>
+      </c>
+      <c r="C87" t="s">
+        <v>1454</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>1484</v>
+      </c>
+      <c r="C88" t="s">
+        <v>1455</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>1485</v>
+      </c>
+      <c r="C89" t="s">
+        <v>1456</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>1486</v>
+      </c>
+      <c r="C90" t="s">
+        <v>1457</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>1487</v>
+      </c>
+      <c r="C91" t="s">
+        <v>1458</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>1488</v>
+      </c>
+      <c r="C92" t="s">
+        <v>1459</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>1489</v>
+      </c>
+      <c r="C93" t="s">
+        <v>1460</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>1490</v>
+      </c>
+      <c r="C94" t="s">
+        <v>1462</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>1491</v>
+      </c>
+      <c r="C95" t="s">
+        <v>1461</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>1492</v>
+      </c>
+      <c r="C96" t="s">
+        <v>1463</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>1493</v>
+      </c>
+      <c r="C97" t="s">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>1494</v>
+      </c>
+      <c r="C98" t="s">
+        <v>1465</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>1495</v>
+      </c>
+      <c r="C99" t="s">
+        <v>1466</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>1504</v>
+      </c>
+      <c r="C100" t="s">
+        <v>1467</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>1497</v>
+      </c>
+      <c r="C101" t="s">
+        <v>1505</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>1498</v>
+      </c>
+      <c r="C102" t="s">
+        <v>1496</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>1499</v>
+      </c>
+      <c r="C103" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>1500</v>
+      </c>
+      <c r="C104" t="s">
+        <v>1469</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>1501</v>
+      </c>
+      <c r="C105" t="s">
+        <v>1470</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>1502</v>
+      </c>
+      <c r="C106" t="s">
+        <v>1596</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>1503</v>
+      </c>
+      <c r="C107" t="s">
+        <v>1471</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>1530</v>
+      </c>
+      <c r="C108" t="s">
+        <v>1508</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>1520</v>
+      </c>
+      <c r="C109" t="s">
+        <v>1430</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>1521</v>
+      </c>
+      <c r="C110" t="s">
+        <v>1509</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>1522</v>
+      </c>
+      <c r="C111" t="s">
+        <v>1511</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>1523</v>
+      </c>
+      <c r="C112" t="s">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>1524</v>
+      </c>
+      <c r="C113" t="s">
+        <v>1512</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>1525</v>
+      </c>
+      <c r="C114" t="s">
+        <v>1531</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>1519</v>
+      </c>
+      <c r="C115" t="s">
+        <v>1513</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>1526</v>
+      </c>
+      <c r="C116" t="s">
+        <v>1594</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>1527</v>
+      </c>
+      <c r="C117" t="s">
+        <v>1595</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>1528</v>
+      </c>
+      <c r="C118" t="s">
+        <v>1514</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>1529</v>
+      </c>
+      <c r="C119" t="s">
+        <v>1532</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>1518</v>
+      </c>
+      <c r="C120" t="s">
+        <v>1515</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>1533</v>
+      </c>
+      <c r="C121" t="s">
+        <v>1516</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C122" t="s">
+        <v>1536</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>1535</v>
+      </c>
+      <c r="C123" t="s">
+        <v>1517</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>1537</v>
+      </c>
+      <c r="C124" t="s">
+        <v>1538</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>1540</v>
+      </c>
+      <c r="C125" t="s">
+        <v>1430</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>1541</v>
+      </c>
+      <c r="C126" t="s">
+        <v>1515</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>1539</v>
+      </c>
+      <c r="C127" t="s">
+        <v>1593</v>
+      </c>
+    </row>
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>1549</v>
+      </c>
+      <c r="C128" t="s">
+        <v>1542</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>1550</v>
+      </c>
+      <c r="C129" t="s">
+        <v>1543</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>1551</v>
+      </c>
+      <c r="C130" t="s">
+        <v>1544</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>1552</v>
+      </c>
+      <c r="C131" t="s">
+        <v>1545</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>1553</v>
+      </c>
+      <c r="C132" t="s">
+        <v>1546</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>1554</v>
+      </c>
+      <c r="C133" t="s">
+        <v>1547</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>1555</v>
+      </c>
+      <c r="C134" t="s">
+        <v>1548</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>1565</v>
+      </c>
+      <c r="C135" t="s">
+        <v>1556</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>1566</v>
+      </c>
+      <c r="C136" t="s">
+        <v>1557</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>1567</v>
+      </c>
+      <c r="C137" t="s">
+        <v>1558</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>1568</v>
+      </c>
+      <c r="C138" t="s">
+        <v>1559</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>1569</v>
+      </c>
+      <c r="C139" t="s">
+        <v>1560</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>1570</v>
+      </c>
+      <c r="C140" t="s">
+        <v>1561</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>1571</v>
+      </c>
+      <c r="C141" t="s">
+        <v>1562</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>1572</v>
+      </c>
+      <c r="C142" t="s">
+        <v>1563</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>1573</v>
+      </c>
+      <c r="C143" t="s">
+        <v>1564</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>1582</v>
+      </c>
+      <c r="C144" t="s">
+        <v>1592</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>1584</v>
+      </c>
+      <c r="C145" t="s">
+        <v>1577</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>1583</v>
+      </c>
+      <c r="C146" t="s">
+        <v>1578</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>1585</v>
+      </c>
+      <c r="C147" t="s">
+        <v>1590</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>1586</v>
+      </c>
+      <c r="C148" t="s">
+        <v>1579</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>1587</v>
+      </c>
+      <c r="C149" t="s">
+        <v>1580</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>1588</v>
+      </c>
+      <c r="C150" t="s">
+        <v>1591</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>1589</v>
+      </c>
+      <c r="C151" t="s">
+        <v>1581</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A152" s="5" t="s">
+        <v>1600</v>
+      </c>
+      <c r="C152" t="s">
+        <v>1598</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A153" s="5" t="s">
+        <v>1601</v>
+      </c>
+      <c r="C153" t="s">
+        <v>1599</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A154" s="5" t="s">
+        <v>1602</v>
+      </c>
+      <c r="C154" t="s">
+        <v>1604</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A155" s="5" t="s">
+        <v>1603</v>
+      </c>
+      <c r="C155" t="s">
+        <v>1605</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>1608</v>
+      </c>
+      <c r="C156" t="s">
+        <v>1613</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>1609</v>
+      </c>
+      <c r="C157" t="s">
+        <v>1606</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>1610</v>
+      </c>
+      <c r="C158" t="s">
+        <v>1607</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>1611</v>
+      </c>
+      <c r="C159" t="s">
+        <v>1795</v>
+      </c>
+    </row>
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>1612</v>
+      </c>
+      <c r="C160" t="s">
+        <v>1819</v>
+      </c>
+    </row>
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>1798</v>
+      </c>
+      <c r="C161" t="s">
+        <v>1796</v>
+      </c>
+    </row>
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>1799</v>
+      </c>
+      <c r="C162" t="s">
+        <v>1820</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>1800</v>
+      </c>
+      <c r="C163" t="s">
+        <v>1797</v>
+      </c>
+    </row>
+    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>1655</v>
+      </c>
+      <c r="C164" s="5" t="s">
+        <v>1631</v>
+      </c>
+    </row>
+    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>1641</v>
+      </c>
+      <c r="C165" t="s">
+        <v>1632</v>
+      </c>
+    </row>
+    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>1642</v>
+      </c>
+      <c r="C166" t="s">
+        <v>1671</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>1643</v>
+      </c>
+      <c r="C167" t="s">
+        <v>1615</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>1644</v>
+      </c>
+      <c r="C168" t="s">
+        <v>1633</v>
+      </c>
+    </row>
+    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>1645</v>
+      </c>
+      <c r="C169" t="s">
+        <v>1616</v>
+      </c>
+    </row>
+    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>1646</v>
+      </c>
+      <c r="C170" t="s">
+        <v>1672</v>
+      </c>
+    </row>
+    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>1647</v>
+      </c>
+      <c r="C171" t="s">
+        <v>1617</v>
+      </c>
+    </row>
+    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>1648</v>
+      </c>
+      <c r="C172" t="s">
+        <v>1618</v>
+      </c>
+    </row>
+    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>1649</v>
+      </c>
+      <c r="C173" t="s">
+        <v>1634</v>
+      </c>
+    </row>
+    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>1650</v>
+      </c>
+      <c r="C174" t="s">
+        <v>1635</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>1651</v>
+      </c>
+      <c r="C175" t="s">
+        <v>1619</v>
+      </c>
+    </row>
+    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>1652</v>
+      </c>
+      <c r="C176" t="s">
+        <v>1620</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>1653</v>
+      </c>
+      <c r="C177" t="s">
+        <v>1674</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>1654</v>
+      </c>
+      <c r="C178" s="5" t="s">
+        <v>1673</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>1657</v>
+      </c>
+      <c r="C179" t="s">
+        <v>1627</v>
+      </c>
+    </row>
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>1656</v>
+      </c>
+      <c r="C180" t="s">
+        <v>1669</v>
+      </c>
+    </row>
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>1658</v>
+      </c>
+      <c r="C181" t="s">
+        <v>1621</v>
+      </c>
+    </row>
+    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>1659</v>
+      </c>
+      <c r="C182" t="s">
+        <v>1670</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>1660</v>
+      </c>
+      <c r="C183" t="s">
+        <v>1622</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>1661</v>
+      </c>
+      <c r="C184" t="s">
+        <v>1628</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>1662</v>
+      </c>
+      <c r="C185" t="s">
+        <v>1623</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>1663</v>
+      </c>
+      <c r="C186" t="s">
+        <v>1624</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A187" t="s">
+        <v>1664</v>
+      </c>
+      <c r="C187" t="s">
+        <v>1629</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>1665</v>
+      </c>
+      <c r="C188" t="s">
+        <v>1625</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>1666</v>
+      </c>
+      <c r="C189" t="s">
+        <v>1626</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>1667</v>
+      </c>
+      <c r="C190" t="s">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
+        <v>1636</v>
+      </c>
+      <c r="C191" t="s">
+        <v>1668</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>1637</v>
+      </c>
+      <c r="C192" t="s">
+        <v>1639</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
+        <v>1638</v>
+      </c>
+      <c r="C193" t="s">
+        <v>1640</v>
+      </c>
+    </row>
+    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A194" t="s">
+        <v>1681</v>
+      </c>
+      <c r="C194" t="s">
+        <v>1675</v>
+      </c>
+    </row>
+    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A195" t="s">
+        <v>1682</v>
+      </c>
+      <c r="C195" t="s">
+        <v>1676</v>
+      </c>
+    </row>
+    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
+        <v>1683</v>
+      </c>
+      <c r="C196" t="s">
+        <v>1677</v>
+      </c>
+    </row>
+    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>1684</v>
+      </c>
+      <c r="C197" t="s">
+        <v>1678</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
+        <v>1685</v>
+      </c>
+      <c r="C198" t="s">
+        <v>1679</v>
+      </c>
+    </row>
+    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A199" t="s">
+        <v>1686</v>
+      </c>
+      <c r="C199" t="s">
+        <v>1680</v>
+      </c>
+    </row>
+    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
+        <v>1693</v>
+      </c>
+      <c r="C200" t="s">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>1694</v>
+      </c>
+      <c r="C201" t="s">
+        <v>1687</v>
+      </c>
+    </row>
+    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>1695</v>
+      </c>
+      <c r="C202" t="s">
+        <v>1688</v>
+      </c>
+    </row>
+    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>1696</v>
+      </c>
+      <c r="C203" t="s">
+        <v>1691</v>
+      </c>
+    </row>
+    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
+        <v>1697</v>
+      </c>
+      <c r="C204" t="s">
+        <v>1689</v>
+      </c>
+    </row>
+    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A205" t="s">
+        <v>1698</v>
+      </c>
+      <c r="C205" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A206" t="s">
+        <v>1709</v>
+      </c>
+      <c r="C206" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A207" t="s">
+        <v>1704</v>
+      </c>
+      <c r="C207" t="s">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A208" t="s">
+        <v>1705</v>
+      </c>
+      <c r="C208" t="s">
+        <v>1701</v>
+      </c>
+    </row>
+    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
+        <v>1706</v>
+      </c>
+      <c r="C209" t="s">
+        <v>1702</v>
+      </c>
+    </row>
+    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A210" t="s">
+        <v>1707</v>
+      </c>
+      <c r="C210" t="s">
+        <v>1710</v>
+      </c>
+    </row>
+    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A211" t="s">
+        <v>1708</v>
+      </c>
+      <c r="C211" t="s">
+        <v>1703</v>
+      </c>
+    </row>
+    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A212" t="s">
+        <v>1716</v>
+      </c>
+      <c r="C212" t="s">
+        <v>1712</v>
+      </c>
+    </row>
+    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A213" t="s">
+        <v>1717</v>
+      </c>
+      <c r="C213" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A214" t="s">
+        <v>1718</v>
+      </c>
+      <c r="C214" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A215" t="s">
+        <v>1719</v>
+      </c>
+      <c r="C215" t="s">
+        <v>1713</v>
+      </c>
+    </row>
+    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
+        <v>1720</v>
+      </c>
+      <c r="C216" t="s">
+        <v>1715</v>
+      </c>
+    </row>
+    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A217" t="s">
+        <v>1745</v>
+      </c>
+      <c r="C217" t="s">
+        <v>1721</v>
+      </c>
+    </row>
+    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A218" t="s">
+        <v>1751</v>
+      </c>
+      <c r="C218" t="s">
+        <v>1722</v>
+      </c>
+    </row>
+    <row r="219" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
+        <v>1752</v>
+      </c>
+      <c r="C219" t="s">
+        <v>1724</v>
+      </c>
+    </row>
+    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
+        <v>1753</v>
+      </c>
+      <c r="C220" t="s">
+        <v>1723</v>
+      </c>
+    </row>
+    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
+        <v>1754</v>
+      </c>
+      <c r="C221" t="s">
+        <v>1725</v>
+      </c>
+    </row>
+    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A222" t="s">
+        <v>1755</v>
+      </c>
+      <c r="C222" t="s">
+        <v>1779</v>
+      </c>
+    </row>
+    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A223" t="s">
+        <v>1756</v>
+      </c>
+      <c r="C223" t="s">
+        <v>1726</v>
+      </c>
+    </row>
+    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A224" t="s">
+        <v>1746</v>
+      </c>
+      <c r="C224" s="5" t="s">
+        <v>1727</v>
+      </c>
+    </row>
+    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A225" t="s">
+        <v>1757</v>
+      </c>
+      <c r="C225" t="s">
+        <v>1729</v>
+      </c>
+    </row>
+    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A226" t="s">
+        <v>1758</v>
+      </c>
+      <c r="C226" t="s">
+        <v>1730</v>
+      </c>
+    </row>
+    <row r="227" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A227" t="s">
+        <v>1759</v>
+      </c>
+      <c r="C227" t="s">
+        <v>1732</v>
+      </c>
+    </row>
+    <row r="228" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A228" t="s">
+        <v>1760</v>
+      </c>
+      <c r="C228" t="s">
+        <v>1731</v>
+      </c>
+    </row>
+    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A229" t="s">
+        <v>1761</v>
+      </c>
+      <c r="C229" t="s">
+        <v>1733</v>
+      </c>
+    </row>
+    <row r="230" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A230" t="s">
+        <v>1762</v>
+      </c>
+      <c r="C230" t="s">
+        <v>1734</v>
+      </c>
+    </row>
+    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A231" t="s">
+        <v>1763</v>
+      </c>
+      <c r="C231" t="s">
+        <v>1783</v>
+      </c>
+    </row>
+    <row r="232" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A232" t="s">
+        <v>1764</v>
+      </c>
+      <c r="C232" t="s">
+        <v>1735</v>
+      </c>
+    </row>
+    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A233" t="s">
+        <v>1765</v>
+      </c>
+      <c r="C233" t="s">
+        <v>1782</v>
+      </c>
+    </row>
+    <row r="234" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A234" t="s">
+        <v>1766</v>
+      </c>
+      <c r="C234" t="s">
+        <v>1781</v>
+      </c>
+    </row>
+    <row r="235" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A235" t="s">
+        <v>1767</v>
+      </c>
+      <c r="C235" t="s">
+        <v>1737</v>
+      </c>
+    </row>
+    <row r="236" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A236" t="s">
+        <v>1768</v>
+      </c>
+      <c r="C236" t="s">
+        <v>1784</v>
+      </c>
+    </row>
+    <row r="237" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A237" t="s">
+        <v>1769</v>
+      </c>
+      <c r="C237" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="238" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A238" t="s">
+        <v>1770</v>
+      </c>
+      <c r="C238" t="s">
+        <v>1736</v>
+      </c>
+    </row>
+    <row r="239" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A239" t="s">
+        <v>1786</v>
+      </c>
+      <c r="C239" t="s">
+        <v>1728</v>
+      </c>
+    </row>
+    <row r="240" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A240" t="s">
+        <v>1747</v>
+      </c>
+      <c r="C240" t="s">
+        <v>1748</v>
+      </c>
+    </row>
+    <row r="241" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A241" t="s">
+        <v>1771</v>
+      </c>
+      <c r="C241" t="s">
+        <v>1738</v>
+      </c>
+    </row>
+    <row r="242" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A242" t="s">
+        <v>1772</v>
+      </c>
+      <c r="C242" t="s">
+        <v>1739</v>
+      </c>
+    </row>
+    <row r="243" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A243" t="s">
+        <v>1773</v>
+      </c>
+      <c r="C243" t="s">
+        <v>1740</v>
+      </c>
+    </row>
+    <row r="244" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A244" t="s">
+        <v>1774</v>
+      </c>
+      <c r="C244" t="s">
+        <v>1780</v>
+      </c>
+    </row>
+    <row r="245" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A245" t="s">
+        <v>1775</v>
+      </c>
+      <c r="C245" t="s">
+        <v>1741</v>
+      </c>
+    </row>
+    <row r="246" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A246" t="s">
+        <v>1776</v>
+      </c>
+      <c r="C246" t="s">
+        <v>1742</v>
+      </c>
+    </row>
+    <row r="247" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A247" t="s">
+        <v>1777</v>
+      </c>
+      <c r="C247" t="s">
+        <v>1743</v>
+      </c>
+    </row>
+    <row r="248" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A248" t="s">
+        <v>1778</v>
+      </c>
+      <c r="C248" t="s">
+        <v>1744</v>
+      </c>
+    </row>
+    <row r="249" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A249" t="s">
+        <v>1750</v>
+      </c>
+      <c r="C249" t="s">
+        <v>1749</v>
+      </c>
+    </row>
+    <row r="250" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A250" t="s">
+        <v>1790</v>
+      </c>
+      <c r="C250" t="s">
+        <v>1789</v>
+      </c>
+    </row>
+    <row r="251" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A251" t="s">
+        <v>1791</v>
+      </c>
+      <c r="C251" t="s">
+        <v>1787</v>
+      </c>
+    </row>
+    <row r="252" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A252" t="s">
+        <v>1792</v>
+      </c>
+      <c r="C252" t="s">
+        <v>1788</v>
+      </c>
+    </row>
+    <row r="253" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A253" t="s">
+        <v>1794</v>
+      </c>
+      <c r="C253" t="s">
+        <v>1793</v>
+      </c>
+    </row>
+    <row r="254" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A254" t="s">
+        <v>1809</v>
+      </c>
+      <c r="C254" t="s">
+        <v>1806</v>
+      </c>
+    </row>
+    <row r="255" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A255" t="s">
+        <v>1810</v>
+      </c>
+      <c r="C255" t="s">
+        <v>1801</v>
+      </c>
+    </row>
+    <row r="256" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A256" t="s">
+        <v>1811</v>
+      </c>
+      <c r="C256" t="s">
+        <v>1802</v>
+      </c>
+    </row>
+    <row r="257" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A257" t="s">
+        <v>1812</v>
+      </c>
+      <c r="C257" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="258" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A258" t="s">
+        <v>1813</v>
+      </c>
+      <c r="C258" t="s">
+        <v>1807</v>
+      </c>
+    </row>
+    <row r="259" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A259" t="s">
+        <v>1814</v>
+      </c>
+      <c r="C259" t="s">
+        <v>1803</v>
+      </c>
+    </row>
+    <row r="260" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A260" t="s">
+        <v>1815</v>
+      </c>
+      <c r="C260" t="s">
+        <v>1808</v>
+      </c>
+    </row>
+    <row r="261" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A261" t="s">
+        <v>1816</v>
+      </c>
+      <c r="C261" t="s">
+        <v>1804</v>
+      </c>
+    </row>
+    <row r="262" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A262" t="s">
+        <v>1817</v>
+      </c>
+      <c r="C262" t="s">
+        <v>1805</v>
       </c>
     </row>
   </sheetData>
@@ -9126,7 +12012,7 @@
         <v>466</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
@@ -9561,29 +12447,29 @@
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
+        <v>1246</v>
+      </c>
+      <c r="B173" t="s">
         <v>1247</v>
       </c>
-      <c r="B173" t="s">
+      <c r="C173" t="s">
         <v>1248</v>
-      </c>
-      <c r="C173" t="s">
-        <v>1249</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
       <c r="B174" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="C174" t="s">
-        <v>1250</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
       <c r="B175" t="s">
         <v>78</v>
@@ -9663,10 +12549,10 @@
         <v>832</v>
       </c>
       <c r="B182" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
       <c r="C182" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
@@ -10326,220 +13212,228 @@
         <v>1242</v>
       </c>
       <c r="C242" t="s">
-        <v>1243</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
+        <v>1253</v>
+      </c>
+      <c r="B243" t="s">
+        <v>1255</v>
+      </c>
+      <c r="C243" t="s">
         <v>1254</v>
-      </c>
-      <c r="B243" t="s">
-        <v>1256</v>
-      </c>
-      <c r="C243" t="s">
-        <v>1255</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
+        <v>1259</v>
+      </c>
+      <c r="B244" t="s">
         <v>1260</v>
       </c>
-      <c r="B244" t="s">
+      <c r="C244" t="s">
         <v>1261</v>
-      </c>
-      <c r="C244" t="s">
-        <v>1262</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
+        <v>1331</v>
+      </c>
+      <c r="B245" t="s">
+        <v>1333</v>
+      </c>
+      <c r="C245" t="s">
         <v>1332</v>
-      </c>
-      <c r="B245" t="s">
-        <v>1334</v>
-      </c>
-      <c r="C245" t="s">
-        <v>1333</v>
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B246" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="C246" t="s">
-        <v>1341</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
+        <v>1335</v>
+      </c>
+      <c r="B247" t="s">
+        <v>1338</v>
+      </c>
+      <c r="C247" t="s">
         <v>1336</v>
-      </c>
-      <c r="B247" t="s">
-        <v>1339</v>
-      </c>
-      <c r="C247" t="s">
-        <v>1337</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>1340</v>
+        <v>1339</v>
       </c>
       <c r="B248" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="C248" t="s">
-        <v>1342</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
+        <v>1342</v>
+      </c>
+      <c r="B249" t="s">
+        <v>1345</v>
+      </c>
+      <c r="C249" t="s">
         <v>1343</v>
-      </c>
-      <c r="B249" t="s">
-        <v>1346</v>
-      </c>
-      <c r="C249" t="s">
-        <v>1344</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
+        <v>1346</v>
+      </c>
+      <c r="B250" t="s">
+        <v>1349</v>
+      </c>
+      <c r="C250" t="s">
         <v>1347</v>
-      </c>
-      <c r="B250" t="s">
-        <v>1350</v>
-      </c>
-      <c r="C250" t="s">
-        <v>1348</v>
       </c>
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>1352</v>
+        <v>1351</v>
       </c>
       <c r="B251" t="s">
-        <v>1351</v>
+        <v>1350</v>
       </c>
       <c r="C251" t="s">
-        <v>1349</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>1353</v>
+        <v>1352</v>
       </c>
       <c r="B252" t="s">
-        <v>1357</v>
+        <v>1356</v>
       </c>
       <c r="C252" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>1354</v>
+        <v>1353</v>
       </c>
       <c r="B253" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="C253" t="s">
-        <v>1356</v>
+        <v>1355</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>1359</v>
+        <v>1358</v>
       </c>
       <c r="B254" t="s">
-        <v>1363</v>
+        <v>1362</v>
       </c>
       <c r="C254" t="s">
-        <v>1361</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>1360</v>
+        <v>1359</v>
       </c>
       <c r="B255" t="s">
-        <v>1364</v>
+        <v>1363</v>
       </c>
       <c r="C255" t="s">
-        <v>1362</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>1365</v>
+        <v>1364</v>
       </c>
       <c r="B256" t="s">
-        <v>1367</v>
+        <v>1366</v>
       </c>
       <c r="C256" t="s">
-        <v>1382</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
+        <v>1367</v>
+      </c>
+      <c r="B257" t="s">
         <v>1368</v>
       </c>
-      <c r="B257" t="s">
-        <v>1369</v>
-      </c>
       <c r="C257" t="s">
-        <v>1366</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>1370</v>
+        <v>1369</v>
       </c>
       <c r="B258" t="s">
-        <v>1374</v>
+        <v>1373</v>
       </c>
       <c r="C258" t="s">
-        <v>1372</v>
+        <v>1371</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>1371</v>
+        <v>1370</v>
       </c>
       <c r="B259" t="s">
-        <v>1375</v>
+        <v>1374</v>
       </c>
       <c r="C259" t="s">
-        <v>1373</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>1376</v>
+        <v>1375</v>
       </c>
       <c r="B260" t="s">
-        <v>1380</v>
+        <v>1379</v>
       </c>
       <c r="C260" t="s">
-        <v>1379</v>
+        <v>1378</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
+        <v>1376</v>
+      </c>
+      <c r="B261" t="s">
+        <v>1380</v>
+      </c>
+      <c r="C261" s="8" t="s">
         <v>1377</v>
       </c>
-      <c r="B261" t="s">
-        <v>1381</v>
-      </c>
-      <c r="C261" s="8" t="s">
-        <v>1378</v>
-      </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C262" s="8"/>
+      <c r="A262" t="s">
+        <v>1574</v>
+      </c>
+      <c r="B262" t="s">
+        <v>1575</v>
+      </c>
+      <c r="C262" t="s">
+        <v>1576</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:A183"/>
@@ -10582,7 +13476,7 @@
         <v>845</v>
       </c>
       <c r="C3" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -10598,7 +13492,7 @@
         <v>846</v>
       </c>
       <c r="C5" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -10614,7 +13508,7 @@
         <v>847</v>
       </c>
       <c r="C7" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -10622,7 +13516,7 @@
         <v>848</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -10630,7 +13524,7 @@
         <v>849</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -10638,7 +13532,7 @@
         <v>850</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -10646,7 +13540,7 @@
         <v>851</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -10654,7 +13548,7 @@
         <v>852</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -10662,7 +13556,7 @@
         <v>853</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -10670,7 +13564,7 @@
         <v>855</v>
       </c>
       <c r="C14" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -10678,7 +13572,7 @@
         <v>856</v>
       </c>
       <c r="C15" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -10686,7 +13580,7 @@
         <v>857</v>
       </c>
       <c r="C16" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -10694,7 +13588,7 @@
         <v>858</v>
       </c>
       <c r="C17" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -10702,7 +13596,7 @@
         <v>859</v>
       </c>
       <c r="C18" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -10710,7 +13604,7 @@
         <v>860</v>
       </c>
       <c r="C19" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -10718,7 +13612,7 @@
         <v>861</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -10726,7 +13620,7 @@
         <v>862</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -10734,15 +13628,15 @@
         <v>863</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>1384</v>
+        <v>1383</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
@@ -10750,15 +13644,15 @@
         <v>864</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -10766,7 +13660,7 @@
         <v>865</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
@@ -10774,7 +13668,7 @@
         <v>866</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
@@ -10782,7 +13676,7 @@
         <v>867</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
@@ -10790,7 +13684,7 @@
         <v>868</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -10798,7 +13692,7 @@
         <v>869</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -10806,7 +13700,7 @@
         <v>870</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
@@ -10814,7 +13708,7 @@
         <v>871</v>
       </c>
       <c r="C32" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
@@ -10822,7 +13716,7 @@
         <v>872</v>
       </c>
       <c r="C33" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -10830,7 +13724,7 @@
         <v>873</v>
       </c>
       <c r="C34" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -10838,7 +13732,7 @@
         <v>874</v>
       </c>
       <c r="C35" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
@@ -10846,7 +13740,7 @@
         <v>875</v>
       </c>
       <c r="C36" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -10854,7 +13748,7 @@
         <v>876</v>
       </c>
       <c r="C37" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
@@ -10862,7 +13756,7 @@
         <v>877</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>1272</v>
+        <v>1271</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
@@ -10870,7 +13764,7 @@
         <v>878</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -10878,7 +13772,7 @@
         <v>879</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -10886,7 +13780,7 @@
         <v>880</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -10894,7 +13788,7 @@
         <v>881</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>1275</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -10902,7 +13796,7 @@
         <v>882</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -10910,7 +13804,7 @@
         <v>883</v>
       </c>
       <c r="C44" t="s">
-        <v>1265</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
@@ -10918,7 +13812,7 @@
         <v>884</v>
       </c>
       <c r="C45" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -10926,7 +13820,7 @@
         <v>885</v>
       </c>
       <c r="C46" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
@@ -10934,7 +13828,7 @@
         <v>886</v>
       </c>
       <c r="C47" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -10942,7 +13836,7 @@
         <v>887</v>
       </c>
       <c r="C48" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -10950,7 +13844,7 @@
         <v>888</v>
       </c>
       <c r="C49" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -11214,7 +14108,7 @@
         <v>1235</v>
       </c>
       <c r="C82" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
@@ -11222,7 +14116,7 @@
         <v>1236</v>
       </c>
       <c r="C83" s="6" t="s">
-        <v>1269</v>
+        <v>1268</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
@@ -11230,7 +14124,7 @@
         <v>1237</v>
       </c>
       <c r="C84" s="6" t="s">
-        <v>1383</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
@@ -11238,7 +14132,7 @@
         <v>1238</v>
       </c>
       <c r="C85" s="6" t="s">
-        <v>1270</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
@@ -11246,7 +14140,7 @@
         <v>1239</v>
       </c>
       <c r="C86" s="6" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
@@ -11254,7 +14148,7 @@
         <v>1240</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
     </row>
   </sheetData>
@@ -11460,15 +14354,15 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>1256</v>
+      </c>
+      <c r="C24" t="s">
         <v>1257</v>
-      </c>
-      <c r="C24" t="s">
-        <v>1258</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>1259</v>
+        <v>1258</v>
       </c>
       <c r="C25" t="s">
         <v>780</v>

</xml_diff>

<commit_message>
+ make main quest system
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1908" uniqueCount="1821">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2006" uniqueCount="1916">
   <si>
     <t>ID</t>
   </si>
@@ -6670,6 +6670,291 @@
   </si>
   <si>
     <t>Được! Ta sẽ dạy con phép Cân Đẩu Vân. Chỉ cần nhún người sẽ bay xa mười vạn tám ngàn dặm.</t>
+  </si>
+  <si>
+    <t>QL_Chapter_01_Name</t>
+  </si>
+  <si>
+    <t>Q_Chapter_01_Act_01_Name</t>
+  </si>
+  <si>
+    <t>Định Hải Thần Trâm</t>
+  </si>
+  <si>
+    <t>Q_Chapter_01_Act_01_Des</t>
+  </si>
+  <si>
+    <t>Q_Chapter_01_Act_02_Name</t>
+  </si>
+  <si>
+    <t>Q_Chapter_01_Act_02_Des</t>
+  </si>
+  <si>
+    <t>Chương 2 Màn 2</t>
+  </si>
+  <si>
+    <t>Trấn Hải Phục Long</t>
+  </si>
+  <si>
+    <t>S_Chapter_01_Act_01_01_Des</t>
+  </si>
+  <si>
+    <t>S_Chapter_01_Act_01_02_Des</t>
+  </si>
+  <si>
+    <t>S_Chapter_01_Act_02_01_Des</t>
+  </si>
+  <si>
+    <t>S_Chapter_01_Act_02_02_Des</t>
+  </si>
+  <si>
+    <t>Có Kim Cô Bỏng trong tay, hãy cùng Long Vương xông vào Lõi Vực Thẳm để ngăn chặn kế hoạch của Ngao Bính.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Áp giải Ngao Bính về, hoàn trả Long Châu cho Long Vương. </t>
+  </si>
+  <si>
+    <t>Đông Hải Phong Ba</t>
+  </si>
+  <si>
+    <t>QL_Chapter_02_Name</t>
+  </si>
+  <si>
+    <t>Tề Thiên Đại Thánh</t>
+  </si>
+  <si>
+    <t>STR_QUEST_LOCKED</t>
+  </si>
+  <si>
+    <t>Quest Locked</t>
+  </si>
+  <si>
+    <t>Nhiệm vụ chưa mở</t>
+  </si>
+  <si>
+    <t>Biển Đông bỗng dưng nổi sóng dữ, những luồng ma Khí màu tím thẫm xé rách đáy biển, cuồn cuộn dâng lên như những vòi quỷ khổng lồ. Hãy xuống Long Cung thăm hỏi lão Long Vương xem đã xảy ra chuyện gì?</t>
+  </si>
+  <si>
+    <t>Đại Thánh! Ngài đến rồi! | Xin hãy cứu lấy Đông Hải!| Ma khí từ Vực Thẫm Cổ Ma bỗng nhiên bùng phát, kéo theo hàng vạn thủy tộc tha hóa… Long Cung sắp không trụ nổi nữa rồi!</t>
+  </si>
+  <si>
+    <t>Ra tay giúp đỡ</t>
+  </si>
+  <si>
+    <t>Lão Long Vương, ta với ông cũng là chỗ hàng xóm lâu năm việc này để Lão Tôn giúp. | Mà sao phong ấn Ma Cổ ngàn năm nay kiên cố, sao tự nhiên bị phá vỡ được.</t>
+  </si>
+  <si>
+    <t>Ngài có manh mối gì không?</t>
+  </si>
+  <si>
+    <t>Đây... đây là Xích Lân Ma Vảy! Loại vảy cá cứng như thép, tỏa ra hỏa ma khí này chỉ có ở một kẻ... Linh Cảm Đại Vương ở Thông Thiên Hà!</t>
+  </si>
+  <si>
+    <t>Linh Cảm Đại Vương? | Tên quái ngư đó vốn tu hành ở vùng nước ngọt, sao tự dưng lại mò xuống đáy đại dương làm chuyện trộm long tráo phụng thế này?</t>
+  </si>
+  <si>
+    <t>Nếu Long Châu rơi vào tay hắn, Cổ Ma sẽ hoàn toàn thoát cấm!</t>
+  </si>
+  <si>
+    <t>Được! Để ta kiếm con Yêu Cá này để hỏi tội nó.</t>
+  </si>
+  <si>
+    <t>Truy bắt Linh Cảm Đại Vương ở khu vực Rạn San Hô Đỏ dưới Đông Hải.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đại Thánh xin tha mạng! </t>
+  </si>
+  <si>
+    <t>Con cá thối nhà ngươi gan to bằng trời! Dám ăn trộm Long Châu phá bỏ phong ấn Ma Cổ. | Mau giao Đông Hải Long Châu ra, bằng không ta sẽ lột sạch vẩy cá trên người ngươi ra.</t>
+  </si>
+  <si>
+    <t>Chưa! Nhưng ta bắn đắt được con cá thối này cho ngài. | Hắn ta khai Ngao Bính là kẻ đứng sau chủ mưu cho toàn bộ việc này.</t>
+  </si>
+  <si>
+    <t>Trời đất ơi! Nghịch tử! Sao ta có đứa con mê muội đến mức này!</t>
+  </si>
+  <si>
+    <t>Vậy chúng ta hãy mau tiến vào Lõi Vực Thẫm ngăn chặn tên nghịch tử đó trước khi mọi chuyện quá muộn.</t>
+  </si>
+  <si>
+    <t>Đại Thanh hãy khoan. Ngao Bính đã hấp thụ sức mạnh từ Ma Cổ giời đây nó đã có sức mạnh cường đại. | Để trấn áp được nó ngài phải có một món binh khí phù hợp. | Chỗ ta có vô vàn món binh khí ngài hãy chọn đấy một món phù hợp. | May đâu mang lên đây.</t>
+  </si>
+  <si>
+    <t>Mấy món này quá nhẹ, có món nào nặng hơn không.</t>
+  </si>
+  <si>
+    <t>Nếu Thượng Tiên vẫn còn chê nhẹ. Chỗ ta còn vật báu bao người khiêng không được. Chỉ sợ ngài không nhấc nổi. | Mời Thượng Tiên xem, đây là khối sắt thần  gọi là Định Hải Thần Trâm dùng để đo mực nước biển.</t>
+  </si>
+  <si>
+    <t>Khối sắt hơi to nếu nhỏ lại một chút thì tuyệt. Ủa, nhỏ thêm nhỏ thêm nữa đi, ngắn lại một chút. |  Ha ha ha. Giời thì vừa tay ta lắm.</t>
+  </si>
+  <si>
+    <t>Thứ lỗi, tại ta phấn khích quá. | Giới ta đã có bảo bối này rồi thì không sợ Ma Cổ nào cả. Hãy mau đi thôi.</t>
+  </si>
+  <si>
+    <t>Từ chối giúp</t>
+  </si>
+  <si>
+    <t>Phong ấn Ma Cổ nào oan cho tôi quá. | Tất cả là do Tam Thái Tử Ngao Bính, hắn hứa với tôi sẽ chia một nửa linh mạch Đông Hải sau khi kế hoạch của hắn hoàn thành. | Tôi tham tài nền mới mù mắt nghe lời hắn!</t>
+  </si>
+  <si>
+    <t>Ngao Bính.. Hóa ra là giặc nhà khó phòng! | Người hãy theo ta về gặp Long Vương để đối chất cho rõ.</t>
+  </si>
+  <si>
+    <t>Đến chỗ Lão Long Vương để làm rõ kẻ chủ mưu đứng âm mưu phá vớ phong ấn giải thoát Ma Cổ.</t>
+  </si>
+  <si>
+    <t>Đại Thánh! Ngài đã tìm được lại Long Châu lại rồi à?</t>
+  </si>
+  <si>
+    <t>Ngao Bính, ngươi mau dừng tay lại trước khi mọi chuyện chưa quá muộn.</t>
+  </si>
+  <si>
+    <t>Môt con khỉ khô sống ở Ha Quả Sơn thì biết gì về đại cục? Thiên Đình đè nén Thủy Tộc bao năm, ta chỉ lấy lại những gì thuôc về Đông Hải.</t>
+  </si>
+  <si>
+    <t>Ta không quan tâm đại cục hay tiểu cục của người. | Nhưng ngươi định thả thứ quái vật Cổ Ma này ra... thì gậy của Lão Tôn không để yên đâu!.</t>
+  </si>
+  <si>
+    <t>Nào! Hãy nhìn cho rõ đi. Thứ sức mạnh này sẽ biến ta thành bá chủ thực sự của đại dương. Ha ha ha.</t>
+  </si>
+  <si>
+    <t>Tên này mất trí rồi. Để ta đánh cho ngươi tỉnh lại. Hãy xem gậy của Lão Tôn đây.</t>
+  </si>
+  <si>
+    <t>Trận chiến đã ngã ngũ. Phong ấn Ma Long hoàn trả lại Long Châu lại cho Lão Long Vương. Đồng thời áp giải Ngao Bính về chịu phạt.</t>
+  </si>
+  <si>
+    <t>Đa tạ Thượng Tiên đã ra tay ngăn cản thằng con nghiệt súc của tiểu thần làm điều dại dột.</t>
+  </si>
+  <si>
+    <t>Giao trả Long Châu.</t>
+  </si>
+  <si>
+    <t>Phong ấn Ma Cổ đã bị bịt kín. Trả lại cho ngài Long Châu. Còn tên Ngao Bính này mong là hắn biết đường hối cải  tránh làm điều ngu dại.</t>
+  </si>
+  <si>
+    <t>Dạ! Cảm tạ Đại Thánh!</t>
+  </si>
+  <si>
+    <t>Vậy không còn việc gì nữa ta về Hoa Quả Sơn của ta đây.</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step01_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step01_Node_Start_Choice_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step01_Node_Start_Choice_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step01_Node_End</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step01_Node_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step01_Node_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step01_Node_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step01_Node_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step01_Node_05</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step01_Node_06</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step01_Node_07</t>
+  </si>
+  <si>
+    <t>S_Chapter_01_Act_01_03_Des</t>
+  </si>
+  <si>
+    <t>Đại Thánh ngài đâu có biết! Trấn Hải Trận Pháp vốn được duy trì là nương tựa vào sức mạnh của Long Châu. | Nhưng không biết kẻ nào đã đánh cắp mất Long Châu?</t>
+  </si>
+  <si>
+    <t>STR_DEFEAT_ENEMY</t>
+  </si>
+  <si>
+    <t>Defeat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đánh bại </t>
+  </si>
+  <si>
+    <t>Tôn... Tôn Ngộ Không?! Ngươi... sao ngươi lại mò tới tận chốn này?</t>
+  </si>
+  <si>
+    <t>Ta tới đây để hỏi tội ngươi vì dám lấy trộm Long Châu của Đông Hải. | Ngươi có biết người đã gây ra họa gì không?</t>
+  </si>
+  <si>
+    <t>Long Châu đã vào tay ta thì là của ta! | Ngươi khôn hồn thì lượn đi, bằng không cặp Trùy này sẽ đập nát cái thân khỉ của ngươi!</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step02_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step02_Node_01</t>
+  </si>
+  <si>
+    <t>Con cá thối nhà ngươi vẫn chưa ăn đòn của ta thì vẫn còn mạnh miệng. Hãy xem bản lĩnh của lão Tôn ta đây.</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step02_Node_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step02_Node_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step02_Complate_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step02_Complate_Node_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step02_Complate_Node_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step02_Complate_Node_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step03_Start_Node_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step03_Start_Node_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step03_Start_Node_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step03_Start_Node_04</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step03_Start_Node_05</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step03_Start_Node_06</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step03_Start_Node_07</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step03_Start_Node_08</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step03_Start_Node_09</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act01_Step03_Node_Start</t>
+  </si>
+  <si>
+    <t>Chúc mừng Thượng Tiên đã tìm bảo bối thần. | Nhưng ngài hãy bớt múa lại được không? Thủy cung của ta rung chuyển, muôn loài thủy tộc hoảng sợ rồi!</t>
   </si>
 </sst>
 </file>
@@ -8421,7 +8706,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C262"/>
+  <dimension ref="A1:C314"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="61.28515625" bestFit="1" customWidth="1"/>
@@ -10558,6 +10843,386 @@
         <v>1800</v>
       </c>
     </row>
+    <row r="263" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A263" t="s">
+        <v>1821</v>
+      </c>
+      <c r="C263" t="s">
+        <v>1835</v>
+      </c>
+    </row>
+    <row r="264" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A264" t="s">
+        <v>1836</v>
+      </c>
+      <c r="C264" t="s">
+        <v>1837</v>
+      </c>
+    </row>
+    <row r="265" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A265" t="s">
+        <v>1822</v>
+      </c>
+      <c r="C265" t="s">
+        <v>1823</v>
+      </c>
+    </row>
+    <row r="266" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A266" t="s">
+        <v>1824</v>
+      </c>
+      <c r="C266" t="s">
+        <v>1384</v>
+      </c>
+    </row>
+    <row r="267" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A267" t="s">
+        <v>1825</v>
+      </c>
+      <c r="C267" t="s">
+        <v>1828</v>
+      </c>
+    </row>
+    <row r="268" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A268" t="s">
+        <v>1826</v>
+      </c>
+      <c r="C268" t="s">
+        <v>1827</v>
+      </c>
+    </row>
+    <row r="269" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A269" t="s">
+        <v>1829</v>
+      </c>
+      <c r="C269" t="s">
+        <v>1841</v>
+      </c>
+    </row>
+    <row r="270" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A270" t="s">
+        <v>1830</v>
+      </c>
+      <c r="C270" t="s">
+        <v>1850</v>
+      </c>
+    </row>
+    <row r="271" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A271" t="s">
+        <v>1888</v>
+      </c>
+      <c r="C271" t="s">
+        <v>1864</v>
+      </c>
+    </row>
+    <row r="272" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A272" t="s">
+        <v>1831</v>
+      </c>
+      <c r="C272" t="s">
+        <v>1833</v>
+      </c>
+    </row>
+    <row r="273" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A273" t="s">
+        <v>1832</v>
+      </c>
+      <c r="C273" t="s">
+        <v>1834</v>
+      </c>
+    </row>
+    <row r="274" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A274" t="s">
+        <v>1877</v>
+      </c>
+      <c r="C274" t="s">
+        <v>1842</v>
+      </c>
+    </row>
+    <row r="275" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A275" t="s">
+        <v>1878</v>
+      </c>
+      <c r="C275" t="s">
+        <v>1843</v>
+      </c>
+    </row>
+    <row r="276" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A276" t="s">
+        <v>1879</v>
+      </c>
+      <c r="C276" t="s">
+        <v>1861</v>
+      </c>
+    </row>
+    <row r="277" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A277" t="s">
+        <v>1880</v>
+      </c>
+      <c r="C277" t="s">
+        <v>1612</v>
+      </c>
+    </row>
+    <row r="278" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A278" t="s">
+        <v>1881</v>
+      </c>
+      <c r="C278" t="s">
+        <v>1844</v>
+      </c>
+    </row>
+    <row r="279" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A279" t="s">
+        <v>1882</v>
+      </c>
+      <c r="C279" t="s">
+        <v>1889</v>
+      </c>
+    </row>
+    <row r="280" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A280" t="s">
+        <v>1883</v>
+      </c>
+      <c r="C280" t="s">
+        <v>1845</v>
+      </c>
+    </row>
+    <row r="281" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A281" t="s">
+        <v>1884</v>
+      </c>
+      <c r="C281" t="s">
+        <v>1846</v>
+      </c>
+    </row>
+    <row r="282" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A282" t="s">
+        <v>1885</v>
+      </c>
+      <c r="C282" t="s">
+        <v>1847</v>
+      </c>
+    </row>
+    <row r="283" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A283" t="s">
+        <v>1886</v>
+      </c>
+      <c r="C283" t="s">
+        <v>1848</v>
+      </c>
+    </row>
+    <row r="284" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A284" t="s">
+        <v>1887</v>
+      </c>
+      <c r="C284" t="s">
+        <v>1849</v>
+      </c>
+    </row>
+    <row r="285" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A285" t="s">
+        <v>1896</v>
+      </c>
+      <c r="C285" t="s">
+        <v>1893</v>
+      </c>
+    </row>
+    <row r="286" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A286" t="s">
+        <v>1897</v>
+      </c>
+      <c r="C286" t="s">
+        <v>1894</v>
+      </c>
+    </row>
+    <row r="287" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A287" t="s">
+        <v>1899</v>
+      </c>
+      <c r="C287" t="s">
+        <v>1895</v>
+      </c>
+    </row>
+    <row r="288" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A288" t="s">
+        <v>1900</v>
+      </c>
+      <c r="C288" t="s">
+        <v>1898</v>
+      </c>
+    </row>
+    <row r="289" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A289" t="s">
+        <v>1901</v>
+      </c>
+      <c r="C289" t="s">
+        <v>1851</v>
+      </c>
+    </row>
+    <row r="290" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A290" t="s">
+        <v>1902</v>
+      </c>
+      <c r="C290" t="s">
+        <v>1852</v>
+      </c>
+    </row>
+    <row r="291" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A291" t="s">
+        <v>1903</v>
+      </c>
+      <c r="C291" t="s">
+        <v>1862</v>
+      </c>
+    </row>
+    <row r="292" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A292" t="s">
+        <v>1904</v>
+      </c>
+      <c r="C292" t="s">
+        <v>1863</v>
+      </c>
+    </row>
+    <row r="293" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A293" t="s">
+        <v>1914</v>
+      </c>
+      <c r="C293" s="5" t="s">
+        <v>1865</v>
+      </c>
+    </row>
+    <row r="294" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A294" t="s">
+        <v>1905</v>
+      </c>
+      <c r="C294" t="s">
+        <v>1853</v>
+      </c>
+    </row>
+    <row r="295" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A295" t="s">
+        <v>1906</v>
+      </c>
+      <c r="C295" t="s">
+        <v>1854</v>
+      </c>
+    </row>
+    <row r="296" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A296" t="s">
+        <v>1907</v>
+      </c>
+      <c r="C296" t="s">
+        <v>1855</v>
+      </c>
+    </row>
+    <row r="297" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A297" t="s">
+        <v>1908</v>
+      </c>
+      <c r="C297" t="s">
+        <v>1856</v>
+      </c>
+    </row>
+    <row r="298" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A298" t="s">
+        <v>1909</v>
+      </c>
+      <c r="C298" t="s">
+        <v>1857</v>
+      </c>
+    </row>
+    <row r="299" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A299" t="s">
+        <v>1910</v>
+      </c>
+      <c r="C299" t="s">
+        <v>1858</v>
+      </c>
+    </row>
+    <row r="300" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A300" t="s">
+        <v>1911</v>
+      </c>
+      <c r="C300" t="s">
+        <v>1859</v>
+      </c>
+    </row>
+    <row r="301" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A301" t="s">
+        <v>1912</v>
+      </c>
+      <c r="C301" t="s">
+        <v>1915</v>
+      </c>
+    </row>
+    <row r="302" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A302" t="s">
+        <v>1913</v>
+      </c>
+      <c r="C302" t="s">
+        <v>1860</v>
+      </c>
+    </row>
+    <row r="303" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C303" t="s">
+        <v>1866</v>
+      </c>
+    </row>
+    <row r="304" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C304" t="s">
+        <v>1867</v>
+      </c>
+    </row>
+    <row r="305" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C305" s="2" t="s">
+        <v>1868</v>
+      </c>
+    </row>
+    <row r="306" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C306" t="s">
+        <v>1869</v>
+      </c>
+    </row>
+    <row r="307" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C307" t="s">
+        <v>1870</v>
+      </c>
+    </row>
+    <row r="308" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C308" t="s">
+        <v>1871</v>
+      </c>
+    </row>
+    <row r="309" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C309" t="s">
+        <v>1872</v>
+      </c>
+    </row>
+    <row r="310" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C310" t="s">
+        <v>1873</v>
+      </c>
+    </row>
+    <row r="311" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C311" t="s">
+        <v>1874</v>
+      </c>
+    </row>
+    <row r="312" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C312" t="s">
+        <v>1875</v>
+      </c>
+    </row>
+    <row r="313" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C313" t="s">
+        <v>1876</v>
+      </c>
+    </row>
+    <row r="314" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C314" t="s">
+        <v>720</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -10566,7 +11231,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C262"/>
+  <dimension ref="A1:C264"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.85546875" bestFit="1" customWidth="1"/>
@@ -12810,629 +13475,651 @@
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>1106</v>
+        <v>1890</v>
       </c>
       <c r="B206" t="s">
-        <v>1107</v>
+        <v>1891</v>
       </c>
       <c r="C206" t="s">
-        <v>1108</v>
+        <v>1892</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
-        <v>1109</v>
+        <v>1106</v>
       </c>
       <c r="B207" t="s">
-        <v>1110</v>
+        <v>1107</v>
       </c>
       <c r="C207" t="s">
-        <v>1111</v>
+        <v>1108</v>
       </c>
     </row>
     <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
-        <v>1115</v>
+        <v>1109</v>
       </c>
       <c r="B208" t="s">
-        <v>1116</v>
+        <v>1110</v>
       </c>
       <c r="C208" t="s">
-        <v>1117</v>
+        <v>1111</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
-        <v>1118</v>
+        <v>1115</v>
       </c>
       <c r="B209" t="s">
-        <v>1120</v>
+        <v>1116</v>
       </c>
       <c r="C209" t="s">
-        <v>1119</v>
+        <v>1117</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
-        <v>1121</v>
+        <v>1118</v>
       </c>
       <c r="B210" t="s">
-        <v>1123</v>
+        <v>1120</v>
       </c>
       <c r="C210" t="s">
-        <v>1122</v>
+        <v>1119</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
-        <v>1124</v>
+        <v>1121</v>
       </c>
       <c r="B211" t="s">
-        <v>1133</v>
+        <v>1123</v>
       </c>
       <c r="C211" t="s">
-        <v>1132</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>1126</v>
+        <v>1124</v>
       </c>
       <c r="B212" t="s">
-        <v>1127</v>
+        <v>1133</v>
       </c>
       <c r="C212" t="s">
-        <v>1203</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
       <c r="B213" t="s">
-        <v>1130</v>
+        <v>1127</v>
       </c>
       <c r="C213" t="s">
-        <v>1129</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>1131</v>
+        <v>1128</v>
       </c>
       <c r="B214" t="s">
-        <v>1125</v>
+        <v>1130</v>
       </c>
       <c r="C214" t="s">
-        <v>1204</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>1134</v>
+        <v>1131</v>
       </c>
       <c r="B215" t="s">
-        <v>1135</v>
+        <v>1125</v>
       </c>
       <c r="C215" t="s">
-        <v>1139</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>1136</v>
+        <v>1134</v>
       </c>
       <c r="B216" t="s">
-        <v>1138</v>
+        <v>1135</v>
       </c>
       <c r="C216" t="s">
-        <v>1137</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>1140</v>
+        <v>1136</v>
       </c>
       <c r="B217" t="s">
-        <v>1142</v>
+        <v>1138</v>
       </c>
       <c r="C217" t="s">
-        <v>1141</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>1143</v>
+        <v>1140</v>
       </c>
       <c r="B218" t="s">
-        <v>1145</v>
+        <v>1142</v>
       </c>
       <c r="C218" t="s">
-        <v>1144</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>1146</v>
+        <v>1143</v>
       </c>
       <c r="B219" t="s">
-        <v>1148</v>
+        <v>1145</v>
       </c>
       <c r="C219" t="s">
-        <v>1147</v>
+        <v>1144</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>1149</v>
+        <v>1146</v>
       </c>
       <c r="B220" t="s">
-        <v>1153</v>
+        <v>1148</v>
       </c>
       <c r="C220" t="s">
-        <v>1152</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="B221" t="s">
-        <v>1155</v>
+        <v>1153</v>
       </c>
       <c r="C221" t="s">
-        <v>1154</v>
+        <v>1152</v>
       </c>
     </row>
     <row r="222" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="B222" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="C222" t="s">
-        <v>1157</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="223" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>1158</v>
+        <v>1151</v>
       </c>
       <c r="B223" t="s">
-        <v>1162</v>
+        <v>1156</v>
       </c>
       <c r="C223" t="s">
-        <v>1161</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="224" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="B224" t="s">
-        <v>1164</v>
+        <v>1162</v>
       </c>
       <c r="C224" t="s">
-        <v>1163</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="225" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="B225" t="s">
-        <v>1166</v>
+        <v>1164</v>
       </c>
       <c r="C225" t="s">
-        <v>1165</v>
+        <v>1163</v>
       </c>
     </row>
     <row r="226" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>1167</v>
+        <v>1160</v>
       </c>
       <c r="B226" t="s">
-        <v>1172</v>
+        <v>1166</v>
       </c>
       <c r="C226" t="s">
-        <v>1170</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="227" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="B227" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C227" t="s">
-        <v>1180</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="228" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="B228" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="C228" t="s">
-        <v>1171</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="229" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>1175</v>
+        <v>1169</v>
       </c>
       <c r="B229" t="s">
-        <v>1185</v>
+        <v>1174</v>
       </c>
       <c r="C229" t="s">
-        <v>1178</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="230" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>1177</v>
+        <v>1175</v>
       </c>
       <c r="B230" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="C230" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
     </row>
     <row r="231" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>1176</v>
+        <v>1177</v>
       </c>
       <c r="B231" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="C231" t="s">
-        <v>1184</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="232" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>1205</v>
+        <v>1176</v>
       </c>
       <c r="B232" t="s">
-        <v>1207</v>
+        <v>1187</v>
       </c>
       <c r="C232" t="s">
-        <v>1206</v>
+        <v>1184</v>
       </c>
     </row>
     <row r="233" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>1208</v>
+        <v>1205</v>
       </c>
       <c r="B233" t="s">
-        <v>1209</v>
+        <v>1207</v>
       </c>
       <c r="C233" t="s">
-        <v>1210</v>
+        <v>1206</v>
       </c>
     </row>
     <row r="234" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>1211</v>
+        <v>1208</v>
       </c>
       <c r="B234" t="s">
-        <v>1212</v>
+        <v>1209</v>
       </c>
       <c r="C234" t="s">
-        <v>1213</v>
+        <v>1210</v>
       </c>
     </row>
     <row r="235" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>1214</v>
+        <v>1211</v>
       </c>
       <c r="B235" t="s">
-        <v>1215</v>
+        <v>1212</v>
       </c>
       <c r="C235" t="s">
-        <v>1216</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="236" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>1217</v>
+        <v>1214</v>
       </c>
       <c r="B236" t="s">
-        <v>1218</v>
+        <v>1215</v>
       </c>
       <c r="C236" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>1223</v>
+        <v>1217</v>
       </c>
       <c r="B237" t="s">
-        <v>1224</v>
+        <v>1218</v>
       </c>
       <c r="C237" t="s">
-        <v>1225</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>1220</v>
+        <v>1223</v>
       </c>
       <c r="B238" t="s">
-        <v>1221</v>
+        <v>1224</v>
       </c>
       <c r="C238" t="s">
-        <v>1222</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="239" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
-        <v>1226</v>
+        <v>1220</v>
       </c>
       <c r="B239" t="s">
-        <v>1227</v>
+        <v>1221</v>
       </c>
       <c r="C239" t="s">
-        <v>1228</v>
+        <v>1222</v>
       </c>
     </row>
     <row r="240" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
-        <v>1231</v>
+        <v>1226</v>
       </c>
       <c r="B240" t="s">
-        <v>1229</v>
+        <v>1227</v>
       </c>
       <c r="C240" t="s">
-        <v>1230</v>
+        <v>1228</v>
       </c>
     </row>
     <row r="241" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
-        <v>1232</v>
+        <v>1231</v>
       </c>
       <c r="B241" t="s">
-        <v>1233</v>
+        <v>1229</v>
       </c>
       <c r="C241" t="s">
-        <v>1234</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="242" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
-        <v>1241</v>
+        <v>1232</v>
       </c>
       <c r="B242" t="s">
-        <v>1242</v>
+        <v>1233</v>
       </c>
       <c r="C242" t="s">
-        <v>1420</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="243" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
-        <v>1253</v>
+        <v>1241</v>
       </c>
       <c r="B243" t="s">
-        <v>1255</v>
+        <v>1242</v>
       </c>
       <c r="C243" t="s">
-        <v>1254</v>
+        <v>1420</v>
       </c>
     </row>
     <row r="244" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
-        <v>1259</v>
+        <v>1253</v>
       </c>
       <c r="B244" t="s">
-        <v>1260</v>
+        <v>1255</v>
       </c>
       <c r="C244" t="s">
-        <v>1261</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="245" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
-        <v>1331</v>
+        <v>1259</v>
       </c>
       <c r="B245" t="s">
-        <v>1333</v>
+        <v>1260</v>
       </c>
       <c r="C245" t="s">
-        <v>1332</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="246" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
-        <v>1334</v>
+        <v>1331</v>
       </c>
       <c r="B246" t="s">
-        <v>1337</v>
+        <v>1333</v>
       </c>
       <c r="C246" t="s">
-        <v>1340</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="247" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B247" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="C247" t="s">
-        <v>1336</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="248" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
-        <v>1339</v>
+        <v>1335</v>
       </c>
       <c r="B248" t="s">
-        <v>1344</v>
+        <v>1338</v>
       </c>
       <c r="C248" t="s">
-        <v>1341</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="249" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
-        <v>1342</v>
+        <v>1339</v>
       </c>
       <c r="B249" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="C249" t="s">
-        <v>1343</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="250" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>1346</v>
+        <v>1342</v>
       </c>
       <c r="B250" t="s">
-        <v>1349</v>
+        <v>1345</v>
       </c>
       <c r="C250" t="s">
-        <v>1347</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="251" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>1351</v>
+        <v>1346</v>
       </c>
       <c r="B251" t="s">
-        <v>1350</v>
+        <v>1349</v>
       </c>
       <c r="C251" t="s">
-        <v>1348</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="252" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>1352</v>
+        <v>1351</v>
       </c>
       <c r="B252" t="s">
-        <v>1356</v>
+        <v>1350</v>
       </c>
       <c r="C252" t="s">
-        <v>1354</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="253" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>1353</v>
+        <v>1352</v>
       </c>
       <c r="B253" t="s">
-        <v>1357</v>
+        <v>1356</v>
       </c>
       <c r="C253" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
     </row>
     <row r="254" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>1358</v>
+        <v>1353</v>
       </c>
       <c r="B254" t="s">
-        <v>1362</v>
+        <v>1357</v>
       </c>
       <c r="C254" t="s">
-        <v>1360</v>
+        <v>1355</v>
       </c>
     </row>
     <row r="255" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>1359</v>
+        <v>1358</v>
       </c>
       <c r="B255" t="s">
-        <v>1363</v>
+        <v>1362</v>
       </c>
       <c r="C255" t="s">
-        <v>1361</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>1364</v>
+        <v>1359</v>
       </c>
       <c r="B256" t="s">
-        <v>1366</v>
+        <v>1363</v>
       </c>
       <c r="C256" t="s">
-        <v>1381</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="257" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>1367</v>
+        <v>1364</v>
       </c>
       <c r="B257" t="s">
-        <v>1368</v>
+        <v>1366</v>
       </c>
       <c r="C257" t="s">
-        <v>1365</v>
+        <v>1381</v>
       </c>
     </row>
     <row r="258" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>1369</v>
+        <v>1367</v>
       </c>
       <c r="B258" t="s">
-        <v>1373</v>
+        <v>1368</v>
       </c>
       <c r="C258" t="s">
-        <v>1371</v>
+        <v>1365</v>
       </c>
     </row>
     <row r="259" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>1370</v>
+        <v>1369</v>
       </c>
       <c r="B259" t="s">
-        <v>1374</v>
+        <v>1373</v>
       </c>
       <c r="C259" t="s">
-        <v>1372</v>
+        <v>1371</v>
       </c>
     </row>
     <row r="260" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>1375</v>
+        <v>1370</v>
       </c>
       <c r="B260" t="s">
-        <v>1379</v>
+        <v>1374</v>
       </c>
       <c r="C260" t="s">
-        <v>1378</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="261" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>1376</v>
+        <v>1375</v>
       </c>
       <c r="B261" t="s">
-        <v>1380</v>
-      </c>
-      <c r="C261" s="8" t="s">
-        <v>1377</v>
+        <v>1379</v>
+      </c>
+      <c r="C261" t="s">
+        <v>1378</v>
       </c>
     </row>
     <row r="262" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
+        <v>1376</v>
+      </c>
+      <c r="B262" t="s">
+        <v>1380</v>
+      </c>
+      <c r="C262" s="8" t="s">
+        <v>1377</v>
+      </c>
+    </row>
+    <row r="263" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A263" t="s">
         <v>1574</v>
       </c>
-      <c r="B262" t="s">
+      <c r="B263" t="s">
         <v>1575</v>
       </c>
-      <c r="C262" t="s">
+      <c r="C263" t="s">
         <v>1576</v>
+      </c>
+    </row>
+    <row r="264" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A264" t="s">
+        <v>1838</v>
+      </c>
+      <c r="B264" t="s">
+        <v>1839</v>
+      </c>
+      <c r="C264" t="s">
+        <v>1840</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
+ Complete Act2 of Chapter01
</commit_message>
<xml_diff>
--- a/Tool/data/Localizations.xlsx
+++ b/Tool/data/Localizations.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="UI" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2006" uniqueCount="1916">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2024" uniqueCount="1934">
   <si>
     <t>ID</t>
   </si>
@@ -6711,9 +6711,6 @@
     <t>Có Kim Cô Bỏng trong tay, hãy cùng Long Vương xông vào Lõi Vực Thẳm để ngăn chặn kế hoạch của Ngao Bính.</t>
   </si>
   <si>
-    <t xml:space="preserve">Áp giải Ngao Bính về, hoàn trả Long Châu cho Long Vương. </t>
-  </si>
-  <si>
     <t>Đông Hải Phong Ba</t>
   </si>
   <si>
@@ -6810,9 +6807,6 @@
     <t>Ngao Bính, ngươi mau dừng tay lại trước khi mọi chuyện chưa quá muộn.</t>
   </si>
   <si>
-    <t>Môt con khỉ khô sống ở Ha Quả Sơn thì biết gì về đại cục? Thiên Đình đè nén Thủy Tộc bao năm, ta chỉ lấy lại những gì thuôc về Đông Hải.</t>
-  </si>
-  <si>
     <t>Ta không quan tâm đại cục hay tiểu cục của người. | Nhưng ngươi định thả thứ quái vật Cổ Ma này ra... thì gậy của Lão Tôn không để yên đâu!.</t>
   </si>
   <si>
@@ -6822,24 +6816,9 @@
     <t>Tên này mất trí rồi. Để ta đánh cho ngươi tỉnh lại. Hãy xem gậy của Lão Tôn đây.</t>
   </si>
   <si>
-    <t>Trận chiến đã ngã ngũ. Phong ấn Ma Long hoàn trả lại Long Châu lại cho Lão Long Vương. Đồng thời áp giải Ngao Bính về chịu phạt.</t>
-  </si>
-  <si>
-    <t>Đa tạ Thượng Tiên đã ra tay ngăn cản thằng con nghiệt súc của tiểu thần làm điều dại dột.</t>
-  </si>
-  <si>
     <t>Giao trả Long Châu.</t>
   </si>
   <si>
-    <t>Phong ấn Ma Cổ đã bị bịt kín. Trả lại cho ngài Long Châu. Còn tên Ngao Bính này mong là hắn biết đường hối cải  tránh làm điều ngu dại.</t>
-  </si>
-  <si>
-    <t>Dạ! Cảm tạ Đại Thánh!</t>
-  </si>
-  <si>
-    <t>Vậy không còn việc gì nữa ta về Hoa Quả Sơn của ta đây.</t>
-  </si>
-  <si>
     <t>STR_DLG_Chapter01_Act01_Step01_Node_Start</t>
   </si>
   <si>
@@ -6955,6 +6934,81 @@
   </si>
   <si>
     <t>Chúc mừng Thượng Tiên đã tìm bảo bối thần. | Nhưng ngài hãy bớt múa lại được không? Thủy cung của ta rung chuyển, muôn loài thủy tộc hoảng sợ rồi!</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act02_Step01_Start_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act02_Step01_Start_Node_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act02_Step01_Start_Node_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act02_Step01_Start_Node_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act02_Step01_Start_Node_04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lão Tôn vốn định cho ngươi một gậy nhưng lại sợ cây gậy này nặng quá đánh chết ngươi. | Nể mặt lão Long Vương, ta sẽ tha cho ngươi một mạng! </t>
+  </si>
+  <si>
+    <t>Nếu không vì kế hoạch cướp Long Châu bị lộ, Ma Long chưa kịp hoàn toàn thoát cấm... thì một con khỉ như ngươi làm sao thắng nổi ta?</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act02_Step01_Complate_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act02_Step01_Complate_Node_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act02_Step01_Complate_Node_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act02_Step01_Complate_Node_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act02_Step02_Node_Start</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act02_Step02_Node_Start_Choice</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act02_Step02_Node_01</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act02_Step02_Node_02</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act02_Step02_Node_03</t>
+  </si>
+  <si>
+    <t>STR_DLG_Chapter01_Act02_Step02_Node_04</t>
+  </si>
+  <si>
+    <t>Trận chiến đã ngã ngũ phong ấn đã được đóng lại, sóng êm biển lặng, ma khí đã tan. Hoàn trả lại Long Châu lại cho Lão Long Vương. áp giải Ngao Bính về chịu phạt.</t>
+  </si>
+  <si>
+    <t>Đại Thánh! Ngài không chỉ cứu lấy Đông Hải, mà còn cứu cả cái mạng cùi của nghịch tử Ngao Bính. | Ơn sâu nghĩa nặng này, Long Cung biết lấy chi đền đáp?</t>
+  </si>
+  <si>
+    <t>Được, được! Thần binh gặp chủ nhân chân chính, đó cũng là thiên ý! Còn ngài... ngài có muốn ở lại dự yến tiệc mừng chiến thắng?</t>
+  </si>
+  <si>
+    <t>Yến tiệc để sau đi! Nơi này xong việc rồi ta về Hoa Quả Sơn của ta đây.</t>
+  </si>
+  <si>
+    <t>Công lao gì đâu. Lão Tôn trước giờ không nợ ai.  Ngài tặng ta món thần khí, ta giúp ngài hai bên hòa nhau!</t>
+  </si>
+  <si>
+    <t>Một con khỉ khô sống ở Hoa Quả Sơn thì biết gì về đại cục? Thiên Đình đè nén Thủy Tộc bao năm, ta chỉ lấy lại những gì thuộc về Đông Hải.</t>
+  </si>
+  <si>
+    <t>Nói nhiều làm gì! Thua thì đã thua rồi, ra tay nhanh đi!</t>
+  </si>
+  <si>
+    <t>Ta không có thời gian đứng đây rảnh rỗi chơi với ngươi! | Càn Khôn Định Vị — Thủy Khí Quy Nguyên! Long Châu Trở Về, Bát Quái Trấn Yêu! | PHONG!</t>
   </si>
 </sst>
 </file>
@@ -8706,7 +8760,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C314"/>
+  <dimension ref="A1:C317"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="61.28515625" bestFit="1" customWidth="1"/>
@@ -10848,15 +10902,15 @@
         <v>1821</v>
       </c>
       <c r="C263" t="s">
-        <v>1835</v>
+        <v>1834</v>
       </c>
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
+        <v>1835</v>
+      </c>
+      <c r="C264" t="s">
         <v>1836</v>
-      </c>
-      <c r="C264" t="s">
-        <v>1837</v>
       </c>
     </row>
     <row r="265" spans="1:3" x14ac:dyDescent="0.25">
@@ -10896,7 +10950,7 @@
         <v>1829</v>
       </c>
       <c r="C269" t="s">
-        <v>1841</v>
+        <v>1840</v>
       </c>
     </row>
     <row r="270" spans="1:3" x14ac:dyDescent="0.25">
@@ -10904,15 +10958,15 @@
         <v>1830</v>
       </c>
       <c r="C270" t="s">
-        <v>1850</v>
+        <v>1849</v>
       </c>
     </row>
     <row r="271" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>1888</v>
+        <v>1881</v>
       </c>
       <c r="C271" t="s">
-        <v>1864</v>
+        <v>1863</v>
       </c>
     </row>
     <row r="272" spans="1:3" x14ac:dyDescent="0.25">
@@ -10928,36 +10982,36 @@
         <v>1832</v>
       </c>
       <c r="C273" t="s">
-        <v>1834</v>
+        <v>1926</v>
       </c>
     </row>
     <row r="274" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>1877</v>
+        <v>1870</v>
       </c>
       <c r="C274" t="s">
-        <v>1842</v>
+        <v>1841</v>
       </c>
     </row>
     <row r="275" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>1878</v>
+        <v>1871</v>
       </c>
       <c r="C275" t="s">
-        <v>1843</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="276" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>1879</v>
+        <v>1872</v>
       </c>
       <c r="C276" t="s">
-        <v>1861</v>
+        <v>1860</v>
       </c>
     </row>
     <row r="277" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>1880</v>
+        <v>1873</v>
       </c>
       <c r="C277" t="s">
         <v>1612</v>
@@ -10965,261 +11019,321 @@
     </row>
     <row r="278" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>1881</v>
+        <v>1874</v>
       </c>
       <c r="C278" t="s">
-        <v>1844</v>
+        <v>1843</v>
       </c>
     </row>
     <row r="279" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
+        <v>1875</v>
+      </c>
+      <c r="C279" t="s">
         <v>1882</v>
-      </c>
-      <c r="C279" t="s">
-        <v>1889</v>
       </c>
     </row>
     <row r="280" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>1883</v>
+        <v>1876</v>
       </c>
       <c r="C280" t="s">
-        <v>1845</v>
+        <v>1844</v>
       </c>
     </row>
     <row r="281" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>1884</v>
+        <v>1877</v>
       </c>
       <c r="C281" t="s">
-        <v>1846</v>
+        <v>1845</v>
       </c>
     </row>
     <row r="282" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>1885</v>
+        <v>1878</v>
       </c>
       <c r="C282" t="s">
-        <v>1847</v>
+        <v>1846</v>
       </c>
     </row>
     <row r="283" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>1886</v>
+        <v>1879</v>
       </c>
       <c r="C283" t="s">
-        <v>1848</v>
+        <v>1847</v>
       </c>
     </row>
     <row r="284" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>1887</v>
+        <v>1880</v>
       </c>
       <c r="C284" t="s">
-        <v>1849</v>
+        <v>1848</v>
       </c>
     </row>
     <row r="285" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>1896</v>
+        <v>1889</v>
       </c>
       <c r="C285" t="s">
-        <v>1893</v>
+        <v>1886</v>
       </c>
     </row>
     <row r="286" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>1897</v>
+        <v>1890</v>
       </c>
       <c r="C286" t="s">
-        <v>1894</v>
+        <v>1887</v>
       </c>
     </row>
     <row r="287" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>1899</v>
+        <v>1892</v>
       </c>
       <c r="C287" t="s">
-        <v>1895</v>
+        <v>1888</v>
       </c>
     </row>
     <row r="288" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>1900</v>
+        <v>1893</v>
       </c>
       <c r="C288" t="s">
-        <v>1898</v>
+        <v>1891</v>
       </c>
     </row>
     <row r="289" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>1901</v>
+        <v>1894</v>
       </c>
       <c r="C289" t="s">
-        <v>1851</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="290" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>1902</v>
+        <v>1895</v>
       </c>
       <c r="C290" t="s">
-        <v>1852</v>
+        <v>1851</v>
       </c>
     </row>
     <row r="291" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>1903</v>
+        <v>1896</v>
       </c>
       <c r="C291" t="s">
-        <v>1862</v>
+        <v>1861</v>
       </c>
     </row>
     <row r="292" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>1904</v>
+        <v>1897</v>
       </c>
       <c r="C292" t="s">
-        <v>1863</v>
+        <v>1862</v>
       </c>
     </row>
     <row r="293" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>1914</v>
+        <v>1907</v>
       </c>
       <c r="C293" s="5" t="s">
-        <v>1865</v>
+        <v>1864</v>
       </c>
     </row>
     <row r="294" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>1905</v>
+        <v>1898</v>
       </c>
       <c r="C294" t="s">
-        <v>1853</v>
+        <v>1852</v>
       </c>
     </row>
     <row r="295" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>1906</v>
+        <v>1899</v>
       </c>
       <c r="C295" t="s">
-        <v>1854</v>
+        <v>1853</v>
       </c>
     </row>
     <row r="296" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>1907</v>
+        <v>1900</v>
       </c>
       <c r="C296" t="s">
-        <v>1855</v>
+        <v>1854</v>
       </c>
     </row>
     <row r="297" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>1908</v>
+        <v>1901</v>
       </c>
       <c r="C297" t="s">
-        <v>1856</v>
+        <v>1855</v>
       </c>
     </row>
     <row r="298" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>1909</v>
+        <v>1902</v>
       </c>
       <c r="C298" t="s">
-        <v>1857</v>
+        <v>1856</v>
       </c>
     </row>
     <row r="299" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>1910</v>
+        <v>1903</v>
       </c>
       <c r="C299" t="s">
-        <v>1858</v>
+        <v>1857</v>
       </c>
     </row>
     <row r="300" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>1911</v>
+        <v>1904</v>
       </c>
       <c r="C300" t="s">
-        <v>1859</v>
+        <v>1858</v>
       </c>
     </row>
     <row r="301" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
-        <v>1912</v>
+        <v>1905</v>
       </c>
       <c r="C301" t="s">
-        <v>1915</v>
+        <v>1908</v>
       </c>
     </row>
     <row r="302" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
+        <v>1906</v>
+      </c>
+      <c r="C302" t="s">
+        <v>1859</v>
+      </c>
+    </row>
+    <row r="303" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A303" s="5" t="s">
+        <v>1909</v>
+      </c>
+      <c r="C303" t="s">
+        <v>1865</v>
+      </c>
+    </row>
+    <row r="304" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A304" t="s">
+        <v>1910</v>
+      </c>
+      <c r="C304" t="s">
+        <v>1931</v>
+      </c>
+    </row>
+    <row r="305" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A305" t="s">
+        <v>1911</v>
+      </c>
+      <c r="C305" s="2" t="s">
+        <v>1866</v>
+      </c>
+    </row>
+    <row r="306" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A306" t="s">
+        <v>1912</v>
+      </c>
+      <c r="C306" t="s">
+        <v>1867</v>
+      </c>
+    </row>
+    <row r="307" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A307" t="s">
         <v>1913</v>
       </c>
-      <c r="C302" t="s">
-        <v>1860</v>
-      </c>
-    </row>
-    <row r="303" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C303" t="s">
-        <v>1866</v>
-      </c>
-    </row>
-    <row r="304" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="C304" t="s">
-        <v>1867</v>
-      </c>
-    </row>
-    <row r="305" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C305" s="2" t="s">
+      <c r="C307" t="s">
         <v>1868</v>
       </c>
     </row>
-    <row r="306" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C306" t="s">
+    <row r="308" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A308" s="5" t="s">
+        <v>1916</v>
+      </c>
+      <c r="C308" t="s">
+        <v>1932</v>
+      </c>
+    </row>
+    <row r="309" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A309" t="s">
+        <v>1917</v>
+      </c>
+      <c r="C309" t="s">
+        <v>1914</v>
+      </c>
+    </row>
+    <row r="310" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A310" t="s">
+        <v>1918</v>
+      </c>
+      <c r="C310" t="s">
+        <v>1915</v>
+      </c>
+    </row>
+    <row r="311" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A311" t="s">
+        <v>1919</v>
+      </c>
+      <c r="C311" t="s">
+        <v>1933</v>
+      </c>
+    </row>
+    <row r="312" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A312" t="s">
+        <v>1920</v>
+      </c>
+      <c r="C312" t="s">
+        <v>1927</v>
+      </c>
+    </row>
+    <row r="313" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A313" t="s">
+        <v>1921</v>
+      </c>
+      <c r="C313" t="s">
         <v>1869</v>
       </c>
     </row>
-    <row r="307" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C307" t="s">
-        <v>1870</v>
-      </c>
-    </row>
-    <row r="308" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C308" t="s">
-        <v>1871</v>
-      </c>
-    </row>
-    <row r="309" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C309" t="s">
-        <v>1872</v>
-      </c>
-    </row>
-    <row r="310" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C310" t="s">
-        <v>1873</v>
-      </c>
-    </row>
-    <row r="311" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C311" t="s">
-        <v>1874</v>
-      </c>
-    </row>
-    <row r="312" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C312" t="s">
-        <v>1875</v>
-      </c>
-    </row>
-    <row r="313" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C313" t="s">
-        <v>1876</v>
-      </c>
-    </row>
-    <row r="314" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A314" s="6" t="s">
+        <v>1922</v>
+      </c>
       <c r="C314" t="s">
+        <v>1930</v>
+      </c>
+    </row>
+    <row r="315" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A315" s="6" t="s">
+        <v>1923</v>
+      </c>
+      <c r="C315" t="s">
+        <v>1928</v>
+      </c>
+    </row>
+    <row r="316" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A316" s="6" t="s">
+        <v>1924</v>
+      </c>
+      <c r="C316" t="s">
+        <v>1929</v>
+      </c>
+    </row>
+    <row r="317" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A317" s="6" t="s">
+        <v>1925</v>
+      </c>
+      <c r="C317" t="s">
         <v>720</v>
       </c>
     </row>
@@ -13475,13 +13589,13 @@
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
-        <v>1890</v>
+        <v>1883</v>
       </c>
       <c r="B206" t="s">
-        <v>1891</v>
+        <v>1884</v>
       </c>
       <c r="C206" t="s">
-        <v>1892</v>
+        <v>1885</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.25">
@@ -14113,13 +14227,13 @@
     </row>
     <row r="264" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
+        <v>1837</v>
+      </c>
+      <c r="B264" t="s">
         <v>1838</v>
       </c>
-      <c r="B264" t="s">
+      <c r="C264" t="s">
         <v>1839</v>
-      </c>
-      <c r="C264" t="s">
-        <v>1840</v>
       </c>
     </row>
   </sheetData>

</xml_diff>